<commit_message>
Devis recalculé et plan d'implantation électrique
- Suppression de la dépose, saignées revues à la baisse
- Détecteurs remplacés par des interrupteurs Céliane with Netatmo
- Ajout hotte, chauffe-eau (contacteur J/N), bibliothèque séjour (spots ou ruban LED en option)
- Lave-linge, sèche-linge, congélateur et cumulus en buanderie
- Plan d'implantation des 38 circuits (SVG + PDF)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BjWSBdyxAjsRnCWBVUUVzr
</commit_message>
<xml_diff>
--- a/devis/Devis_electricite_T4_connecte_Legrand.xlsx
+++ b/devis/Devis_electricite_T4_connecte_Legrand.xlsx
@@ -30,7 +30,7 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="D108" authorId="0">
+    <comment ref="D110" authorId="0">
       <text>
         <r>
           <rPr>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="284">
   <si>
     <t xml:space="preserve">MAUREL'EC</t>
   </si>
@@ -112,7 +112,7 @@
     <t xml:space="preserve">1</t>
   </si>
   <si>
-    <t xml:space="preserve">INSTALLATION DE CHANTIER, DÉPOSE ET DÉCHETS</t>
+    <t xml:space="preserve">INSTALLATION DE CHANTIER ET DÉCHETS</t>
   </si>
   <si>
     <t xml:space="preserve">1.1</t>
@@ -127,12 +127,6 @@
     <t xml:space="preserve">1.2</t>
   </si>
   <si>
-    <t xml:space="preserve">Dépose complète de l'installation électrique existante (tableau, appareillage, câbles et gaines accessibles)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.3</t>
-  </si>
-  <si>
     <t xml:space="preserve">Débarrassage, tri, évacuation et mise en déchetterie des déchets (gravats de saignées, câbles, emballages), frais de déchetterie inclus</t>
   </si>
   <si>
@@ -235,7 +229,7 @@
     <t xml:space="preserve">3.8</t>
   </si>
   <si>
-    <t xml:space="preserve">Disjoncteur Legrand DX3 Ph+N 16 A (prises, volets, stores, porte WC, filtre à eau, balcons, alarme/caméras, coffret com.)</t>
+    <t xml:space="preserve">Disjoncteur Legrand DX3 Ph+N 16 A (prises, volets, stores, porte WC, filtre à eau, balcons, alarme/caméras, coffret com., hotte)</t>
   </si>
   <si>
     <t xml:space="preserve">3.9</t>
@@ -247,7 +241,7 @@
     <t xml:space="preserve">3.10</t>
   </si>
   <si>
-    <t xml:space="preserve">Disjoncteur Legrand DX3 Ph+N 20 A (prises séjour/cuisine, four, lave-vaisselle, lave-linge, sèche-linge, congélateur, 4 climatisations)</t>
+    <t xml:space="preserve">Disjoncteur Legrand DX3 Ph+N 20 A (prises séjour/cuisine, four, lave-vaisselle, lave-linge, sèche-linge, congélateur, chauffe-eau, 4 climatisations)</t>
   </si>
   <si>
     <t xml:space="preserve">3.11</t>
@@ -259,28 +253,34 @@
     <t xml:space="preserve">3.12</t>
   </si>
   <si>
+    <t xml:space="preserve">Contacteur jour/nuit Legrand 20 A (chauffe-eau, heures creuses)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.13</t>
+  </si>
+  <si>
     <t xml:space="preserve">Parafoudre Legrand type 2 Ph+N avec disjoncteur de déconnexion associé</t>
   </si>
   <si>
-    <t xml:space="preserve">3.13</t>
+    <t xml:space="preserve">3.14</t>
   </si>
   <si>
     <t xml:space="preserve">Pack Legrand Drivia with Netatmo : module Control (passerelle), mesure des consommations, contacteur connecté</t>
   </si>
   <si>
-    <t xml:space="preserve">3.14</t>
+    <t xml:space="preserve">3.15</t>
   </si>
   <si>
     <t xml:space="preserve">Peignes, borniers, repérage des circuits, câblage et mise en ordre du tableau</t>
   </si>
   <si>
-    <t xml:space="preserve">3.15</t>
+    <t xml:space="preserve">3.16</t>
   </si>
   <si>
     <t xml:space="preserve">Tableau de communication Legrand Drivia grade 3TV (DTI, répartiteur RJ45, prise de courant intégrée)</t>
   </si>
   <si>
-    <t xml:space="preserve">3.16</t>
+    <t xml:space="preserve">3.17</t>
   </si>
   <si>
     <t xml:space="preserve">Mise à la terre : barrette de coupure, conducteur principal, liaisons équipotentielles</t>
@@ -304,13 +304,13 @@
     <t xml:space="preserve">4.2</t>
   </si>
   <si>
-    <t xml:space="preserve">Interrupteur connecté Céliane with Netatmo (avec neutre) + plaque – séjour 2, cuisine 2, chambres 3, SDB 2, hall 1</t>
+    <t xml:space="preserve">Interrupteur connecté Céliane with Netatmo (avec neutre) + plaque – séjour 2, cuisine 2, chambres 3, SDB 2, WC 1, hall 1, dégagement 1, buanderie 1, dressing 1</t>
   </si>
   <si>
     <t xml:space="preserve">4.3</t>
   </si>
   <si>
-    <t xml:space="preserve">Détecteur de présence plafond Legrand (allumage SANS CONTACT) – WC, dégagement, buanderie, dressing</t>
+    <t xml:space="preserve">Éclairage bibliothèque du séjour : alimentation (boîte de raccordement, emplacement à définir) + variateur connecté Céliane with Netatmo – spots ou ruban LED en option</t>
   </si>
   <si>
     <t xml:space="preserve">4.4</t>
@@ -337,7 +337,7 @@
     <t xml:space="preserve">5.1</t>
   </si>
   <si>
-    <t xml:space="preserve">Prise de courant 16 A 2P+T Céliane + plaque, circuit 2,5 mm² – séjour 6, chambres 9, cuisine plan de travail 4 + 2 autres, SDB 4, buanderie 1, hall 1, dégagement 1, dressing 1</t>
+    <t xml:space="preserve">Prise de courant 16 A 2P+T Céliane + plaque, circuit 2,5 mm² – séjour 6, chambres 9, cuisine 6 (4 plan de travail, frigo, 1 libre), SDB 4, buanderie 1, hall 1, dégagement 1, dressing 1</t>
   </si>
   <si>
     <t xml:space="preserve">5.2</t>
@@ -445,34 +445,46 @@
     <t xml:space="preserve">9.4</t>
   </si>
   <si>
-    <t xml:space="preserve">Prise spécialisée 20 A lave-linge, circuit dédié 2,5 mm²</t>
+    <t xml:space="preserve">Alimentation hotte : sortie de câble, circuit 16 A dédié</t>
   </si>
   <si>
     <t xml:space="preserve">9.5</t>
   </si>
   <si>
-    <t xml:space="preserve">Prise spécialisée 20 A sèche-linge, circuit dédié 2,5 mm²</t>
+    <t xml:space="preserve">Buanderie – prise spécialisée 20 A lave-linge, circuit dédié 2,5 mm²</t>
   </si>
   <si>
     <t xml:space="preserve">9.6</t>
   </si>
   <si>
-    <t xml:space="preserve">Prise spécialisée 20 A congélateur, circuit dédié 2,5 mm²</t>
+    <t xml:space="preserve">Buanderie – prise spécialisée 20 A sèche-linge, circuit dédié 2,5 mm²</t>
   </si>
   <si>
     <t xml:space="preserve">9.7</t>
   </si>
   <si>
+    <t xml:space="preserve">Buanderie – prise spécialisée 20 A congélateur, circuit dédié 2,5 mm²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buanderie – alimentation chauffe-eau électrique : circuit 20 A en 3G2,5 mm² via contacteur jour/nuit, sortie de câble</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.9</t>
+  </si>
+  <si>
     <t xml:space="preserve">Alimentation filtre à eau : prise dédiée sous évier, circuit 16 A</t>
   </si>
   <si>
-    <t xml:space="preserve">9.8</t>
+    <t xml:space="preserve">9.10</t>
   </si>
   <si>
     <t xml:space="preserve">Alimentation filtre à air : sortie de câble + commande connectée, circuit 2 A</t>
   </si>
   <si>
-    <t xml:space="preserve">9.9</t>
+    <t xml:space="preserve">9.11</t>
   </si>
   <si>
     <t xml:space="preserve">Alimentation porte électrique WC (sortie de câble, circuit 16 A) – porte non fournie</t>
@@ -625,12 +637,24 @@
     <t xml:space="preserve">OPT.3</t>
   </si>
   <si>
-    <t xml:space="preserve">Alimentation hotte de cuisine + commande</t>
+    <t xml:space="preserve">Bibliothèque – VARIANTE A : spots LED encastrés basse tension + alimentation variable</t>
   </si>
   <si>
     <t xml:space="preserve">OPT.4</t>
   </si>
   <si>
+    <t xml:space="preserve">Bibliothèque – VARIANTE B : ruban LED en profilé aluminium avec diffuseur (≈ 12 ml)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPT.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bibliothèque – VARIANTE B : alimentation 24 V variable pour ruban LED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPT.6</t>
+  </si>
+  <si>
     <t xml:space="preserve">Délesteur / gestionnaire d'énergie (chauffage + climatisations)</t>
   </si>
   <si>
@@ -640,7 +664,7 @@
     <t xml:space="preserve">CONDITIONS ET RÉSERVES</t>
   </si>
   <si>
-    <t xml:space="preserve">• NON COMPRIS : fourniture des volets roulants, stores, moteurs, climatisations, électroménager, filtres à eau/air, brumisateurs, ventilateurs et porte électrique WC (alimentation et commande uniquement) ; luminaires intérieurs (hors DCL) ; peinture après rebouchage ; demande de raccordement / modification d'abonnement Enedis.</t>
+    <t xml:space="preserve">• Bibliothèque : choisir la variante A (spots) OU B (ruban LED) – ne pas additionner les deux. NON COMPRIS : dépose de l'installation existante ; fourniture des volets roulants, stores, moteurs, climatisations, électroménager, chauffe-eau, hotte, filtres à eau/air, brumisateurs, ventilateurs et porte électrique WC (alimentation et commande uniquement) ; luminaires intérieurs (hors DCL) ; peinture après rebouchage ; demande de raccordement / modification d'abonnement Enedis.</t>
   </si>
   <si>
     <t xml:space="preserve">• Moteurs de volets et de stores : filaires standard (montée/descente) pour être commandés par les interrupteurs Céliane with Netatmo.</t>
@@ -679,7 +703,7 @@
     <t xml:space="preserve">ID1 – 40 A type A</t>
   </si>
   <si>
-    <t xml:space="preserve">Éclairage zone jour (séjour, cuisine, hall)</t>
+    <t xml:space="preserve">Éclairage zone jour (séjour, bibliothèque, cuisine, hall)</t>
   </si>
   <si>
     <t xml:space="preserve">10 A</t>
@@ -715,7 +739,7 @@
     <t xml:space="preserve">Coffret de communication</t>
   </si>
   <si>
-    <t xml:space="preserve">Filtre à air / ventilation</t>
+    <t xml:space="preserve">Filtre à air</t>
   </si>
   <si>
     <t xml:space="preserve">2 A</t>
@@ -724,13 +748,16 @@
     <t xml:space="preserve">ID2 – 40 A type A</t>
   </si>
   <si>
-    <t xml:space="preserve">Éclairage pièces d'eau, WC, buanderie</t>
+    <t xml:space="preserve">Éclairage SDB 1, SDB 2, WC, buanderie</t>
   </si>
   <si>
     <t xml:space="preserve">Éclairage balcons (extérieur)</t>
   </si>
   <si>
-    <t xml:space="preserve">Prises chambre 3, hall, dégagement, dressing, SDB (8)</t>
+    <t xml:space="preserve">Prises chambre 3, hall, dégagement, dressing (7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prises SDB 1, SDB 2, buanderie (5)</t>
   </si>
   <si>
     <t xml:space="preserve">Prises balcons + brumisateurs + ventilateurs</t>
@@ -739,16 +766,16 @@
     <t xml:space="preserve">Porte électrique WC</t>
   </si>
   <si>
-    <t xml:space="preserve">Alarme / caméras / détecteurs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Filtre à eau</t>
+    <t xml:space="preserve">Alarme / caméras</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtre à eau (sous évier)</t>
   </si>
   <si>
     <t xml:space="preserve">ID3 – 40 A type A</t>
   </si>
   <si>
-    <t xml:space="preserve">Prises plan de travail cuisine (6)</t>
+    <t xml:space="preserve">Prises cuisine : plan de travail + frigo (6)</t>
   </si>
   <si>
     <t xml:space="preserve">Four</t>
@@ -757,10 +784,16 @@
     <t xml:space="preserve">Lave-vaisselle</t>
   </si>
   <si>
-    <t xml:space="preserve">Congélateur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sèche-linge</t>
+    <t xml:space="preserve">Congélateur (buanderie)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sèche-linge (buanderie)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hotte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chauffe-eau (buanderie) via contacteur jour/nuit</t>
   </si>
   <si>
     <t xml:space="preserve">ID4 – 40 A type F</t>
@@ -775,19 +808,19 @@
     <t xml:space="preserve">6 mm²</t>
   </si>
   <si>
-    <t xml:space="preserve">Lave-linge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Climatisation 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Climatisation 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Climatisation 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Climatisation 4</t>
+    <t xml:space="preserve">Lave-linge (buanderie)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Climatisation séjour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Climatisation chambre 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Climatisation chambre 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Climatisation chambre 3</t>
   </si>
   <si>
     <t xml:space="preserve">ID5 – 63 A type A</t>
@@ -835,19 +868,19 @@
     <t xml:space="preserve">•</t>
   </si>
   <si>
-    <t xml:space="preserve">SANS CONTACT : la gamme Céliane with Netatmo n'a pas d'interrupteur tactile capacitif. Le « sans contact » est obtenu par détecteurs de présence (WC, dégagement, buanderie, dressing), commandes vocales et smartphone. Si la cliente veut des interrupteurs tactiles partout, prévoir une autre solution (ex. écran tactile MyHOME) à rechiffrer.</t>
+    <t xml:space="preserve">SANS CONTACT : à valider avec la cliente. Devis établi avec des interrupteurs connectés Céliane with Netatmo partout (pas de tactile dans cette gamme) ; le sans contact passe par la voix et le smartphone.</t>
   </si>
   <si>
     <t xml:space="preserve">PUISSANCE : plancher chauffant (~8,5 kW) + 4 climatisations + cuisson → vérifier l'abonnement (probablement 18 kVA mono ou passage en triphasé). Délesteur conseillé (en option).</t>
   </si>
   <si>
-    <t xml:space="preserve">PLANCHER CHAUFFANT : électrique ou à eau ? Le devis comprend alimentations + régulation. La fourniture/pose des trames est en option. Si plancher à eau, supprimer l'option et revoir les circuits (pompe / régulation).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHAUFFE-EAU : non mentionné (collectif ou individuel ?). Si ballon électrique : ajouter circuit 20 A + contacteur heures creuses.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HOTTE : non mentionnée – en option.</t>
+    <t xml:space="preserve">PLANCHER CHAUFFANT ÉLECTRIQUE (confirmé) : le devis comprend alimentations + régulation. La fourniture/pose des trames reste en option : la passer dans le devis si c'est toi qui les poses.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUANDERIE : lave-linge, sèche-linge, congélateur et chauffe-eau. Vérifier la place (2,56 m² sur le plan) et le passage des câbles.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BIBLIOTHÈQUE DU SÉJOUR : emplacement à définir ; alimentation + variateur connecté prévus, spots (variante A) ou ruban LED (variante B) en option.</t>
   </si>
   <si>
     <t xml:space="preserve">VOLETS : 6 estimés d'après le plan (3 chambres, 2 séjour, 1 cuisine). STORES : 2 estimés (balcons). À compter sur place.</t>
@@ -859,7 +892,7 @@
     <t xml:space="preserve">PIÈCES : la cliente annonce 3 chambres, séjour, cuisine, buanderie, dressing, 2 SDB, WC. Les « SÉCH. » / « RANGT. » du plan sont supposés être la buanderie et le dressing.</t>
   </si>
   <si>
-    <t xml:space="preserve">Saignées : 190 ml murs + 85 ml sol estimés pour un immeuble béton – à recaler à la visite (ce poste pèse lourd dans le total).</t>
+    <t xml:space="preserve">Saignées : 160 ml murs + 70 ml sol estimés pour un immeuble béton – à recaler à la visite (ce poste pèse lourd dans le total).</t>
   </si>
   <si>
     <t xml:space="preserve">Prix fourniture + pose basés sur des tarifs publics moyens Legrand/Netatmo : à vérifier avec ton grossiste et à ajuster selon ta remise.</t>
@@ -1469,7 +1502,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F128"/>
+  <dimension ref="A1:F132"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -1601,74 +1634,74 @@
         <v>1</v>
       </c>
       <c r="E12" s="13" t="n">
-        <v>1200</v>
+        <v>850</v>
       </c>
       <c r="F12" s="14" t="n">
         <f aca="false">D12*E12</f>
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="s">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E13" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="F13" s="16" t="n">
+        <f aca="false">SUM(F11:F12)</f>
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D13" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="13" t="n">
-        <v>850</v>
-      </c>
-      <c r="F13" s="14" t="n">
-        <f aca="false">D13*E13</f>
-        <v>850</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E14" s="15" t="s">
+      <c r="B15" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F14" s="16" t="n">
-        <f aca="false">SUM(F11:F13)</f>
-        <v>2700</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8" t="s">
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
+      <c r="C16" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D16" s="12" t="n">
+        <v>160</v>
+      </c>
+      <c r="E16" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="F16" s="14" t="n">
+        <f aca="false">D16*E16</f>
+        <v>4800</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>34</v>
-      </c>
       <c r="D17" s="12" t="n">
-        <v>190</v>
+        <v>70</v>
       </c>
       <c r="E17" s="13" t="n">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="F17" s="14" t="n">
         <f aca="false">D17*E17</f>
-        <v>7980</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1679,38 +1712,38 @@
         <v>36</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D18" s="12" t="n">
-        <v>85</v>
+        <v>140</v>
       </c>
       <c r="E18" s="13" t="n">
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="F18" s="14" t="n">
         <f aca="false">D18*E18</f>
-        <v>3230</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D19" s="12" t="n">
-        <v>140</v>
+        <v>10</v>
       </c>
       <c r="E19" s="13" t="n">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="F19" s="14" t="n">
         <f aca="false">D19*E19</f>
-        <v>1960</v>
+        <v>450</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1721,60 +1754,60 @@
         <v>41</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D20" s="12" t="n">
-        <v>14</v>
+        <v>230</v>
       </c>
       <c r="E20" s="13" t="n">
-        <v>55</v>
+        <v>7</v>
       </c>
       <c r="F20" s="14" t="n">
         <f aca="false">D20*E20</f>
-        <v>770</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="10" t="s">
+        <v>1610</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E21" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="F21" s="16" t="n">
+        <f aca="false">SUM(F16:F20)</f>
+        <v>9940</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="C21" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="D21" s="12" t="n">
-        <v>275</v>
-      </c>
-      <c r="E21" s="13" t="n">
-        <v>11</v>
-      </c>
-      <c r="F21" s="14" t="n">
-        <f aca="false">D21*E21</f>
-        <v>3025</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E22" s="15" t="s">
+      <c r="B23" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="F22" s="16" t="n">
-        <f aca="false">SUM(F17:F21)</f>
-        <v>16965</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="8" t="s">
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
+      <c r="C24" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D24" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="13" t="n">
+        <v>420</v>
+      </c>
+      <c r="F24" s="14" t="n">
+        <f aca="false">D24*E24</f>
+        <v>420</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
@@ -1784,20 +1817,20 @@
         <v>48</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D25" s="12" t="n">
         <v>1</v>
       </c>
       <c r="E25" s="13" t="n">
-        <v>420</v>
+        <v>460</v>
       </c>
       <c r="F25" s="14" t="n">
         <f aca="false">D25*E25</f>
-        <v>420</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
         <v>49</v>
       </c>
@@ -1805,17 +1838,17 @@
         <v>50</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D26" s="12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E26" s="13" t="n">
-        <v>460</v>
+        <v>175</v>
       </c>
       <c r="F26" s="14" t="n">
         <f aca="false">D26*E26</f>
-        <v>460</v>
+        <v>525</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1826,20 +1859,20 @@
         <v>52</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D27" s="12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E27" s="13" t="n">
-        <v>175</v>
+        <v>260</v>
       </c>
       <c r="F27" s="14" t="n">
         <f aca="false">D27*E27</f>
-        <v>525</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
         <v>53</v>
       </c>
@@ -1847,17 +1880,17 @@
         <v>54</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D28" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E28" s="13" t="n">
-        <v>260</v>
+        <v>210</v>
       </c>
       <c r="F28" s="14" t="n">
         <f aca="false">D28*E28</f>
-        <v>260</v>
+        <v>420</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1868,17 +1901,17 @@
         <v>56</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D29" s="12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E29" s="13" t="n">
-        <v>210</v>
+        <v>38</v>
       </c>
       <c r="F29" s="14" t="n">
         <f aca="false">D29*E29</f>
-        <v>420</v>
+        <v>38</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1889,20 +1922,20 @@
         <v>58</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D30" s="12" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E30" s="13" t="n">
         <v>38</v>
       </c>
       <c r="F30" s="14" t="n">
         <f aca="false">D30*E30</f>
-        <v>38</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
         <v>59</v>
       </c>
@@ -1910,20 +1943,20 @@
         <v>60</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D31" s="12" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E31" s="13" t="n">
         <v>38</v>
       </c>
       <c r="F31" s="14" t="n">
         <f aca="false">D31*E31</f>
-        <v>152</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
         <v>61</v>
       </c>
@@ -1931,7 +1964,7 @@
         <v>62</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D32" s="12" t="n">
         <v>9</v>
@@ -1944,7 +1977,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
         <v>63</v>
       </c>
@@ -1952,20 +1985,20 @@
         <v>64</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D33" s="12" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E33" s="13" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="F33" s="14" t="n">
         <f aca="false">D33*E33</f>
-        <v>342</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
         <v>65</v>
       </c>
@@ -1973,17 +2006,17 @@
         <v>66</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D34" s="12" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="E34" s="13" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="F34" s="14" t="n">
         <f aca="false">D34*E34</f>
-        <v>462</v>
+        <v>48</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1994,17 +2027,17 @@
         <v>68</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D35" s="12" t="n">
         <v>1</v>
       </c>
       <c r="E35" s="13" t="n">
-        <v>48</v>
+        <v>95</v>
       </c>
       <c r="F35" s="14" t="n">
         <f aca="false">D35*E35</f>
-        <v>48</v>
+        <v>95</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2015,7 +2048,7 @@
         <v>70</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D36" s="12" t="n">
         <v>1</v>
@@ -2036,7 +2069,7 @@
         <v>72</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D37" s="12" t="n">
         <v>1</v>
@@ -2078,7 +2111,7 @@
         <v>76</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D39" s="12" t="n">
         <v>1</v>
@@ -2117,8 +2150,8 @@
         <v>79</v>
       </c>
       <c r="F41" s="16" t="n">
-        <f aca="false">SUM(F25:F40)</f>
-        <v>5739</v>
+        <f aca="false">SUM(F24:F40)</f>
+        <v>5952</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2141,7 +2174,7 @@
         <v>83</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D44" s="12" t="n">
         <v>18</v>
@@ -2162,17 +2195,17 @@
         <v>85</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D45" s="12" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E45" s="13" t="n">
         <v>175</v>
       </c>
       <c r="F45" s="14" t="n">
         <f aca="false">D45*E45</f>
-        <v>1750</v>
+        <v>2450</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2183,17 +2216,17 @@
         <v>87</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D46" s="12" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E46" s="13" t="n">
-        <v>165</v>
+        <v>260</v>
       </c>
       <c r="F46" s="14" t="n">
         <f aca="false">D46*E46</f>
-        <v>660</v>
+        <v>260</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2204,7 +2237,7 @@
         <v>89</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D47" s="12" t="n">
         <v>5</v>
@@ -2225,7 +2258,7 @@
         <v>91</v>
       </c>
       <c r="C48" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D48" s="12" t="n">
         <v>2</v>
@@ -2244,7 +2277,7 @@
       </c>
       <c r="F49" s="16" t="n">
         <f aca="false">SUM(F44:F48)</f>
-        <v>4959</v>
+        <v>5259</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2267,7 +2300,7 @@
         <v>96</v>
       </c>
       <c r="C52" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D52" s="12" t="n">
         <v>29</v>
@@ -2288,7 +2321,7 @@
         <v>98</v>
       </c>
       <c r="C53" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D53" s="12" t="n">
         <v>5</v>
@@ -2309,7 +2342,7 @@
         <v>100</v>
       </c>
       <c r="C54" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D54" s="12" t="n">
         <v>6</v>
@@ -2351,7 +2384,7 @@
         <v>105</v>
       </c>
       <c r="C58" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D58" s="12" t="n">
         <v>6</v>
@@ -2372,7 +2405,7 @@
         <v>107</v>
       </c>
       <c r="C59" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D59" s="12" t="n">
         <v>1</v>
@@ -2393,7 +2426,7 @@
         <v>109</v>
       </c>
       <c r="C60" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D60" s="12" t="n">
         <v>2</v>
@@ -2435,7 +2468,7 @@
         <v>114</v>
       </c>
       <c r="C64" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D64" s="12" t="n">
         <v>9</v>
@@ -2456,7 +2489,7 @@
         <v>116</v>
       </c>
       <c r="C65" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D65" s="12" t="n">
         <v>9</v>
@@ -2498,7 +2531,7 @@
         <v>121</v>
       </c>
       <c r="C69" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D69" s="12" t="n">
         <v>4</v>
@@ -2540,7 +2573,7 @@
         <v>126</v>
       </c>
       <c r="C73" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D73" s="12" t="n">
         <v>1</v>
@@ -2561,7 +2594,7 @@
         <v>128</v>
       </c>
       <c r="C74" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D74" s="12" t="n">
         <v>1</v>
@@ -2582,7 +2615,7 @@
         <v>130</v>
       </c>
       <c r="C75" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D75" s="12" t="n">
         <v>1</v>
@@ -2603,17 +2636,17 @@
         <v>132</v>
       </c>
       <c r="C76" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D76" s="12" t="n">
         <v>1</v>
       </c>
       <c r="E76" s="13" t="n">
-        <v>195</v>
+        <v>180</v>
       </c>
       <c r="F76" s="14" t="n">
         <f aca="false">D76*E76</f>
-        <v>195</v>
+        <v>180</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2624,7 +2657,7 @@
         <v>134</v>
       </c>
       <c r="C77" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D77" s="12" t="n">
         <v>1</v>
@@ -2645,7 +2678,7 @@
         <v>136</v>
       </c>
       <c r="C78" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D78" s="12" t="n">
         <v>1</v>
@@ -2666,20 +2699,20 @@
         <v>138</v>
       </c>
       <c r="C79" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D79" s="12" t="n">
         <v>1</v>
       </c>
       <c r="E79" s="13" t="n">
-        <v>175</v>
+        <v>195</v>
       </c>
       <c r="F79" s="14" t="n">
         <f aca="false">D79*E79</f>
-        <v>175</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="10" t="s">
         <v>139</v>
       </c>
@@ -2687,17 +2720,17 @@
         <v>140</v>
       </c>
       <c r="C80" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D80" s="12" t="n">
         <v>1</v>
       </c>
       <c r="E80" s="13" t="n">
-        <v>250</v>
+        <v>230</v>
       </c>
       <c r="F80" s="14" t="n">
         <f aca="false">D80*E80</f>
-        <v>250</v>
+        <v>230</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2708,83 +2741,83 @@
         <v>142</v>
       </c>
       <c r="C81" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D81" s="12" t="n">
         <v>1</v>
       </c>
       <c r="E81" s="13" t="n">
-        <v>230</v>
+        <v>175</v>
       </c>
       <c r="F81" s="14" t="n">
         <f aca="false">D81*E81</f>
+        <v>175</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A82" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="B82" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="C82" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D82" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E82" s="13" t="n">
+        <v>250</v>
+      </c>
+      <c r="F82" s="14" t="n">
+        <f aca="false">D82*E82</f>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A83" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="B83" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="C83" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D83" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E83" s="13" t="n">
         <v>230</v>
       </c>
-    </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E82" s="15" t="s">
-        <v>143</v>
-      </c>
-      <c r="F82" s="16" t="n">
-        <f aca="false">SUM(F73:F81)</f>
-        <v>1900</v>
+      <c r="F83" s="14" t="n">
+        <f aca="false">D83*E83</f>
+        <v>230</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="B84" s="9" t="s">
-        <v>145</v>
-      </c>
-      <c r="C84" s="9"/>
-      <c r="D84" s="9"/>
-      <c r="E84" s="9"/>
-      <c r="F84" s="9"/>
-    </row>
-    <row r="85" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A85" s="10" t="s">
-        <v>146</v>
-      </c>
-      <c r="B85" s="11" t="s">
+      <c r="E84" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="C85" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="D85" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="E85" s="13" t="n">
-        <v>195</v>
-      </c>
-      <c r="F85" s="14" t="n">
-        <f aca="false">D85*E85</f>
-        <v>585</v>
-      </c>
-    </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A86" s="10" t="s">
+      <c r="F84" s="16" t="n">
+        <f aca="false">SUM(F73:F83)</f>
+        <v>2310</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="B86" s="11" t="s">
+      <c r="B86" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="C86" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="D86" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E86" s="13" t="n">
-        <v>175</v>
-      </c>
-      <c r="F86" s="14" t="n">
-        <f aca="false">D86*E86</f>
-        <v>350</v>
-      </c>
-    </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C86" s="9"/>
+      <c r="D86" s="9"/>
+      <c r="E86" s="9"/>
+      <c r="F86" s="9"/>
+    </row>
+    <row r="87" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="10" t="s">
         <v>150</v>
       </c>
@@ -2792,17 +2825,17 @@
         <v>151</v>
       </c>
       <c r="C87" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D87" s="12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E87" s="13" t="n">
-        <v>240</v>
+        <v>195</v>
       </c>
       <c r="F87" s="14" t="n">
         <f aca="false">D87*E87</f>
-        <v>480</v>
+        <v>585</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2813,17 +2846,17 @@
         <v>153</v>
       </c>
       <c r="C88" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D88" s="12" t="n">
         <v>2</v>
       </c>
       <c r="E88" s="13" t="n">
-        <v>240</v>
+        <v>175</v>
       </c>
       <c r="F88" s="14" t="n">
         <f aca="false">D88*E88</f>
-        <v>480</v>
+        <v>350</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2834,83 +2867,83 @@
         <v>155</v>
       </c>
       <c r="C89" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D89" s="12" t="n">
         <v>2</v>
       </c>
       <c r="E89" s="13" t="n">
-        <v>125</v>
+        <v>240</v>
       </c>
       <c r="F89" s="14" t="n">
         <f aca="false">D89*E89</f>
+        <v>480</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A90" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="B90" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="C90" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D90" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E90" s="13" t="n">
+        <v>240</v>
+      </c>
+      <c r="F90" s="14" t="n">
+        <f aca="false">D90*E90</f>
+        <v>480</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A91" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="B91" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="C91" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D91" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E91" s="13" t="n">
+        <v>125</v>
+      </c>
+      <c r="F91" s="14" t="n">
+        <f aca="false">D91*E91</f>
         <v>250</v>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E90" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="F90" s="16" t="n">
-        <f aca="false">SUM(F85:F89)</f>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E92" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="F92" s="16" t="n">
+        <f aca="false">SUM(F87:F91)</f>
         <v>2145</v>
       </c>
     </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="B92" s="9" t="s">
-        <v>158</v>
-      </c>
-      <c r="C92" s="9"/>
-      <c r="D92" s="9"/>
-      <c r="E92" s="9"/>
-      <c r="F92" s="9"/>
-    </row>
-    <row r="93" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A93" s="10" t="s">
-        <v>159</v>
-      </c>
-      <c r="B93" s="11" t="s">
-        <v>160</v>
-      </c>
-      <c r="C93" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="D93" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="E93" s="13" t="n">
-        <v>125</v>
-      </c>
-      <c r="F93" s="14" t="n">
-        <f aca="false">D93*E93</f>
-        <v>375</v>
-      </c>
-    </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A94" s="10" t="s">
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="B94" s="11" t="s">
+      <c r="B94" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="C94" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="D94" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E94" s="13" t="n">
-        <v>270</v>
-      </c>
-      <c r="F94" s="14" t="n">
-        <f aca="false">D94*E94</f>
-        <v>270</v>
-      </c>
-    </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C94" s="9"/>
+      <c r="D94" s="9"/>
+      <c r="E94" s="9"/>
+      <c r="F94" s="9"/>
+    </row>
+    <row r="95" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="10" t="s">
         <v>163</v>
       </c>
@@ -2918,17 +2951,17 @@
         <v>164</v>
       </c>
       <c r="C95" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D95" s="12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E95" s="13" t="n">
-        <v>150</v>
+        <v>125</v>
       </c>
       <c r="F95" s="14" t="n">
         <f aca="false">D95*E95</f>
-        <v>150</v>
+        <v>375</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2939,17 +2972,17 @@
         <v>166</v>
       </c>
       <c r="C96" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D96" s="12" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E96" s="13" t="n">
-        <v>58</v>
+        <v>270</v>
       </c>
       <c r="F96" s="14" t="n">
         <f aca="false">D96*E96</f>
-        <v>406</v>
+        <v>270</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2960,17 +2993,17 @@
         <v>168</v>
       </c>
       <c r="C97" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D97" s="12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E97" s="13" t="n">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="F97" s="14" t="n">
         <f aca="false">D97*E97</f>
-        <v>435</v>
+        <v>150</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2981,81 +3014,81 @@
         <v>170</v>
       </c>
       <c r="C98" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D98" s="12" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E98" s="13" t="n">
-        <v>350</v>
+        <v>58</v>
       </c>
       <c r="F98" s="14" t="n">
         <f aca="false">D98*E98</f>
+        <v>406</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A99" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="B99" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="C99" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D99" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E99" s="13" t="n">
+        <v>145</v>
+      </c>
+      <c r="F99" s="14" t="n">
+        <f aca="false">D99*E99</f>
+        <v>435</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A100" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="B100" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="C100" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D100" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E100" s="13" t="n">
+        <v>350</v>
+      </c>
+      <c r="F100" s="14" t="n">
+        <f aca="false">D100*E100</f>
         <v>700</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E99" s="15" t="s">
-        <v>171</v>
-      </c>
-      <c r="F99" s="16" t="n">
-        <f aca="false">SUM(F93:F98)</f>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E101" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="F101" s="16" t="n">
+        <f aca="false">SUM(F95:F100)</f>
         <v>2336</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="8" t="s">
-        <v>172</v>
-      </c>
-      <c r="B101" s="9" t="s">
-        <v>173</v>
-      </c>
-      <c r="C101" s="9"/>
-      <c r="D101" s="9"/>
-      <c r="E101" s="9"/>
-      <c r="F101" s="9"/>
-    </row>
-    <row r="102" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A102" s="10" t="s">
-        <v>174</v>
-      </c>
-      <c r="B102" s="11" t="s">
-        <v>175</v>
-      </c>
-      <c r="C102" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D102" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E102" s="13" t="n">
-        <v>480</v>
-      </c>
-      <c r="F102" s="14" t="n">
-        <f aca="false">D102*E102</f>
-        <v>480</v>
-      </c>
-    </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A103" s="10" t="s">
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="B103" s="11" t="s">
+      <c r="B103" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="C103" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D103" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E103" s="13" t="n">
-        <v>280</v>
-      </c>
-      <c r="F103" s="14" t="n">
-        <f aca="false">D103*E103</f>
-        <v>280</v>
-      </c>
+      <c r="C103" s="9"/>
+      <c r="D103" s="9"/>
+      <c r="E103" s="9"/>
+      <c r="F103" s="9"/>
     </row>
     <row r="104" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="10" t="s">
@@ -3071,127 +3104,127 @@
         <v>1</v>
       </c>
       <c r="E104" s="13" t="n">
-        <v>360</v>
+        <v>480</v>
       </c>
       <c r="F104" s="14" t="n">
         <f aca="false">D104*E104</f>
+        <v>480</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A105" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="B105" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="C105" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D105" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E105" s="13" t="n">
+        <v>280</v>
+      </c>
+      <c r="F105" s="14" t="n">
+        <f aca="false">D105*E105</f>
+        <v>280</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A106" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="B106" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="C106" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D106" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E106" s="13" t="n">
         <v>360</v>
       </c>
-    </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E105" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="F105" s="16" t="n">
-        <f aca="false">SUM(F102:F104)</f>
+      <c r="F106" s="14" t="n">
+        <f aca="false">D106*E106</f>
+        <v>360</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E107" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="F107" s="16" t="n">
+        <f aca="false">SUM(F104:F106)</f>
         <v>1120</v>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E107" s="17" t="s">
-        <v>181</v>
-      </c>
-      <c r="F107" s="18" t="n">
-        <f aca="false">F14+F22+F41+F49+F55+F61+F66+F70+F82+F90+F99+F105</f>
-        <v>49746</v>
-      </c>
-    </row>
-    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D108" s="19" t="n">
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E109" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="F109" s="18" t="n">
+        <f aca="false">F13+F21+F41+F49+F55+F61+F66+F70+F84+F92+F101+F107</f>
+        <v>42444</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D110" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="E108" s="17" t="s">
-        <v>182</v>
-      </c>
-      <c r="F108" s="18" t="n">
-        <f aca="false">F107*D108</f>
-        <v>4974.6</v>
-      </c>
-    </row>
-    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E109" s="20" t="s">
-        <v>183</v>
-      </c>
-      <c r="F109" s="21" t="n">
-        <f aca="false">F107+F108</f>
-        <v>54720.6</v>
-      </c>
-    </row>
-    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E110" s="22" t="s">
-        <v>184</v>
-      </c>
-      <c r="F110" s="23" t="n">
-        <f aca="false">F109*0.3</f>
-        <v>16416.18</v>
-      </c>
-    </row>
-    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="24" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="114" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A114" s="10" t="s">
+      <c r="E110" s="17" t="s">
         <v>186</v>
       </c>
-      <c r="B114" s="11" t="s">
+      <c r="F110" s="18" t="n">
+        <f aca="false">F109*D110</f>
+        <v>4244.4</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E111" s="20" t="s">
         <v>187</v>
       </c>
-      <c r="C114" s="10" t="s">
+      <c r="F111" s="21" t="n">
+        <f aca="false">F109+F110</f>
+        <v>46688.4</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E112" s="22" t="s">
         <v>188</v>
       </c>
-      <c r="D114" s="12" t="n">
+      <c r="F112" s="23" t="n">
+        <f aca="false">F111*0.3</f>
+        <v>14006.52</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="24" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A116" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="B116" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="C116" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="D116" s="12" t="n">
         <v>85</v>
       </c>
-      <c r="E114" s="13" t="n">
+      <c r="E116" s="13" t="n">
         <v>78</v>
-      </c>
-      <c r="F114" s="14" t="n">
-        <f aca="false">D114*E114</f>
-        <v>6630</v>
-      </c>
-    </row>
-    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A115" s="10" t="s">
-        <v>189</v>
-      </c>
-      <c r="B115" s="11" t="s">
-        <v>190</v>
-      </c>
-      <c r="C115" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="D115" s="12" t="n">
-        <v>12</v>
-      </c>
-      <c r="E115" s="13" t="n">
-        <v>65</v>
-      </c>
-      <c r="F115" s="14" t="n">
-        <f aca="false">D115*E115</f>
-        <v>780</v>
-      </c>
-    </row>
-    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A116" s="10" t="s">
-        <v>191</v>
-      </c>
-      <c r="B116" s="11" t="s">
-        <v>192</v>
-      </c>
-      <c r="C116" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="D116" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E116" s="13" t="n">
-        <v>160</v>
       </c>
       <c r="F116" s="14" t="n">
         <f aca="false">D116*E116</f>
-        <v>160</v>
+        <v>6630</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3202,61 +3235,145 @@
         <v>194</v>
       </c>
       <c r="C117" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D117" s="12" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E117" s="13" t="n">
-        <v>420</v>
+        <v>65</v>
       </c>
       <c r="F117" s="14" t="n">
         <f aca="false">D117*E117</f>
+        <v>780</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A118" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="B118" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="C118" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D118" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="E118" s="13" t="n">
+        <v>75</v>
+      </c>
+      <c r="F118" s="14" t="n">
+        <f aca="false">D118*E118</f>
+        <v>600</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A119" s="10" t="s">
+        <v>197</v>
+      </c>
+      <c r="B119" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="C119" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D119" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="E119" s="13" t="n">
+        <v>65</v>
+      </c>
+      <c r="F119" s="14" t="n">
+        <f aca="false">D119*E119</f>
+        <v>780</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A120" s="10" t="s">
+        <v>199</v>
+      </c>
+      <c r="B120" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="C120" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D120" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E120" s="13" t="n">
+        <v>120</v>
+      </c>
+      <c r="F120" s="14" t="n">
+        <f aca="false">D120*E120</f>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A121" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="B121" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="C121" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D121" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E121" s="13" t="n">
         <v>420</v>
       </c>
-    </row>
-    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E118" s="15" t="s">
-        <v>195</v>
-      </c>
-      <c r="F118" s="16" t="n">
-        <f aca="false">SUM(F114:F117)</f>
-        <v>7990</v>
-      </c>
-    </row>
-    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A121" s="2" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="122" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B122" s="25" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="123" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B123" s="25" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="124" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B124" s="25" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="125" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B125" s="25" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="126" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F121" s="14" t="n">
+        <f aca="false">D121*E121</f>
+        <v>420</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E122" s="15" t="s">
+        <v>203</v>
+      </c>
+      <c r="F122" s="16" t="n">
+        <f aca="false">SUM(F116:F121)</f>
+        <v>9330</v>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="2" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B126" s="25" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B128" s="2" t="s">
-        <v>202</v>
+        <v>205</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B127" s="25" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B128" s="25" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="129" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B129" s="25" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B130" s="25" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B132" s="2" t="s">
+        <v>210</v>
       </c>
     </row>
   </sheetData>
@@ -3276,7 +3393,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -3287,12 +3404,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="26" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="27" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3300,16 +3417,16 @@
         <v>14</v>
       </c>
       <c r="B4" s="28" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="C4" s="28" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="D4" s="28" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="E4" s="28" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3317,16 +3434,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="D5" s="29" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3334,16 +3451,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="29" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="C6" s="29" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="D6" s="29" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="E6" s="29" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3351,16 +3468,16 @@
         <v>3</v>
       </c>
       <c r="B7" s="29" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="C7" s="29" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="D7" s="29" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3368,16 +3485,16 @@
         <v>4</v>
       </c>
       <c r="B8" s="29" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="C8" s="29" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="D8" s="29" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="E8" s="29" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3385,16 +3502,16 @@
         <v>5</v>
       </c>
       <c r="B9" s="29" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="D9" s="29" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3402,16 +3519,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="29" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="C10" s="29" t="s">
+        <v>228</v>
+      </c>
+      <c r="D10" s="29" t="s">
+        <v>226</v>
+      </c>
+      <c r="E10" s="29" t="s">
         <v>220</v>
-      </c>
-      <c r="D10" s="29" t="s">
-        <v>218</v>
-      </c>
-      <c r="E10" s="29" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3419,16 +3536,16 @@
         <v>7</v>
       </c>
       <c r="B11" s="29" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="C11" s="29" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="D11" s="29" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="E11" s="29" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3436,16 +3553,16 @@
         <v>8</v>
       </c>
       <c r="B12" s="29" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="C12" s="29" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="D12" s="29" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="E12" s="29" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3453,16 +3570,16 @@
         <v>9</v>
       </c>
       <c r="B13" s="29" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="C13" s="29" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="D13" s="29" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="E13" s="29" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3470,16 +3587,16 @@
         <v>10</v>
       </c>
       <c r="B14" s="29" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="D14" s="29" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="E14" s="29" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3487,16 +3604,16 @@
         <v>11</v>
       </c>
       <c r="B15" s="29" t="s">
+        <v>232</v>
+      </c>
+      <c r="C15" s="29" t="s">
+        <v>235</v>
+      </c>
+      <c r="D15" s="29" t="s">
+        <v>226</v>
+      </c>
+      <c r="E15" s="29" t="s">
         <v>224</v>
-      </c>
-      <c r="C15" s="29" t="s">
-        <v>227</v>
-      </c>
-      <c r="D15" s="29" t="s">
-        <v>218</v>
-      </c>
-      <c r="E15" s="29" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3504,16 +3621,16 @@
         <v>12</v>
       </c>
       <c r="B16" s="29" t="s">
+        <v>232</v>
+      </c>
+      <c r="C16" s="29" t="s">
+        <v>236</v>
+      </c>
+      <c r="D16" s="29" t="s">
+        <v>226</v>
+      </c>
+      <c r="E16" s="29" t="s">
         <v>224</v>
-      </c>
-      <c r="C16" s="29" t="s">
-        <v>228</v>
-      </c>
-      <c r="D16" s="29" t="s">
-        <v>218</v>
-      </c>
-      <c r="E16" s="29" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3521,16 +3638,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="29" t="s">
+        <v>232</v>
+      </c>
+      <c r="C17" s="29" t="s">
+        <v>237</v>
+      </c>
+      <c r="D17" s="29" t="s">
+        <v>226</v>
+      </c>
+      <c r="E17" s="29" t="s">
         <v>224</v>
-      </c>
-      <c r="C17" s="29" t="s">
-        <v>229</v>
-      </c>
-      <c r="D17" s="29" t="s">
-        <v>218</v>
-      </c>
-      <c r="E17" s="29" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3538,16 +3655,16 @@
         <v>14</v>
       </c>
       <c r="B18" s="29" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="C18" s="29" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="D18" s="29" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="E18" s="29" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3555,16 +3672,16 @@
         <v>15</v>
       </c>
       <c r="B19" s="29" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="C19" s="29" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="D19" s="29" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="E19" s="29" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3575,13 +3692,13 @@
         <v>232</v>
       </c>
       <c r="C20" s="29" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="D20" s="29" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="E20" s="29" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3589,16 +3706,16 @@
         <v>17</v>
       </c>
       <c r="B21" s="29" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="C21" s="29" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="D21" s="29" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="E21" s="29" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3606,16 +3723,16 @@
         <v>18</v>
       </c>
       <c r="B22" s="29" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="C22" s="29" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="D22" s="29" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="E22" s="29" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3623,16 +3740,16 @@
         <v>19</v>
       </c>
       <c r="B23" s="29" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="C23" s="29" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="D23" s="29" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="E23" s="29" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3640,16 +3757,16 @@
         <v>20</v>
       </c>
       <c r="B24" s="29" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="C24" s="29" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D24" s="29" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="E24" s="29" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3657,16 +3774,16 @@
         <v>21</v>
       </c>
       <c r="B25" s="29" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="C25" s="29" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="D25" s="29" t="s">
-        <v>240</v>
+        <v>223</v>
       </c>
       <c r="E25" s="29" t="s">
-        <v>241</v>
+        <v>224</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3674,16 +3791,16 @@
         <v>22</v>
       </c>
       <c r="B26" s="29" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="C26" s="29" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="D26" s="29" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="E26" s="29" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3691,16 +3808,16 @@
         <v>23</v>
       </c>
       <c r="B27" s="29" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="C27" s="29" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="D27" s="29" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="E27" s="29" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3708,16 +3825,16 @@
         <v>24</v>
       </c>
       <c r="B28" s="29" t="s">
-        <v>238</v>
+        <v>249</v>
       </c>
       <c r="C28" s="29" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="D28" s="29" t="s">
-        <v>215</v>
+        <v>251</v>
       </c>
       <c r="E28" s="29" t="s">
-        <v>216</v>
+        <v>252</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3725,16 +3842,16 @@
         <v>25</v>
       </c>
       <c r="B29" s="29" t="s">
-        <v>238</v>
+        <v>249</v>
       </c>
       <c r="C29" s="29" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="D29" s="29" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="E29" s="29" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3742,16 +3859,16 @@
         <v>26</v>
       </c>
       <c r="B30" s="29" t="s">
-        <v>238</v>
+        <v>249</v>
       </c>
       <c r="C30" s="29" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="D30" s="29" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="E30" s="29" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3759,16 +3876,16 @@
         <v>27</v>
       </c>
       <c r="B31" s="29" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C31" s="29" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="D31" s="29" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="E31" s="29" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3776,16 +3893,16 @@
         <v>28</v>
       </c>
       <c r="B32" s="29" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C32" s="29" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
       <c r="D32" s="29" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="E32" s="29" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3793,16 +3910,16 @@
         <v>29</v>
       </c>
       <c r="B33" s="29" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C33" s="29" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="D33" s="29" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="E33" s="29" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3810,16 +3927,16 @@
         <v>30</v>
       </c>
       <c r="B34" s="29" t="s">
-        <v>247</v>
+        <v>258</v>
       </c>
       <c r="C34" s="29" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="D34" s="29" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="E34" s="29" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3827,16 +3944,16 @@
         <v>31</v>
       </c>
       <c r="B35" s="29" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="C35" s="29" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="D35" s="29" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="E35" s="29" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3844,16 +3961,16 @@
         <v>32</v>
       </c>
       <c r="B36" s="29" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="C36" s="29" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="D36" s="29" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="E36" s="29" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3861,16 +3978,16 @@
         <v>33</v>
       </c>
       <c r="B37" s="29" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="C37" s="29" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="D37" s="29" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="E37" s="29" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3878,16 +3995,16 @@
         <v>34</v>
       </c>
       <c r="B38" s="29" t="s">
-        <v>252</v>
+        <v>263</v>
       </c>
       <c r="C38" s="29" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="D38" s="29" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="E38" s="29" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3895,33 +4012,84 @@
         <v>35</v>
       </c>
       <c r="B39" s="29" t="s">
-        <v>252</v>
+        <v>263</v>
       </c>
       <c r="C39" s="29" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="D39" s="29" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="E39" s="29" t="s">
-        <v>216</v>
+        <v>224</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="29" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="29" t="s">
+        <v>263</v>
+      </c>
+      <c r="C40" s="29" t="s">
+        <v>266</v>
+      </c>
+      <c r="D40" s="29" t="s">
+        <v>226</v>
+      </c>
+      <c r="E40" s="29" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C41" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="D41" s="2" t="n">
-        <f aca="false">COUNTA(C5:C39)</f>
-        <v>35</v>
+      <c r="A41" s="29" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="29" t="s">
+        <v>263</v>
+      </c>
+      <c r="C41" s="29" t="s">
+        <v>267</v>
+      </c>
+      <c r="D41" s="29" t="s">
+        <v>226</v>
+      </c>
+      <c r="E41" s="29" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C42" s="5" t="s">
-        <v>259</v>
-      </c>
-      <c r="D42" s="30" t="n">
-        <f aca="false">MAX(COUNTIF(B5:B39,"ID1*"),COUNTIF(B5:B39,"ID2*"),COUNTIF(B5:B39,"ID3*"),COUNTIF(B5:B39,"ID4*"),COUNTIF(B5:B39,"ID5*"),COUNTIF(B5:B39,"ID6*"))</f>
+      <c r="A42" s="29" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="29" t="s">
+        <v>263</v>
+      </c>
+      <c r="C42" s="29" t="s">
+        <v>268</v>
+      </c>
+      <c r="D42" s="29" t="s">
+        <v>226</v>
+      </c>
+      <c r="E42" s="29" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C44" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="D44" s="2" t="n">
+        <f aca="false">COUNTA(C5:C42)</f>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C45" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="D45" s="30" t="n">
+        <f aca="false">MAX(COUNTIF(B5:B42,"ID1*"),COUNTIF(B5:B42,"ID2*"),COUNTIF(B5:B42,"ID3*"),COUNTIF(B5:B42,"ID4*"),COUNTIF(B5:B42,"ID5*"),COUNTIF(B5:B42,"ID6*"))</f>
         <v>8</v>
       </c>
     </row>
@@ -3950,92 +4118,92 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="26" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>261</v>
+        <v>272</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>262</v>
+        <v>273</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>261</v>
+        <v>272</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>263</v>
+        <v>274</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>261</v>
+        <v>272</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>264</v>
+        <v>275</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>261</v>
+        <v>272</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>261</v>
+        <v>272</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>266</v>
+        <v>277</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>261</v>
+        <v>272</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>267</v>
+        <v>278</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>261</v>
+        <v>272</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>268</v>
+        <v>279</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>261</v>
+        <v>272</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>269</v>
+        <v>280</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>261</v>
+        <v>272</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>270</v>
+        <v>281</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>261</v>
+        <v>272</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>271</v>
+        <v>282</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="31" t="s">
-        <v>272</v>
+        <v>283</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Devis v3 : attentes clim/plancher/balcons, prises au minimum NF C 15-100
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BjWSBdyxAjsRnCWBVUUVzr
</commit_message>
<xml_diff>
--- a/devis/Devis_electricite_T4_connecte_Legrand.xlsx
+++ b/devis/Devis_electricite_T4_connecte_Legrand.xlsx
@@ -30,7 +30,7 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="D110" authorId="0">
+    <comment ref="D108" authorId="0">
       <text>
         <r>
           <rPr>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="278">
   <si>
     <t xml:space="preserve">MAUREL'EC</t>
   </si>
@@ -310,7 +310,7 @@
     <t xml:space="preserve">4.3</t>
   </si>
   <si>
-    <t xml:space="preserve">Éclairage bibliothèque du séjour : alimentation (boîte de raccordement, emplacement à définir) + variateur connecté Céliane with Netatmo – spots ou ruban LED en option</t>
+    <t xml:space="preserve">Éclairage bibliothèque du séjour : alimentation (boîte de raccordement, emplacement à définir) + commande variateur connecté Céliane with Netatmo – spots ou ruban LED en option</t>
   </si>
   <si>
     <t xml:space="preserve">4.4</t>
@@ -337,7 +337,7 @@
     <t xml:space="preserve">5.1</t>
   </si>
   <si>
-    <t xml:space="preserve">Prise de courant 16 A 2P+T Céliane + plaque, circuit 2,5 mm² – séjour 6, chambres 9, cuisine 6 (4 plan de travail, frigo, 1 libre), SDB 4, buanderie 1, hall 1, dégagement 1, dressing 1</t>
+    <t xml:space="preserve">Prise de courant 16 A 2P+T Céliane + plaque, circuit 2,5 mm² – minimum NF C 15-100 – séjour 5 (+2 connectées = 7), chambres 2 (+1 connectée = 3) x3, cuisine 6 (dont 4 plan de travail, frigo), SDB 1 x2, hall 1, dégagement 1</t>
   </si>
   <si>
     <t xml:space="preserve">5.2</t>
@@ -349,7 +349,7 @@
     <t xml:space="preserve">5.3</t>
   </si>
   <si>
-    <t xml:space="preserve">Prise RJ45 grade 3TV Céliane (séjour 2, chambres 3, cuisine 1) avec câble depuis le tableau de communication</t>
+    <t xml:space="preserve">Prise RJ45 grade 3TV Céliane – minimum NF C 15-100 (séjour 2, chambres 3), câble depuis le tableau de communication</t>
   </si>
   <si>
     <t xml:space="preserve">Sous-total lot 5</t>
@@ -370,7 +370,7 @@
     <t xml:space="preserve">6.2</t>
   </si>
   <si>
-    <t xml:space="preserve">Commande générale volets roulants sans fil Céliane with Netatmo</t>
+    <t xml:space="preserve">Commande générale volets roulants sans fil Céliane with Netatmo (ouverture/fermeture centralisée)</t>
   </si>
   <si>
     <t xml:space="preserve">6.3</t>
@@ -385,19 +385,13 @@
     <t xml:space="preserve">7</t>
   </si>
   <si>
-    <t xml:space="preserve">CHAUFFAGE AU SOL – ALIMENTATION ET RÉGULATION CONNECTÉE</t>
+    <t xml:space="preserve">CHAUFFAGE AU SOL – ALIMENTATIONS EN ATTENTE</t>
   </si>
   <si>
     <t xml:space="preserve">7.1</t>
   </si>
   <si>
-    <t xml:space="preserve">Alimentation zone de plancher chauffant : circuit dédié, boîte de raccordement, raccordement trame + sonde de sol – séjour, 3 chambres, cuisine, 2 SDB, hall/dégagement, buanderie/dressing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thermostat connecté à sonde de sol par zone, pilotable sur smartphone (modèle selon fabricant du plancher)</t>
+    <t xml:space="preserve">Alimentation en attente zone de plancher chauffant : circuit dédié 16 A en 2,5 mm², boîte de raccordement – séjour, 3 chambres, cuisine, 2 SDB, hall/dégagement, buanderie/dressing (trame et thermostat non fournis)</t>
   </si>
   <si>
     <t xml:space="preserve">Sous-total lot 7</t>
@@ -412,7 +406,7 @@
     <t xml:space="preserve">8.1</t>
   </si>
   <si>
-    <t xml:space="preserve">Alimentation dédiée climatisation réversible : circuit 20 A en 3G2,5 mm², sortie de câble + interrupteur de proximité côté unité extérieure</t>
+    <t xml:space="preserve">Alimentation en attente climatisation réversible à côté de l'unité extérieure : circuit 20 A dédié en 3G2,5 mm² (raccordement direct sur le groupe par le climaticien)</t>
   </si>
   <si>
     <t xml:space="preserve">Sous-total lot 8</t>
@@ -502,7 +496,7 @@
     <t xml:space="preserve">10.1</t>
   </si>
   <si>
-    <t xml:space="preserve">Point lumineux extérieur + applique LED étanche IP65 fournie (balcon séjour 2, balcon chambre/cuisine 1)</t>
+    <t xml:space="preserve">Alimentation en attente éclairage extérieur (boîte étanche, câble depuis le tableau) – balcon séjour 2, balcon chambre/cuisine 1 – appliques non fournies</t>
   </si>
   <si>
     <t xml:space="preserve">10.2</t>
@@ -523,12 +517,6 @@
     <t xml:space="preserve">Alimentation ventilateur + commande connectée (1 par balcon)</t>
   </si>
   <si>
-    <t xml:space="preserve">10.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prise de courant étanche Legrand Plexo IP55 (1 par balcon)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Sous-total lot 10</t>
   </si>
   <si>
@@ -622,39 +610,30 @@
     <t xml:space="preserve">OPT.1</t>
   </si>
   <si>
-    <t xml:space="preserve">Fourniture et pose de trames chauffantes électriques pour plancher chauffant (≈ 85 m² chauffés, hors chape)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">m²</t>
+    <t xml:space="preserve">Spots LED encastrés étanches (séjour, cuisine, salles de bain), fourniture et pose</t>
   </si>
   <si>
     <t xml:space="preserve">OPT.2</t>
   </si>
   <si>
-    <t xml:space="preserve">Spots LED encastrés étanches (séjour, cuisine, salles de bain), fourniture et pose</t>
+    <t xml:space="preserve">Bibliothèque – VARIANTE A : spots LED encastrés basse tension + alimentation variable</t>
   </si>
   <si>
     <t xml:space="preserve">OPT.3</t>
   </si>
   <si>
-    <t xml:space="preserve">Bibliothèque – VARIANTE A : spots LED encastrés basse tension + alimentation variable</t>
+    <t xml:space="preserve">Bibliothèque – VARIANTE B : ruban LED en profilé aluminium avec diffuseur (≈ 6 ml)</t>
   </si>
   <si>
     <t xml:space="preserve">OPT.4</t>
   </si>
   <si>
-    <t xml:space="preserve">Bibliothèque – VARIANTE B : ruban LED en profilé aluminium avec diffuseur (≈ 12 ml)</t>
+    <t xml:space="preserve">Bibliothèque – VARIANTE B : alimentation 24 V variable pour ruban LED</t>
   </si>
   <si>
     <t xml:space="preserve">OPT.5</t>
   </si>
   <si>
-    <t xml:space="preserve">Bibliothèque – VARIANTE B : alimentation 24 V variable pour ruban LED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OPT.6</t>
-  </si>
-  <si>
     <t xml:space="preserve">Délesteur / gestionnaire d'énergie (chauffage + climatisations)</t>
   </si>
   <si>
@@ -664,7 +643,7 @@
     <t xml:space="preserve">CONDITIONS ET RÉSERVES</t>
   </si>
   <si>
-    <t xml:space="preserve">• Bibliothèque : choisir la variante A (spots) OU B (ruban LED) – ne pas additionner les deux. NON COMPRIS : dépose de l'installation existante ; fourniture des volets roulants, stores, moteurs, climatisations, électroménager, chauffe-eau, hotte, filtres à eau/air, brumisateurs, ventilateurs et porte électrique WC (alimentation et commande uniquement) ; luminaires intérieurs (hors DCL) ; peinture après rebouchage ; demande de raccordement / modification d'abonnement Enedis.</t>
+    <t xml:space="preserve">• Bibliothèque : choisir la variante A (spots) OU B (ruban LED) – ne pas additionner les deux. NON COMPRIS : dépose de l'installation existante ; trames chauffantes et thermostats du plancher chauffant ; appliques extérieures des balcons ; fourniture des volets roulants, stores, moteurs, climatisations, électroménager, chauffe-eau, hotte, filtres à eau/air, brumisateurs, ventilateurs et porte électrique WC (alimentation et commande uniquement) ; luminaires intérieurs (hors DCL) ; peinture après rebouchage ; demande de raccordement / modification d'abonnement Enedis.</t>
   </si>
   <si>
     <t xml:space="preserve">• Moteurs de volets et de stores : filaires standard (montée/descente) pour être commandés par les interrupteurs Céliane with Netatmo.</t>
@@ -715,7 +694,7 @@
     <t xml:space="preserve">Éclairage zone nuit (chambres, dégagement, dressing)</t>
   </si>
   <si>
-    <t xml:space="preserve">Prises séjour (8)</t>
+    <t xml:space="preserve">Prises séjour (7)</t>
   </si>
   <si>
     <t xml:space="preserve">20 A</t>
@@ -724,7 +703,7 @@
     <t xml:space="preserve">2,5 mm²</t>
   </si>
   <si>
-    <t xml:space="preserve">Prises chambres 1 et 2 (8)</t>
+    <t xml:space="preserve">Prises chambres 1 et 2 (6)</t>
   </si>
   <si>
     <t xml:space="preserve">16 A</t>
@@ -754,13 +733,13 @@
     <t xml:space="preserve">Éclairage balcons (extérieur)</t>
   </si>
   <si>
-    <t xml:space="preserve">Prises chambre 3, hall, dégagement, dressing (7)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prises SDB 1, SDB 2, buanderie (5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prises balcons + brumisateurs + ventilateurs</t>
+    <t xml:space="preserve">Prises chambre 3, hall, dégagement (5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prises SDB 1, SDB 2 (2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Balcons : brumisateurs + ventilateurs</t>
   </si>
   <si>
     <t xml:space="preserve">Porte électrique WC</t>
@@ -811,7 +790,7 @@
     <t xml:space="preserve">Lave-linge (buanderie)</t>
   </si>
   <si>
-    <t xml:space="preserve">Climatisation séjour</t>
+    <t xml:space="preserve">Climatisation séjour (attente UE)</t>
   </si>
   <si>
     <t xml:space="preserve">Climatisation chambre 1</t>
@@ -874,7 +853,7 @@
     <t xml:space="preserve">PUISSANCE : plancher chauffant (~8,5 kW) + 4 climatisations + cuisson → vérifier l'abonnement (probablement 18 kVA mono ou passage en triphasé). Délesteur conseillé (en option).</t>
   </si>
   <si>
-    <t xml:space="preserve">PLANCHER CHAUFFANT ÉLECTRIQUE (confirmé) : le devis comprend alimentations + régulation. La fourniture/pose des trames reste en option : la passer dans le devis si c'est toi qui les poses.</t>
+    <t xml:space="preserve">PLANCHER CHAUFFANT ÉLECTRIQUE : alimentations en attente uniquement. Trames et thermostats fournis et posés par le fournisseur du plancher (prévoir leurs thermostats compatibles smartphone si la cliente veut tout piloter).</t>
   </si>
   <si>
     <t xml:space="preserve">BUANDERIE : lave-linge, sèche-linge, congélateur et chauffe-eau. Vérifier la place (2,56 m² sur le plan) et le passage des câbles.</t>
@@ -890,6 +869,9 @@
   </si>
   <si>
     <t xml:space="preserve">PIÈCES : la cliente annonce 3 chambres, séjour, cuisine, buanderie, dressing, 2 SDB, WC. Les « SÉCH. » / « RANGT. » du plan sont supposés être la buanderie et le dressing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRISES : nombre minimum NF C 15-100 (séjour 7, chambres 3, cuisine 6, SDB 1, hall et dégagement 1). Dressing, buanderie et WC &lt; 4 m² : pas de prise imposée. Balcons : pas de prise.</t>
   </si>
   <si>
     <t xml:space="preserve">Saignées : 160 ml murs + 70 ml sol estimés pour un immeuble béton – à recaler à la visite (ce poste pèse lourd dans le total).</t>
@@ -1502,7 +1484,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F132"/>
+  <dimension ref="A1:F129"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -2208,7 +2190,7 @@
         <v>2450</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="10" t="s">
         <v>86</v>
       </c>
@@ -2303,14 +2285,14 @@
         <v>37</v>
       </c>
       <c r="D52" s="12" t="n">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="E52" s="13" t="n">
         <v>88</v>
       </c>
       <c r="F52" s="14" t="n">
         <f aca="false">D52*E52</f>
-        <v>2552</v>
+        <v>1848</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2345,14 +2327,14 @@
         <v>37</v>
       </c>
       <c r="D54" s="12" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E54" s="13" t="n">
         <v>125</v>
       </c>
       <c r="F54" s="14" t="n">
         <f aca="false">D54*E54</f>
-        <v>750</v>
+        <v>625</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2361,7 +2343,7 @@
       </c>
       <c r="F55" s="16" t="n">
         <f aca="false">SUM(F52:F54)</f>
-        <v>4127</v>
+        <v>3298</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2397,7 +2379,7 @@
         <v>1350</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="10" t="s">
         <v>106</v>
       </c>
@@ -2474,96 +2456,96 @@
         <v>9</v>
       </c>
       <c r="E64" s="13" t="n">
-        <v>270</v>
+        <v>220</v>
       </c>
       <c r="F64" s="14" t="n">
         <f aca="false">D64*E64</f>
-        <v>2430</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="10" t="s">
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E65" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="B65" s="11" t="s">
+      <c r="F65" s="16" t="n">
+        <f aca="false">SUM(F64:F64)</f>
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="C65" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D65" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="E65" s="13" t="n">
-        <v>235</v>
-      </c>
-      <c r="F65" s="14" t="n">
-        <f aca="false">D65*E65</f>
-        <v>2115</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E66" s="15" t="s">
+      <c r="B67" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="F66" s="16" t="n">
-        <f aca="false">SUM(F64:F65)</f>
-        <v>4545</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="8" t="s">
+      <c r="C67" s="9"/>
+      <c r="D67" s="9"/>
+      <c r="E67" s="9"/>
+      <c r="F67" s="9"/>
+    </row>
+    <row r="68" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="B68" s="9" t="s">
+      <c r="B68" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="C68" s="9"/>
-      <c r="D68" s="9"/>
-      <c r="E68" s="9"/>
-      <c r="F68" s="9"/>
-    </row>
-    <row r="69" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="10" t="s">
+      <c r="C68" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D68" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E68" s="13" t="n">
+        <v>220</v>
+      </c>
+      <c r="F68" s="14" t="n">
+        <f aca="false">D68*E68</f>
+        <v>880</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E69" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="B69" s="11" t="s">
+      <c r="F69" s="16" t="n">
+        <f aca="false">SUM(F68:F68)</f>
+        <v>880</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="C69" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D69" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E69" s="13" t="n">
-        <v>310</v>
-      </c>
-      <c r="F69" s="14" t="n">
-        <f aca="false">D69*E69</f>
-        <v>1240</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E70" s="15" t="s">
+      <c r="B71" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="F70" s="16" t="n">
-        <f aca="false">SUM(F69:F69)</f>
-        <v>1240</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="8" t="s">
+      <c r="C71" s="9"/>
+      <c r="D71" s="9"/>
+      <c r="E71" s="9"/>
+      <c r="F71" s="9"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B72" s="9" t="s">
+      <c r="B72" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="C72" s="9"/>
-      <c r="D72" s="9"/>
-      <c r="E72" s="9"/>
-      <c r="F72" s="9"/>
+      <c r="C72" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D72" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E72" s="13" t="n">
+        <v>270</v>
+      </c>
+      <c r="F72" s="14" t="n">
+        <f aca="false">D72*E72</f>
+        <v>270</v>
+      </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="10" t="s">
@@ -2579,11 +2561,11 @@
         <v>1</v>
       </c>
       <c r="E73" s="13" t="n">
-        <v>270</v>
+        <v>195</v>
       </c>
       <c r="F73" s="14" t="n">
         <f aca="false">D73*E73</f>
-        <v>270</v>
+        <v>195</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2621,11 +2603,11 @@
         <v>1</v>
       </c>
       <c r="E75" s="13" t="n">
-        <v>195</v>
+        <v>180</v>
       </c>
       <c r="F75" s="14" t="n">
         <f aca="false">D75*E75</f>
-        <v>195</v>
+        <v>180</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2642,11 +2624,11 @@
         <v>1</v>
       </c>
       <c r="E76" s="13" t="n">
-        <v>180</v>
+        <v>195</v>
       </c>
       <c r="F76" s="14" t="n">
         <f aca="false">D76*E76</f>
-        <v>180</v>
+        <v>195</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2691,7 +2673,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="10" t="s">
         <v>137</v>
       </c>
@@ -2705,14 +2687,14 @@
         <v>1</v>
       </c>
       <c r="E79" s="13" t="n">
-        <v>195</v>
+        <v>230</v>
       </c>
       <c r="F79" s="14" t="n">
         <f aca="false">D79*E79</f>
-        <v>195</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="10" t="s">
         <v>139</v>
       </c>
@@ -2726,11 +2708,11 @@
         <v>1</v>
       </c>
       <c r="E80" s="13" t="n">
-        <v>230</v>
+        <v>175</v>
       </c>
       <c r="F80" s="14" t="n">
         <f aca="false">D80*E80</f>
-        <v>230</v>
+        <v>175</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2747,11 +2729,11 @@
         <v>1</v>
       </c>
       <c r="E81" s="13" t="n">
-        <v>175</v>
+        <v>250</v>
       </c>
       <c r="F81" s="14" t="n">
         <f aca="false">D81*E81</f>
-        <v>175</v>
+        <v>250</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2768,56 +2750,56 @@
         <v>1</v>
       </c>
       <c r="E82" s="13" t="n">
-        <v>250</v>
+        <v>230</v>
       </c>
       <c r="F82" s="14" t="n">
         <f aca="false">D82*E82</f>
-        <v>250</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A83" s="10" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E83" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="B83" s="11" t="s">
+      <c r="F83" s="16" t="n">
+        <f aca="false">SUM(F72:F82)</f>
+        <v>2310</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="C83" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D83" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E83" s="13" t="n">
-        <v>230</v>
-      </c>
-      <c r="F83" s="14" t="n">
-        <f aca="false">D83*E83</f>
-        <v>230</v>
-      </c>
-    </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E84" s="15" t="s">
+      <c r="B85" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="F84" s="16" t="n">
-        <f aca="false">SUM(F73:F83)</f>
-        <v>2310</v>
-      </c>
-    </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="8" t="s">
+      <c r="C85" s="9"/>
+      <c r="D85" s="9"/>
+      <c r="E85" s="9"/>
+      <c r="F85" s="9"/>
+    </row>
+    <row r="86" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A86" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="B86" s="9" t="s">
+      <c r="B86" s="11" t="s">
         <v>149</v>
       </c>
-      <c r="C86" s="9"/>
-      <c r="D86" s="9"/>
-      <c r="E86" s="9"/>
-      <c r="F86" s="9"/>
-    </row>
-    <row r="87" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C86" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D86" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E86" s="13" t="n">
+        <v>110</v>
+      </c>
+      <c r="F86" s="14" t="n">
+        <f aca="false">D86*E86</f>
+        <v>330</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="10" t="s">
         <v>150</v>
       </c>
@@ -2828,14 +2810,14 @@
         <v>37</v>
       </c>
       <c r="D87" s="12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E87" s="13" t="n">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="F87" s="14" t="n">
         <f aca="false">D87*E87</f>
-        <v>585</v>
+        <v>350</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2852,11 +2834,11 @@
         <v>2</v>
       </c>
       <c r="E88" s="13" t="n">
-        <v>175</v>
+        <v>240</v>
       </c>
       <c r="F88" s="14" t="n">
         <f aca="false">D88*E88</f>
-        <v>350</v>
+        <v>480</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2880,70 +2862,70 @@
         <v>480</v>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A90" s="10" t="s">
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E90" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="B90" s="11" t="s">
+      <c r="F90" s="16" t="n">
+        <f aca="false">SUM(F86:F89)</f>
+        <v>1640</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="C90" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D90" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E90" s="13" t="n">
-        <v>240</v>
-      </c>
-      <c r="F90" s="14" t="n">
-        <f aca="false">D90*E90</f>
-        <v>480</v>
-      </c>
-    </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A91" s="10" t="s">
+      <c r="B92" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="B91" s="11" t="s">
+      <c r="C92" s="9"/>
+      <c r="D92" s="9"/>
+      <c r="E92" s="9"/>
+      <c r="F92" s="9"/>
+    </row>
+    <row r="93" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A93" s="10" t="s">
         <v>159</v>
       </c>
-      <c r="C91" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D91" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E91" s="13" t="n">
+      <c r="B93" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="C93" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D93" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E93" s="13" t="n">
         <v>125</v>
       </c>
-      <c r="F91" s="14" t="n">
-        <f aca="false">D91*E91</f>
-        <v>250</v>
-      </c>
-    </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E92" s="15" t="s">
-        <v>160</v>
-      </c>
-      <c r="F92" s="16" t="n">
-        <f aca="false">SUM(F87:F91)</f>
-        <v>2145</v>
-      </c>
-    </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="8" t="s">
+      <c r="F93" s="14" t="n">
+        <f aca="false">D93*E93</f>
+        <v>375</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A94" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="B94" s="9" t="s">
+      <c r="B94" s="11" t="s">
         <v>162</v>
       </c>
-      <c r="C94" s="9"/>
-      <c r="D94" s="9"/>
-      <c r="E94" s="9"/>
-      <c r="F94" s="9"/>
-    </row>
-    <row r="95" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C94" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D94" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E94" s="13" t="n">
+        <v>270</v>
+      </c>
+      <c r="F94" s="14" t="n">
+        <f aca="false">D94*E94</f>
+        <v>270</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="10" t="s">
         <v>163</v>
       </c>
@@ -2954,14 +2936,14 @@
         <v>37</v>
       </c>
       <c r="D95" s="12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E95" s="13" t="n">
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="F95" s="14" t="n">
         <f aca="false">D95*E95</f>
-        <v>375</v>
+        <v>150</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2975,14 +2957,14 @@
         <v>37</v>
       </c>
       <c r="D96" s="12" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E96" s="13" t="n">
-        <v>270</v>
+        <v>58</v>
       </c>
       <c r="F96" s="14" t="n">
         <f aca="false">D96*E96</f>
-        <v>270</v>
+        <v>406</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2996,14 +2978,14 @@
         <v>37</v>
       </c>
       <c r="D97" s="12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E97" s="13" t="n">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="F97" s="14" t="n">
         <f aca="false">D97*E97</f>
-        <v>150</v>
+        <v>435</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3017,78 +2999,78 @@
         <v>37</v>
       </c>
       <c r="D98" s="12" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E98" s="13" t="n">
-        <v>58</v>
+        <v>350</v>
       </c>
       <c r="F98" s="14" t="n">
         <f aca="false">D98*E98</f>
-        <v>406</v>
-      </c>
-    </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A99" s="10" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E99" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="B99" s="11" t="s">
+      <c r="F99" s="16" t="n">
+        <f aca="false">SUM(F93:F98)</f>
+        <v>2336</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="C99" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D99" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="E99" s="13" t="n">
-        <v>145</v>
-      </c>
-      <c r="F99" s="14" t="n">
-        <f aca="false">D99*E99</f>
-        <v>435</v>
-      </c>
-    </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A100" s="10" t="s">
+      <c r="B101" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="B100" s="11" t="s">
+      <c r="C101" s="9"/>
+      <c r="D101" s="9"/>
+      <c r="E101" s="9"/>
+      <c r="F101" s="9"/>
+    </row>
+    <row r="102" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A102" s="10" t="s">
         <v>174</v>
       </c>
-      <c r="C100" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D100" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E100" s="13" t="n">
-        <v>350</v>
-      </c>
-      <c r="F100" s="14" t="n">
-        <f aca="false">D100*E100</f>
-        <v>700</v>
-      </c>
-    </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E101" s="15" t="s">
+      <c r="B102" s="11" t="s">
         <v>175</v>
       </c>
-      <c r="F101" s="16" t="n">
-        <f aca="false">SUM(F95:F100)</f>
-        <v>2336</v>
-      </c>
-    </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="8" t="s">
+      <c r="C102" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D102" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E102" s="13" t="n">
+        <v>480</v>
+      </c>
+      <c r="F102" s="14" t="n">
+        <f aca="false">D102*E102</f>
+        <v>480</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A103" s="10" t="s">
         <v>176</v>
       </c>
-      <c r="B103" s="9" t="s">
+      <c r="B103" s="11" t="s">
         <v>177</v>
       </c>
-      <c r="C103" s="9"/>
-      <c r="D103" s="9"/>
-      <c r="E103" s="9"/>
-      <c r="F103" s="9"/>
+      <c r="C103" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D103" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E103" s="13" t="n">
+        <v>280</v>
+      </c>
+      <c r="F103" s="14" t="n">
+        <f aca="false">D103*E103</f>
+        <v>280</v>
+      </c>
     </row>
     <row r="104" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="10" t="s">
@@ -3104,109 +3086,109 @@
         <v>1</v>
       </c>
       <c r="E104" s="13" t="n">
-        <v>480</v>
+        <v>360</v>
       </c>
       <c r="F104" s="14" t="n">
         <f aca="false">D104*E104</f>
-        <v>480</v>
-      </c>
-    </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A105" s="10" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E105" s="15" t="s">
         <v>180</v>
       </c>
-      <c r="B105" s="11" t="s">
+      <c r="F105" s="16" t="n">
+        <f aca="false">SUM(F102:F104)</f>
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E107" s="17" t="s">
         <v>181</v>
       </c>
-      <c r="C105" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D105" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E105" s="13" t="n">
-        <v>280</v>
-      </c>
-      <c r="F105" s="14" t="n">
-        <f aca="false">D105*E105</f>
-        <v>280</v>
-      </c>
-    </row>
-    <row r="106" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A106" s="10" t="s">
+      <c r="F107" s="18" t="n">
+        <f aca="false">F13+F21+F41+F49+F55+F61+F65+F69+F83+F90+F99+F105</f>
+        <v>38185</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D108" s="19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E108" s="17" t="s">
         <v>182</v>
       </c>
-      <c r="B106" s="11" t="s">
+      <c r="F108" s="18" t="n">
+        <f aca="false">F107*D108</f>
+        <v>3818.5</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E109" s="20" t="s">
         <v>183</v>
       </c>
-      <c r="C106" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D106" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E106" s="13" t="n">
-        <v>360</v>
-      </c>
-      <c r="F106" s="14" t="n">
-        <f aca="false">D106*E106</f>
-        <v>360</v>
-      </c>
-    </row>
-    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E107" s="15" t="s">
+      <c r="F109" s="21" t="n">
+        <f aca="false">F107+F108</f>
+        <v>42003.5</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E110" s="22" t="s">
         <v>184</v>
       </c>
-      <c r="F107" s="16" t="n">
-        <f aca="false">SUM(F104:F106)</f>
-        <v>1120</v>
-      </c>
-    </row>
-    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E109" s="17" t="s">
+      <c r="F110" s="23" t="n">
+        <f aca="false">F109*0.3</f>
+        <v>12601.05</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="24" t="s">
         <v>185</v>
       </c>
-      <c r="F109" s="18" t="n">
-        <f aca="false">F13+F21+F41+F49+F55+F61+F66+F70+F84+F92+F101+F107</f>
-        <v>42444</v>
-      </c>
-    </row>
-    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D110" s="19" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E110" s="17" t="s">
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A114" s="10" t="s">
         <v>186</v>
       </c>
-      <c r="F110" s="18" t="n">
-        <f aca="false">F109*D110</f>
-        <v>4244.4</v>
-      </c>
-    </row>
-    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E111" s="20" t="s">
+      <c r="B114" s="11" t="s">
         <v>187</v>
       </c>
-      <c r="F111" s="21" t="n">
-        <f aca="false">F109+F110</f>
-        <v>46688.4</v>
-      </c>
-    </row>
-    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E112" s="22" t="s">
+      <c r="C114" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D114" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="E114" s="13" t="n">
+        <v>65</v>
+      </c>
+      <c r="F114" s="14" t="n">
+        <f aca="false">D114*E114</f>
+        <v>780</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A115" s="10" t="s">
         <v>188</v>
       </c>
-      <c r="F112" s="23" t="n">
-        <f aca="false">F111*0.3</f>
-        <v>14006.52</v>
-      </c>
-    </row>
-    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="24" t="s">
+      <c r="B115" s="11" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="116" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C115" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D115" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="E115" s="13" t="n">
+        <v>75</v>
+      </c>
+      <c r="F115" s="14" t="n">
+        <f aca="false">D115*E115</f>
+        <v>600</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="10" t="s">
         <v>190</v>
       </c>
@@ -3214,166 +3196,103 @@
         <v>191</v>
       </c>
       <c r="C116" s="10" t="s">
-        <v>192</v>
+        <v>32</v>
       </c>
       <c r="D116" s="12" t="n">
-        <v>85</v>
+        <v>6</v>
       </c>
       <c r="E116" s="13" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="F116" s="14" t="n">
         <f aca="false">D116*E116</f>
-        <v>6630</v>
+        <v>390</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="B117" s="11" t="s">
         <v>193</v>
       </c>
-      <c r="B117" s="11" t="s">
-        <v>194</v>
-      </c>
       <c r="C117" s="10" t="s">
         <v>37</v>
       </c>
       <c r="D117" s="12" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E117" s="13" t="n">
-        <v>65</v>
+        <v>120</v>
       </c>
       <c r="F117" s="14" t="n">
         <f aca="false">D117*E117</f>
-        <v>780</v>
-      </c>
-    </row>
-    <row r="118" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="10" t="s">
+        <v>194</v>
+      </c>
+      <c r="B118" s="11" t="s">
         <v>195</v>
       </c>
-      <c r="B118" s="11" t="s">
-        <v>196</v>
-      </c>
       <c r="C118" s="10" t="s">
         <v>37</v>
       </c>
       <c r="D118" s="12" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E118" s="13" t="n">
-        <v>75</v>
+        <v>420</v>
       </c>
       <c r="F118" s="14" t="n">
         <f aca="false">D118*E118</f>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A119" s="10" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E119" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="F119" s="16" t="n">
+        <f aca="false">SUM(F114:F118)</f>
+        <v>2310</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="B119" s="11" t="s">
+    </row>
+    <row r="123" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B123" s="25" t="s">
         <v>198</v>
       </c>
-      <c r="C119" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="D119" s="12" t="n">
-        <v>12</v>
-      </c>
-      <c r="E119" s="13" t="n">
-        <v>65</v>
-      </c>
-      <c r="F119" s="14" t="n">
-        <f aca="false">D119*E119</f>
-        <v>780</v>
-      </c>
-    </row>
-    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A120" s="10" t="s">
+    </row>
+    <row r="124" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B124" s="25" t="s">
         <v>199</v>
       </c>
-      <c r="B120" s="11" t="s">
+    </row>
+    <row r="125" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B125" s="25" t="s">
         <v>200</v>
       </c>
-      <c r="C120" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D120" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E120" s="13" t="n">
-        <v>120</v>
-      </c>
-      <c r="F120" s="14" t="n">
-        <f aca="false">D120*E120</f>
-        <v>120</v>
-      </c>
-    </row>
-    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A121" s="10" t="s">
+    </row>
+    <row r="126" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B126" s="25" t="s">
         <v>201</v>
       </c>
-      <c r="B121" s="11" t="s">
+    </row>
+    <row r="127" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B127" s="25" t="s">
         <v>202</v>
       </c>
-      <c r="C121" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D121" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E121" s="13" t="n">
-        <v>420</v>
-      </c>
-      <c r="F121" s="14" t="n">
-        <f aca="false">D121*E121</f>
-        <v>420</v>
-      </c>
-    </row>
-    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E122" s="15" t="s">
+    </row>
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B129" s="2" t="s">
         <v>203</v>
-      </c>
-      <c r="F122" s="16" t="n">
-        <f aca="false">SUM(F116:F121)</f>
-        <v>9330</v>
-      </c>
-    </row>
-    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A125" s="2" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="126" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B126" s="25" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="127" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B127" s="25" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="128" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B128" s="25" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="129" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B129" s="25" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="130" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B130" s="25" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B132" s="2" t="s">
-        <v>210</v>
       </c>
     </row>
   </sheetData>
@@ -3404,12 +3323,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="26" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="27" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3417,16 +3336,16 @@
         <v>14</v>
       </c>
       <c r="B4" s="28" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="C4" s="28" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="D4" s="28" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="E4" s="28" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3434,16 +3353,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="D5" s="29" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3451,16 +3370,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="29" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="C6" s="29" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="D6" s="29" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="E6" s="29" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3468,16 +3387,16 @@
         <v>3</v>
       </c>
       <c r="B7" s="29" t="s">
+        <v>210</v>
+      </c>
+      <c r="C7" s="29" t="s">
+        <v>215</v>
+      </c>
+      <c r="D7" s="29" t="s">
+        <v>216</v>
+      </c>
+      <c r="E7" s="29" t="s">
         <v>217</v>
-      </c>
-      <c r="C7" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="D7" s="29" t="s">
-        <v>223</v>
-      </c>
-      <c r="E7" s="29" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3485,16 +3404,16 @@
         <v>4</v>
       </c>
       <c r="B8" s="29" t="s">
+        <v>210</v>
+      </c>
+      <c r="C8" s="29" t="s">
+        <v>218</v>
+      </c>
+      <c r="D8" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="E8" s="29" t="s">
         <v>217</v>
-      </c>
-      <c r="C8" s="29" t="s">
-        <v>225</v>
-      </c>
-      <c r="D8" s="29" t="s">
-        <v>226</v>
-      </c>
-      <c r="E8" s="29" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3502,16 +3421,16 @@
         <v>5</v>
       </c>
       <c r="B9" s="29" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="D9" s="29" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3519,16 +3438,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="29" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="D10" s="29" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3536,16 +3455,16 @@
         <v>7</v>
       </c>
       <c r="B11" s="29" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="C11" s="29" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="D11" s="29" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="E11" s="29" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3553,16 +3472,16 @@
         <v>8</v>
       </c>
       <c r="B12" s="29" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="C12" s="29" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="D12" s="29" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="E12" s="29" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3570,16 +3489,16 @@
         <v>9</v>
       </c>
       <c r="B13" s="29" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="C13" s="29" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="D13" s="29" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="E13" s="29" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3587,16 +3506,16 @@
         <v>10</v>
       </c>
       <c r="B14" s="29" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="D14" s="29" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="E14" s="29" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3604,16 +3523,16 @@
         <v>11</v>
       </c>
       <c r="B15" s="29" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="C15" s="29" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="D15" s="29" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="E15" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3621,16 +3540,16 @@
         <v>12</v>
       </c>
       <c r="B16" s="29" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="C16" s="29" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="D16" s="29" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="E16" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3638,16 +3557,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="29" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="C17" s="29" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="D17" s="29" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="E17" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3655,16 +3574,16 @@
         <v>14</v>
       </c>
       <c r="B18" s="29" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="C18" s="29" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="D18" s="29" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="E18" s="29" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3672,16 +3591,16 @@
         <v>15</v>
       </c>
       <c r="B19" s="29" t="s">
+        <v>225</v>
+      </c>
+      <c r="C19" s="29" t="s">
         <v>232</v>
       </c>
-      <c r="C19" s="29" t="s">
-        <v>239</v>
-      </c>
       <c r="D19" s="29" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="E19" s="29" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3689,16 +3608,16 @@
         <v>16</v>
       </c>
       <c r="B20" s="29" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="C20" s="29" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="D20" s="29" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="E20" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3706,16 +3625,16 @@
         <v>17</v>
       </c>
       <c r="B21" s="29" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="C21" s="29" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="D21" s="29" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="E21" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3723,16 +3642,16 @@
         <v>18</v>
       </c>
       <c r="B22" s="29" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="C22" s="29" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="D22" s="29" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="E22" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3740,16 +3659,16 @@
         <v>19</v>
       </c>
       <c r="B23" s="29" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="C23" s="29" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="D23" s="29" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="E23" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3757,16 +3676,16 @@
         <v>20</v>
       </c>
       <c r="B24" s="29" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="C24" s="29" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="D24" s="29" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="E24" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3774,16 +3693,16 @@
         <v>21</v>
       </c>
       <c r="B25" s="29" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="C25" s="29" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="D25" s="29" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="E25" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3791,16 +3710,16 @@
         <v>22</v>
       </c>
       <c r="B26" s="29" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="C26" s="29" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="D26" s="29" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="E26" s="29" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3808,16 +3727,16 @@
         <v>23</v>
       </c>
       <c r="B27" s="29" t="s">
+        <v>234</v>
+      </c>
+      <c r="C27" s="29" t="s">
         <v>241</v>
       </c>
-      <c r="C27" s="29" t="s">
-        <v>248</v>
-      </c>
       <c r="D27" s="29" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="E27" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3825,16 +3744,16 @@
         <v>24</v>
       </c>
       <c r="B28" s="29" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="C28" s="29" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="D28" s="29" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="E28" s="29" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3842,16 +3761,16 @@
         <v>25</v>
       </c>
       <c r="B29" s="29" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="C29" s="29" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="D29" s="29" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="E29" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3859,16 +3778,16 @@
         <v>26</v>
       </c>
       <c r="B30" s="29" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="C30" s="29" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="D30" s="29" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="E30" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3876,16 +3795,16 @@
         <v>27</v>
       </c>
       <c r="B31" s="29" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="C31" s="29" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="D31" s="29" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="E31" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3893,16 +3812,16 @@
         <v>28</v>
       </c>
       <c r="B32" s="29" t="s">
+        <v>242</v>
+      </c>
+      <c r="C32" s="29" t="s">
         <v>249</v>
       </c>
-      <c r="C32" s="29" t="s">
-        <v>256</v>
-      </c>
       <c r="D32" s="29" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="E32" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3910,16 +3829,16 @@
         <v>29</v>
       </c>
       <c r="B33" s="29" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="C33" s="29" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="D33" s="29" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="E33" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3927,16 +3846,16 @@
         <v>30</v>
       </c>
       <c r="B34" s="29" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="C34" s="29" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="D34" s="29" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="E34" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3944,16 +3863,16 @@
         <v>31</v>
       </c>
       <c r="B35" s="29" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="C35" s="29" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="D35" s="29" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="E35" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3961,16 +3880,16 @@
         <v>32</v>
       </c>
       <c r="B36" s="29" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="C36" s="29" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="D36" s="29" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="E36" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3978,16 +3897,16 @@
         <v>33</v>
       </c>
       <c r="B37" s="29" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="C37" s="29" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="D37" s="29" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="E37" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3995,16 +3914,16 @@
         <v>34</v>
       </c>
       <c r="B38" s="29" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="C38" s="29" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="D38" s="29" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="E38" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4012,16 +3931,16 @@
         <v>35</v>
       </c>
       <c r="B39" s="29" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="C39" s="29" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="D39" s="29" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="E39" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4029,16 +3948,16 @@
         <v>36</v>
       </c>
       <c r="B40" s="29" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="C40" s="29" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="D40" s="29" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="E40" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4046,16 +3965,16 @@
         <v>37</v>
       </c>
       <c r="B41" s="29" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="C41" s="29" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="D41" s="29" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="E41" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4063,21 +3982,21 @@
         <v>38</v>
       </c>
       <c r="B42" s="29" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="C42" s="29" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="D42" s="29" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="E42" s="29" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C44" s="2" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="D44" s="2" t="n">
         <f aca="false">COUNTA(C5:C42)</f>
@@ -4086,7 +4005,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C45" s="5" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="D45" s="30" t="n">
         <f aca="false">MAX(COUNTIF(B5:B42,"ID1*"),COUNTIF(B5:B42,"ID2*"),COUNTIF(B5:B42,"ID3*"),COUNTIF(B5:B42,"ID4*"),COUNTIF(B5:B42,"ID5*"),COUNTIF(B5:B42,"ID6*"))</f>
@@ -4118,92 +4037,100 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="26" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
+        <v>265</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>272</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>282</v>
+        <v>275</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="s">
+        <v>265</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="31" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Devis sans TVA (micro-entreprise, art. 293 B du CGI)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BjWSBdyxAjsRnCWBVUUVzr
</commit_message>
<xml_diff>
--- a/devis/Devis_electricite_T4_connecte_Legrand.xlsx
+++ b/devis/Devis_electricite_T4_connecte_Legrand.xlsx
@@ -24,30 +24,8 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <authors>
-    <author>Unknown Author</author>
-  </authors>
-  <commentList>
-    <comment ref="D108" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">TVA 10 % : travaux d'amélioration dans un logement de plus de 2 ans (attestation simplifiée à faire signer par la cliente). Mettre 20 % si non éligible.</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="277">
   <si>
     <t xml:space="preserve">MAUREL'EC</t>
   </si>
@@ -76,7 +54,7 @@
     <t xml:space="preserve">3 mois</t>
   </si>
   <si>
-    <t xml:space="preserve">SIRET : [à compléter] – Assurance décennale : [à compléter]</t>
+    <t xml:space="preserve">Entrepreneur individuel (micro-entreprise) – SIRET : [à compléter] – Assurance décennale : [à compléter]</t>
   </si>
   <si>
     <t xml:space="preserve">CLIENTE :</t>
@@ -103,10 +81,10 @@
     <t xml:space="preserve">Qté</t>
   </si>
   <si>
-    <t xml:space="preserve">PU HT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total HT</t>
+    <t xml:space="preserve">PU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
   </si>
   <si>
     <t xml:space="preserve">1</t>
@@ -592,13 +570,10 @@
     <t xml:space="preserve">Sous-total lot 12</t>
   </si>
   <si>
-    <t xml:space="preserve">TOTAL HT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TVA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL TTC</t>
+    <t xml:space="preserve">TOTAL NET À PAYER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TVA non applicable, article 293 B du CGI</t>
   </si>
   <si>
     <t xml:space="preserve">Acompte 30 % à la commande</t>
@@ -637,7 +612,7 @@
     <t xml:space="preserve">Délesteur / gestionnaire d'énergie (chauffage + climatisations)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total options HT</t>
+    <t xml:space="preserve">Total options</t>
   </si>
   <si>
     <t xml:space="preserve">CONDITIONS ET RÉSERVES</t>
@@ -880,18 +855,17 @@
     <t xml:space="preserve">Prix fourniture + pose basés sur des tarifs publics moyens Legrand/Netatmo : à vérifier avec ton grossiste et à ajuster selon ta remise.</t>
   </si>
   <si>
-    <t xml:space="preserve">Légende : chiffres en BLEU = quantités / prix modifiables ; cellule JAUNE = taux de TVA.</t>
+    <t xml:space="preserve">Légende : chiffres en BLEU = quantités / prix modifiables. Montants sans TVA (micro-entreprise, art. 293 B du CGI).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.00&quot; €&quot;;\-#,##0.00&quot; €&quot;;\-"/>
-    <numFmt numFmtId="166" formatCode="0%"/>
-    <numFmt numFmtId="167" formatCode="General"/>
+    <numFmt numFmtId="166" formatCode="General"/>
   </numFmts>
   <fonts count="18">
     <font>
@@ -986,16 +960,20 @@
     </font>
     <font>
       <b val="true"/>
+      <i val="true"/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="11"/>
       <color rgb="FFC00000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -1022,7 +1000,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1039,12 +1017,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
         <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -1103,7 +1075,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1172,24 +1144,16 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -1200,7 +1164,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1224,7 +1188,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1484,7 +1448,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F129"/>
+  <dimension ref="A1:F128"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -3112,15 +3076,8 @@
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D108" s="19" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E108" s="17" t="s">
+      <c r="E108" s="19" t="s">
         <v>182</v>
-      </c>
-      <c r="F108" s="18" t="n">
-        <f aca="false">F107*D108</f>
-        <v>3818.5</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3128,93 +3085,105 @@
         <v>183</v>
       </c>
       <c r="F109" s="21" t="n">
-        <f aca="false">F107+F108</f>
-        <v>42003.5</v>
-      </c>
-    </row>
-    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E110" s="22" t="s">
+        <f aca="false">F107*0.3</f>
+        <v>11455.5</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="22" t="s">
         <v>184</v>
       </c>
-      <c r="F110" s="23" t="n">
-        <f aca="false">F109*0.3</f>
-        <v>12601.05</v>
-      </c>
-    </row>
-    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="24" t="s">
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A113" s="10" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B113" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="C113" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D113" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="E113" s="13" t="n">
+        <v>65</v>
+      </c>
+      <c r="F113" s="14" t="n">
+        <f aca="false">D113*E113</f>
+        <v>780</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B114" s="11" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C114" s="10" t="s">
         <v>37</v>
       </c>
       <c r="D114" s="12" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E114" s="13" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="F114" s="14" t="n">
         <f aca="false">D114*E114</f>
-        <v>780</v>
-      </c>
-    </row>
-    <row r="115" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="10" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B115" s="11" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C115" s="10" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D115" s="12" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E115" s="13" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="F115" s="14" t="n">
         <f aca="false">D115*E115</f>
-        <v>600</v>
+        <v>390</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B116" s="11" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C116" s="10" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D116" s="12" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E116" s="13" t="n">
-        <v>65</v>
+        <v>120</v>
       </c>
       <c r="F116" s="14" t="n">
         <f aca="false">D116*E116</f>
-        <v>390</v>
+        <v>120</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="10" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B117" s="11" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C117" s="10" t="s">
         <v>37</v>
@@ -3223,76 +3192,55 @@
         <v>1</v>
       </c>
       <c r="E117" s="13" t="n">
-        <v>120</v>
+        <v>420</v>
       </c>
       <c r="F117" s="14" t="n">
         <f aca="false">D117*E117</f>
-        <v>120</v>
-      </c>
-    </row>
-    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A118" s="10" t="s">
-        <v>194</v>
-      </c>
-      <c r="B118" s="11" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E118" s="15" t="s">
         <v>195</v>
       </c>
-      <c r="C118" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D118" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E118" s="13" t="n">
-        <v>420</v>
-      </c>
-      <c r="F118" s="14" t="n">
-        <f aca="false">D118*E118</f>
-        <v>420</v>
-      </c>
-    </row>
-    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E119" s="15" t="s">
+      <c r="F118" s="16" t="n">
+        <f aca="false">SUM(F113:F117)</f>
+        <v>2310</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="F119" s="16" t="n">
-        <f aca="false">SUM(F114:F118)</f>
-        <v>2310</v>
-      </c>
-    </row>
-    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A122" s="2" t="s">
+    </row>
+    <row r="122" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B122" s="23" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="123" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B123" s="25" t="s">
+    <row r="123" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B123" s="23" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="124" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B124" s="25" t="s">
+    <row r="124" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B124" s="23" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="125" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B125" s="25" t="s">
+    <row r="125" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B125" s="23" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="126" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B126" s="25" t="s">
+    <row r="126" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B126" s="23" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="127" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B127" s="25" t="s">
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B128" s="2" t="s">
         <v>202</v>
-      </c>
-    </row>
-    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B129" s="2" t="s">
-        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -3303,7 +3251,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -3322,681 +3269,681 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="24" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="25" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="27" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="26" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="28" t="s">
+      <c r="C4" s="26" t="s">
+        <v>206</v>
+      </c>
+      <c r="D4" s="26" t="s">
+        <v>207</v>
+      </c>
+      <c r="E4" s="26" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>209</v>
+      </c>
+      <c r="C5" s="27" t="s">
+        <v>210</v>
+      </c>
+      <c r="D5" s="27" t="s">
+        <v>211</v>
+      </c>
+      <c r="E5" s="27" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="27" t="s">
+        <v>209</v>
+      </c>
+      <c r="C6" s="27" t="s">
+        <v>213</v>
+      </c>
+      <c r="D6" s="27" t="s">
+        <v>211</v>
+      </c>
+      <c r="E6" s="27" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="27" t="s">
+        <v>209</v>
+      </c>
+      <c r="C7" s="27" t="s">
+        <v>214</v>
+      </c>
+      <c r="D7" s="27" t="s">
+        <v>215</v>
+      </c>
+      <c r="E7" s="27" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="27" t="s">
+        <v>209</v>
+      </c>
+      <c r="C8" s="27" t="s">
+        <v>217</v>
+      </c>
+      <c r="D8" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="E8" s="27" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="27" t="s">
+        <v>209</v>
+      </c>
+      <c r="C9" s="27" t="s">
+        <v>219</v>
+      </c>
+      <c r="D9" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="E9" s="27" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="27" t="s">
+        <v>209</v>
+      </c>
+      <c r="C10" s="27" t="s">
+        <v>220</v>
+      </c>
+      <c r="D10" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="E10" s="27" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="27" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="27" t="s">
+        <v>209</v>
+      </c>
+      <c r="C11" s="27" t="s">
+        <v>221</v>
+      </c>
+      <c r="D11" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="E11" s="27" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="27" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="27" t="s">
+        <v>209</v>
+      </c>
+      <c r="C12" s="27" t="s">
+        <v>222</v>
+      </c>
+      <c r="D12" s="27" t="s">
+        <v>223</v>
+      </c>
+      <c r="E12" s="27" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="27" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="27" t="s">
+        <v>224</v>
+      </c>
+      <c r="C13" s="27" t="s">
+        <v>225</v>
+      </c>
+      <c r="D13" s="27" t="s">
+        <v>211</v>
+      </c>
+      <c r="E13" s="27" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="27" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="27" t="s">
+        <v>224</v>
+      </c>
+      <c r="C14" s="27" t="s">
+        <v>226</v>
+      </c>
+      <c r="D14" s="27" t="s">
+        <v>211</v>
+      </c>
+      <c r="E14" s="27" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="27" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="27" t="s">
+        <v>224</v>
+      </c>
+      <c r="C15" s="27" t="s">
+        <v>227</v>
+      </c>
+      <c r="D15" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="E15" s="27" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="27" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="27" t="s">
+        <v>224</v>
+      </c>
+      <c r="C16" s="27" t="s">
+        <v>228</v>
+      </c>
+      <c r="D16" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="E16" s="27" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="27" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="27" t="s">
+        <v>224</v>
+      </c>
+      <c r="C17" s="27" t="s">
+        <v>229</v>
+      </c>
+      <c r="D17" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="E17" s="27" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="27" t="n">
         <v>14</v>
       </c>
-      <c r="B4" s="28" t="s">
-        <v>206</v>
-      </c>
-      <c r="C4" s="28" t="s">
-        <v>207</v>
-      </c>
-      <c r="D4" s="28" t="s">
-        <v>208</v>
-      </c>
-      <c r="E4" s="28" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="29" t="s">
-        <v>210</v>
-      </c>
-      <c r="C5" s="29" t="s">
-        <v>211</v>
-      </c>
-      <c r="D5" s="29" t="s">
+      <c r="B18" s="27" t="s">
+        <v>224</v>
+      </c>
+      <c r="C18" s="27" t="s">
+        <v>230</v>
+      </c>
+      <c r="D18" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="E18" s="27" t="s">
         <v>212</v>
       </c>
-      <c r="E5" s="29" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="29" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="29" t="s">
-        <v>210</v>
-      </c>
-      <c r="C6" s="29" t="s">
-        <v>214</v>
-      </c>
-      <c r="D6" s="29" t="s">
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="27" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="27" t="s">
+        <v>224</v>
+      </c>
+      <c r="C19" s="27" t="s">
+        <v>231</v>
+      </c>
+      <c r="D19" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="E19" s="27" t="s">
         <v>212</v>
       </c>
-      <c r="E6" s="29" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="29" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="29" t="s">
-        <v>210</v>
-      </c>
-      <c r="C7" s="29" t="s">
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="27" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="27" t="s">
+        <v>224</v>
+      </c>
+      <c r="C20" s="27" t="s">
+        <v>232</v>
+      </c>
+      <c r="D20" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="E20" s="27" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="27" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="27" t="s">
+        <v>233</v>
+      </c>
+      <c r="C21" s="27" t="s">
+        <v>234</v>
+      </c>
+      <c r="D21" s="27" t="s">
         <v>215</v>
       </c>
-      <c r="D7" s="29" t="s">
+      <c r="E21" s="27" t="s">
         <v>216</v>
       </c>
-      <c r="E7" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="29" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="29" t="s">
-        <v>210</v>
-      </c>
-      <c r="C8" s="29" t="s">
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="27" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="27" t="s">
+        <v>233</v>
+      </c>
+      <c r="C22" s="27" t="s">
+        <v>235</v>
+      </c>
+      <c r="D22" s="27" t="s">
+        <v>215</v>
+      </c>
+      <c r="E22" s="27" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="27" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="27" t="s">
+        <v>233</v>
+      </c>
+      <c r="C23" s="27" t="s">
+        <v>236</v>
+      </c>
+      <c r="D23" s="27" t="s">
+        <v>215</v>
+      </c>
+      <c r="E23" s="27" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="27" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="27" t="s">
+        <v>233</v>
+      </c>
+      <c r="C24" s="27" t="s">
+        <v>237</v>
+      </c>
+      <c r="D24" s="27" t="s">
+        <v>215</v>
+      </c>
+      <c r="E24" s="27" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="27" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="27" t="s">
+        <v>233</v>
+      </c>
+      <c r="C25" s="27" t="s">
+        <v>238</v>
+      </c>
+      <c r="D25" s="27" t="s">
+        <v>215</v>
+      </c>
+      <c r="E25" s="27" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="27" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="27" t="s">
+        <v>233</v>
+      </c>
+      <c r="C26" s="27" t="s">
+        <v>239</v>
+      </c>
+      <c r="D26" s="27" t="s">
         <v>218</v>
       </c>
-      <c r="D8" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="E8" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="29" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="29" t="s">
-        <v>210</v>
-      </c>
-      <c r="C9" s="29" t="s">
-        <v>220</v>
-      </c>
-      <c r="D9" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="E9" s="29" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="29" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="29" t="s">
-        <v>210</v>
-      </c>
-      <c r="C10" s="29" t="s">
-        <v>221</v>
-      </c>
-      <c r="D10" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="E10" s="29" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="29" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="29" t="s">
-        <v>210</v>
-      </c>
-      <c r="C11" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="D11" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="E11" s="29" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="29" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="29" t="s">
-        <v>210</v>
-      </c>
-      <c r="C12" s="29" t="s">
-        <v>223</v>
-      </c>
-      <c r="D12" s="29" t="s">
-        <v>224</v>
-      </c>
-      <c r="E12" s="29" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="29" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="29" t="s">
-        <v>225</v>
-      </c>
-      <c r="C13" s="29" t="s">
-        <v>226</v>
-      </c>
-      <c r="D13" s="29" t="s">
+      <c r="E26" s="27" t="s">
         <v>212</v>
       </c>
-      <c r="E13" s="29" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="29" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="29" t="s">
-        <v>225</v>
-      </c>
-      <c r="C14" s="29" t="s">
-        <v>227</v>
-      </c>
-      <c r="D14" s="29" t="s">
-        <v>212</v>
-      </c>
-      <c r="E14" s="29" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="29" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="29" t="s">
-        <v>225</v>
-      </c>
-      <c r="C15" s="29" t="s">
-        <v>228</v>
-      </c>
-      <c r="D15" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="E15" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="29" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="29" t="s">
-        <v>225</v>
-      </c>
-      <c r="C16" s="29" t="s">
-        <v>229</v>
-      </c>
-      <c r="D16" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="E16" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="29" t="n">
-        <v>13</v>
-      </c>
-      <c r="B17" s="29" t="s">
-        <v>225</v>
-      </c>
-      <c r="C17" s="29" t="s">
-        <v>230</v>
-      </c>
-      <c r="D17" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="E17" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="29" t="n">
-        <v>14</v>
-      </c>
-      <c r="B18" s="29" t="s">
-        <v>225</v>
-      </c>
-      <c r="C18" s="29" t="s">
-        <v>231</v>
-      </c>
-      <c r="D18" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="E18" s="29" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="29" t="n">
-        <v>15</v>
-      </c>
-      <c r="B19" s="29" t="s">
-        <v>225</v>
-      </c>
-      <c r="C19" s="29" t="s">
-        <v>232</v>
-      </c>
-      <c r="D19" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="E19" s="29" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="29" t="n">
-        <v>16</v>
-      </c>
-      <c r="B20" s="29" t="s">
-        <v>225</v>
-      </c>
-      <c r="C20" s="29" t="s">
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="27" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="27" t="s">
         <v>233</v>
       </c>
-      <c r="D20" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="E20" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="29" t="n">
-        <v>17</v>
-      </c>
-      <c r="B21" s="29" t="s">
-        <v>234</v>
-      </c>
-      <c r="C21" s="29" t="s">
-        <v>235</v>
-      </c>
-      <c r="D21" s="29" t="s">
+      <c r="C27" s="27" t="s">
+        <v>240</v>
+      </c>
+      <c r="D27" s="27" t="s">
+        <v>215</v>
+      </c>
+      <c r="E27" s="27" t="s">
         <v>216</v>
       </c>
-      <c r="E21" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="29" t="n">
-        <v>18</v>
-      </c>
-      <c r="B22" s="29" t="s">
-        <v>234</v>
-      </c>
-      <c r="C22" s="29" t="s">
-        <v>236</v>
-      </c>
-      <c r="D22" s="29" t="s">
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="27" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="27" t="s">
+        <v>241</v>
+      </c>
+      <c r="C28" s="27" t="s">
+        <v>242</v>
+      </c>
+      <c r="D28" s="27" t="s">
+        <v>243</v>
+      </c>
+      <c r="E28" s="27" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="27" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="27" t="s">
+        <v>241</v>
+      </c>
+      <c r="C29" s="27" t="s">
+        <v>245</v>
+      </c>
+      <c r="D29" s="27" t="s">
+        <v>215</v>
+      </c>
+      <c r="E29" s="27" t="s">
         <v>216</v>
       </c>
-      <c r="E22" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="29" t="n">
-        <v>19</v>
-      </c>
-      <c r="B23" s="29" t="s">
-        <v>234</v>
-      </c>
-      <c r="C23" s="29" t="s">
-        <v>237</v>
-      </c>
-      <c r="D23" s="29" t="s">
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="27" t="s">
+        <v>241</v>
+      </c>
+      <c r="C30" s="27" t="s">
+        <v>246</v>
+      </c>
+      <c r="D30" s="27" t="s">
+        <v>215</v>
+      </c>
+      <c r="E30" s="27" t="s">
         <v>216</v>
       </c>
-      <c r="E23" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="29" t="n">
-        <v>20</v>
-      </c>
-      <c r="B24" s="29" t="s">
-        <v>234</v>
-      </c>
-      <c r="C24" s="29" t="s">
-        <v>238</v>
-      </c>
-      <c r="D24" s="29" t="s">
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="27" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="27" t="s">
+        <v>241</v>
+      </c>
+      <c r="C31" s="27" t="s">
+        <v>247</v>
+      </c>
+      <c r="D31" s="27" t="s">
+        <v>215</v>
+      </c>
+      <c r="E31" s="27" t="s">
         <v>216</v>
       </c>
-      <c r="E24" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="29" t="n">
-        <v>21</v>
-      </c>
-      <c r="B25" s="29" t="s">
-        <v>234</v>
-      </c>
-      <c r="C25" s="29" t="s">
-        <v>239</v>
-      </c>
-      <c r="D25" s="29" t="s">
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="27" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="27" t="s">
+        <v>241</v>
+      </c>
+      <c r="C32" s="27" t="s">
+        <v>248</v>
+      </c>
+      <c r="D32" s="27" t="s">
+        <v>215</v>
+      </c>
+      <c r="E32" s="27" t="s">
         <v>216</v>
       </c>
-      <c r="E25" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="29" t="n">
-        <v>22</v>
-      </c>
-      <c r="B26" s="29" t="s">
-        <v>234</v>
-      </c>
-      <c r="C26" s="29" t="s">
-        <v>240</v>
-      </c>
-      <c r="D26" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="E26" s="29" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="29" t="n">
-        <v>23</v>
-      </c>
-      <c r="B27" s="29" t="s">
-        <v>234</v>
-      </c>
-      <c r="C27" s="29" t="s">
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="27" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="27" t="s">
         <v>241</v>
       </c>
-      <c r="D27" s="29" t="s">
+      <c r="C33" s="27" t="s">
+        <v>249</v>
+      </c>
+      <c r="D33" s="27" t="s">
+        <v>215</v>
+      </c>
+      <c r="E33" s="27" t="s">
         <v>216</v>
       </c>
-      <c r="E27" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="29" t="n">
-        <v>24</v>
-      </c>
-      <c r="B28" s="29" t="s">
-        <v>242</v>
-      </c>
-      <c r="C28" s="29" t="s">
-        <v>243</v>
-      </c>
-      <c r="D28" s="29" t="s">
-        <v>244</v>
-      </c>
-      <c r="E28" s="29" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="29" t="n">
-        <v>25</v>
-      </c>
-      <c r="B29" s="29" t="s">
-        <v>242</v>
-      </c>
-      <c r="C29" s="29" t="s">
-        <v>246</v>
-      </c>
-      <c r="D29" s="29" t="s">
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="27" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="27" t="s">
+        <v>250</v>
+      </c>
+      <c r="C34" s="27" t="s">
+        <v>251</v>
+      </c>
+      <c r="D34" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="E34" s="27" t="s">
         <v>216</v>
       </c>
-      <c r="E29" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="29" t="n">
-        <v>26</v>
-      </c>
-      <c r="B30" s="29" t="s">
-        <v>242</v>
-      </c>
-      <c r="C30" s="29" t="s">
-        <v>247</v>
-      </c>
-      <c r="D30" s="29" t="s">
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="27" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="27" t="s">
+        <v>250</v>
+      </c>
+      <c r="C35" s="27" t="s">
+        <v>252</v>
+      </c>
+      <c r="D35" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="E35" s="27" t="s">
         <v>216</v>
       </c>
-      <c r="E30" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="29" t="n">
-        <v>27</v>
-      </c>
-      <c r="B31" s="29" t="s">
-        <v>242</v>
-      </c>
-      <c r="C31" s="29" t="s">
-        <v>248</v>
-      </c>
-      <c r="D31" s="29" t="s">
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="27" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="27" t="s">
+        <v>250</v>
+      </c>
+      <c r="C36" s="27" t="s">
+        <v>253</v>
+      </c>
+      <c r="D36" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="E36" s="27" t="s">
         <v>216</v>
       </c>
-      <c r="E31" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="29" t="n">
-        <v>28</v>
-      </c>
-      <c r="B32" s="29" t="s">
-        <v>242</v>
-      </c>
-      <c r="C32" s="29" t="s">
-        <v>249</v>
-      </c>
-      <c r="D32" s="29" t="s">
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="27" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="27" t="s">
+        <v>250</v>
+      </c>
+      <c r="C37" s="27" t="s">
+        <v>254</v>
+      </c>
+      <c r="D37" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="E37" s="27" t="s">
         <v>216</v>
       </c>
-      <c r="E32" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="29" t="n">
-        <v>29</v>
-      </c>
-      <c r="B33" s="29" t="s">
-        <v>242</v>
-      </c>
-      <c r="C33" s="29" t="s">
-        <v>250</v>
-      </c>
-      <c r="D33" s="29" t="s">
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="27" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="27" t="s">
+        <v>255</v>
+      </c>
+      <c r="C38" s="27" t="s">
+        <v>256</v>
+      </c>
+      <c r="D38" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="E38" s="27" t="s">
         <v>216</v>
       </c>
-      <c r="E33" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="29" t="n">
-        <v>30</v>
-      </c>
-      <c r="B34" s="29" t="s">
-        <v>251</v>
-      </c>
-      <c r="C34" s="29" t="s">
-        <v>252</v>
-      </c>
-      <c r="D34" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="E34" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="29" t="n">
-        <v>31</v>
-      </c>
-      <c r="B35" s="29" t="s">
-        <v>251</v>
-      </c>
-      <c r="C35" s="29" t="s">
-        <v>253</v>
-      </c>
-      <c r="D35" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="E35" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="29" t="n">
-        <v>32</v>
-      </c>
-      <c r="B36" s="29" t="s">
-        <v>251</v>
-      </c>
-      <c r="C36" s="29" t="s">
-        <v>254</v>
-      </c>
-      <c r="D36" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="E36" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="29" t="n">
-        <v>33</v>
-      </c>
-      <c r="B37" s="29" t="s">
-        <v>251</v>
-      </c>
-      <c r="C37" s="29" t="s">
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="27" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="27" t="s">
         <v>255</v>
       </c>
-      <c r="D37" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="E37" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="29" t="n">
-        <v>34</v>
-      </c>
-      <c r="B38" s="29" t="s">
-        <v>256</v>
-      </c>
-      <c r="C38" s="29" t="s">
+      <c r="C39" s="27" t="s">
         <v>257</v>
       </c>
-      <c r="D38" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="E38" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="29" t="n">
-        <v>35</v>
-      </c>
-      <c r="B39" s="29" t="s">
-        <v>256</v>
-      </c>
-      <c r="C39" s="29" t="s">
+      <c r="D39" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="E39" s="27" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="27" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="27" t="s">
+        <v>255</v>
+      </c>
+      <c r="C40" s="27" t="s">
         <v>258</v>
       </c>
-      <c r="D39" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="E39" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="29" t="n">
-        <v>36</v>
-      </c>
-      <c r="B40" s="29" t="s">
-        <v>256</v>
-      </c>
-      <c r="C40" s="29" t="s">
+      <c r="D40" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="E40" s="27" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="27" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="27" t="s">
+        <v>255</v>
+      </c>
+      <c r="C41" s="27" t="s">
         <v>259</v>
       </c>
-      <c r="D40" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="E40" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="29" t="n">
-        <v>37</v>
-      </c>
-      <c r="B41" s="29" t="s">
-        <v>256</v>
-      </c>
-      <c r="C41" s="29" t="s">
+      <c r="D41" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="E41" s="27" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="27" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="27" t="s">
+        <v>255</v>
+      </c>
+      <c r="C42" s="27" t="s">
         <v>260</v>
       </c>
-      <c r="D41" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="E41" s="29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="29" t="n">
-        <v>38</v>
-      </c>
-      <c r="B42" s="29" t="s">
-        <v>256</v>
-      </c>
-      <c r="C42" s="29" t="s">
-        <v>261</v>
-      </c>
-      <c r="D42" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="E42" s="29" t="s">
-        <v>217</v>
+      <c r="D42" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="E42" s="27" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C44" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D44" s="2" t="n">
         <f aca="false">COUNTA(C5:C42)</f>
@@ -4005,9 +3952,9 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C45" s="5" t="s">
-        <v>263</v>
-      </c>
-      <c r="D45" s="30" t="n">
+        <v>262</v>
+      </c>
+      <c r="D45" s="28" t="n">
         <f aca="false">MAX(COUNTIF(B5:B42,"ID1*"),COUNTIF(B5:B42,"ID2*"),COUNTIF(B5:B42,"ID3*"),COUNTIF(B5:B42,"ID4*"),COUNTIF(B5:B42,"ID5*"),COUNTIF(B5:B42,"ID6*"))</f>
         <v>8</v>
       </c>
@@ -4036,101 +3983,101 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="26" t="s">
-        <v>264</v>
+      <c r="B1" s="24" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
+        <v>264</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>265</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B13" s="6" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="29" t="s">
         <v>276</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="31" t="s">
-        <v>277</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ajout d'une prise étanche par balcon + option prises connectées
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BjWSBdyxAjsRnCWBVUUVzr
</commit_message>
<xml_diff>
--- a/devis/Devis_electricite_T4_connecte_Legrand.xlsx
+++ b/devis/Devis_electricite_T4_connecte_Legrand.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="281">
   <si>
     <t xml:space="preserve">MAUREL'EC</t>
   </si>
@@ -495,6 +495,12 @@
     <t xml:space="preserve">Alimentation ventilateur + commande connectée (1 par balcon)</t>
   </si>
   <si>
+    <t xml:space="preserve">10.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prise de courant étanche Legrand Plexo IP55 (1 par balcon)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sous-total lot 10</t>
   </si>
   <si>
@@ -609,6 +615,12 @@
     <t xml:space="preserve">OPT.5</t>
   </si>
   <si>
+    <t xml:space="preserve">Plus-value : remplacement des 21 prises standard par des prises connectées Céliane with Netatmo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPT.6</t>
+  </si>
+  <si>
     <t xml:space="preserve">Délesteur / gestionnaire d'énergie (chauffage + climatisations)</t>
   </si>
   <si>
@@ -714,7 +726,7 @@
     <t xml:space="preserve">Prises SDB 1, SDB 2 (2)</t>
   </si>
   <si>
-    <t xml:space="preserve">Balcons : brumisateurs + ventilateurs</t>
+    <t xml:space="preserve">Balcons : prises, brumisateurs + ventilateurs</t>
   </si>
   <si>
     <t xml:space="preserve">Porte électrique WC</t>
@@ -846,7 +858,7 @@
     <t xml:space="preserve">PIÈCES : la cliente annonce 3 chambres, séjour, cuisine, buanderie, dressing, 2 SDB, WC. Les « SÉCH. » / « RANGT. » du plan sont supposés être la buanderie et le dressing.</t>
   </si>
   <si>
-    <t xml:space="preserve">PRISES : nombre minimum NF C 15-100 (séjour 7, chambres 3, cuisine 6, SDB 1, hall et dégagement 1). Dressing, buanderie et WC &lt; 4 m² : pas de prise imposée. Balcons : pas de prise.</t>
+    <t xml:space="preserve">PRISES : nombre minimum NF C 15-100 (séjour 7, chambres 3, cuisine 6, SDB 1, hall et dégagement 1). Dressing, buanderie et WC &lt; 4 m² : pas de prise imposée. Balcons : 1 prise étanche par balcon (demande client).</t>
   </si>
   <si>
     <t xml:space="preserve">Saignées : 160 ml murs + 70 ml sol estimés pour un immeuble béton – à recaler à la visite (ce poste pèse lourd dans le total).</t>
@@ -1448,7 +1460,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F128"/>
+  <dimension ref="A1:F130"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -2826,49 +2838,49 @@
         <v>480</v>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E90" s="15" t="s">
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A90" s="10" t="s">
         <v>156</v>
       </c>
-      <c r="F90" s="16" t="n">
-        <f aca="false">SUM(F86:F89)</f>
-        <v>1640</v>
-      </c>
-    </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="8" t="s">
+      <c r="B90" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="B92" s="9" t="s">
+      <c r="C90" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D90" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E90" s="13" t="n">
+        <v>125</v>
+      </c>
+      <c r="F90" s="14" t="n">
+        <f aca="false">D90*E90</f>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E91" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="C92" s="9"/>
-      <c r="D92" s="9"/>
-      <c r="E92" s="9"/>
-      <c r="F92" s="9"/>
-    </row>
-    <row r="93" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A93" s="10" t="s">
+      <c r="F91" s="16" t="n">
+        <f aca="false">SUM(F86:F90)</f>
+        <v>1890</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="B93" s="11" t="s">
+      <c r="B93" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="C93" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D93" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="E93" s="13" t="n">
-        <v>125</v>
-      </c>
-      <c r="F93" s="14" t="n">
-        <f aca="false">D93*E93</f>
-        <v>375</v>
-      </c>
-    </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C93" s="9"/>
+      <c r="D93" s="9"/>
+      <c r="E93" s="9"/>
+      <c r="F93" s="9"/>
+    </row>
+    <row r="94" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="10" t="s">
         <v>161</v>
       </c>
@@ -2879,14 +2891,14 @@
         <v>37</v>
       </c>
       <c r="D94" s="12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E94" s="13" t="n">
-        <v>270</v>
+        <v>125</v>
       </c>
       <c r="F94" s="14" t="n">
         <f aca="false">D94*E94</f>
-        <v>270</v>
+        <v>375</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2903,11 +2915,11 @@
         <v>1</v>
       </c>
       <c r="E95" s="13" t="n">
-        <v>150</v>
+        <v>270</v>
       </c>
       <c r="F95" s="14" t="n">
         <f aca="false">D95*E95</f>
-        <v>150</v>
+        <v>270</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2921,14 +2933,14 @@
         <v>37</v>
       </c>
       <c r="D96" s="12" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E96" s="13" t="n">
-        <v>58</v>
+        <v>150</v>
       </c>
       <c r="F96" s="14" t="n">
         <f aca="false">D96*E96</f>
-        <v>406</v>
+        <v>150</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2942,14 +2954,14 @@
         <v>37</v>
       </c>
       <c r="D97" s="12" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E97" s="13" t="n">
-        <v>145</v>
+        <v>58</v>
       </c>
       <c r="F97" s="14" t="n">
         <f aca="false">D97*E97</f>
-        <v>435</v>
+        <v>406</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2963,59 +2975,59 @@
         <v>37</v>
       </c>
       <c r="D98" s="12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E98" s="13" t="n">
-        <v>350</v>
+        <v>145</v>
       </c>
       <c r="F98" s="14" t="n">
         <f aca="false">D98*E98</f>
+        <v>435</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A99" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="B99" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="C99" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D99" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E99" s="13" t="n">
+        <v>350</v>
+      </c>
+      <c r="F99" s="14" t="n">
+        <f aca="false">D99*E99</f>
         <v>700</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E99" s="15" t="s">
-        <v>171</v>
-      </c>
-      <c r="F99" s="16" t="n">
-        <f aca="false">SUM(F93:F98)</f>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E100" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="F100" s="16" t="n">
+        <f aca="false">SUM(F94:F99)</f>
         <v>2336</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="8" t="s">
-        <v>172</v>
-      </c>
-      <c r="B101" s="9" t="s">
-        <v>173</v>
-      </c>
-      <c r="C101" s="9"/>
-      <c r="D101" s="9"/>
-      <c r="E101" s="9"/>
-      <c r="F101" s="9"/>
-    </row>
-    <row r="102" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A102" s="10" t="s">
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="B102" s="11" t="s">
+      <c r="B102" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="C102" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D102" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E102" s="13" t="n">
-        <v>480</v>
-      </c>
-      <c r="F102" s="14" t="n">
-        <f aca="false">D102*E102</f>
-        <v>480</v>
-      </c>
-    </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C102" s="9"/>
+      <c r="D102" s="9"/>
+      <c r="E102" s="9"/>
+      <c r="F102" s="9"/>
+    </row>
+    <row r="103" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="10" t="s">
         <v>176</v>
       </c>
@@ -3029,14 +3041,14 @@
         <v>1</v>
       </c>
       <c r="E103" s="13" t="n">
-        <v>280</v>
+        <v>480</v>
       </c>
       <c r="F103" s="14" t="n">
         <f aca="false">D103*E103</f>
-        <v>280</v>
-      </c>
-    </row>
-    <row r="104" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="10" t="s">
         <v>178</v>
       </c>
@@ -3050,72 +3062,72 @@
         <v>1</v>
       </c>
       <c r="E104" s="13" t="n">
-        <v>360</v>
+        <v>280</v>
       </c>
       <c r="F104" s="14" t="n">
         <f aca="false">D104*E104</f>
+        <v>280</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A105" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="B105" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="C105" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D105" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E105" s="13" t="n">
         <v>360</v>
       </c>
-    </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E105" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="F105" s="16" t="n">
-        <f aca="false">SUM(F102:F104)</f>
+      <c r="F105" s="14" t="n">
+        <f aca="false">D105*E105</f>
+        <v>360</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E106" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="F106" s="16" t="n">
+        <f aca="false">SUM(F103:F105)</f>
         <v>1120</v>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E107" s="17" t="s">
-        <v>181</v>
-      </c>
-      <c r="F107" s="18" t="n">
-        <f aca="false">F13+F21+F41+F49+F55+F61+F65+F69+F83+F90+F99+F105</f>
-        <v>38185</v>
-      </c>
-    </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E108" s="19" t="s">
-        <v>182</v>
+      <c r="E108" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="F108" s="18" t="n">
+        <f aca="false">F13+F21+F41+F49+F55+F61+F65+F69+F83+F91+F100+F106</f>
+        <v>38435</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E109" s="20" t="s">
-        <v>183</v>
-      </c>
-      <c r="F109" s="21" t="n">
-        <f aca="false">F107*0.3</f>
-        <v>11455.5</v>
-      </c>
-    </row>
-    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="22" t="s">
+      <c r="E109" s="19" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A113" s="10" t="s">
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E110" s="20" t="s">
         <v>185</v>
       </c>
-      <c r="B113" s="11" t="s">
+      <c r="F110" s="21" t="n">
+        <f aca="false">F108*0.3</f>
+        <v>11530.5</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="22" t="s">
         <v>186</v>
       </c>
-      <c r="C113" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D113" s="12" t="n">
-        <v>12</v>
-      </c>
-      <c r="E113" s="13" t="n">
-        <v>65</v>
-      </c>
-      <c r="F113" s="14" t="n">
-        <f aca="false">D113*E113</f>
-        <v>780</v>
-      </c>
-    </row>
-    <row r="114" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="10" t="s">
         <v>187</v>
       </c>
@@ -3126,17 +3138,17 @@
         <v>37</v>
       </c>
       <c r="D114" s="12" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E114" s="13" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="F114" s="14" t="n">
         <f aca="false">D114*E114</f>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="10" t="s">
         <v>189</v>
       </c>
@@ -3144,17 +3156,17 @@
         <v>190</v>
       </c>
       <c r="C115" s="10" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D115" s="12" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E115" s="13" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="F115" s="14" t="n">
         <f aca="false">D115*E115</f>
-        <v>390</v>
+        <v>600</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3165,17 +3177,17 @@
         <v>192</v>
       </c>
       <c r="C116" s="10" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D116" s="12" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E116" s="13" t="n">
-        <v>120</v>
+        <v>65</v>
       </c>
       <c r="F116" s="14" t="n">
         <f aca="false">D116*E116</f>
-        <v>120</v>
+        <v>390</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3192,55 +3204,97 @@
         <v>1</v>
       </c>
       <c r="E117" s="13" t="n">
-        <v>420</v>
+        <v>120</v>
       </c>
       <c r="F117" s="14" t="n">
         <f aca="false">D117*E117</f>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A118" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="B118" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="C118" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D118" s="12" t="n">
+        <v>21</v>
+      </c>
+      <c r="E118" s="13" t="n">
+        <v>77</v>
+      </c>
+      <c r="F118" s="14" t="n">
+        <f aca="false">D118*E118</f>
+        <v>1617</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A119" s="10" t="s">
+        <v>197</v>
+      </c>
+      <c r="B119" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="C119" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D119" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E119" s="13" t="n">
         <v>420</v>
       </c>
-    </row>
-    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E118" s="15" t="s">
-        <v>195</v>
-      </c>
-      <c r="F118" s="16" t="n">
-        <f aca="false">SUM(F113:F117)</f>
-        <v>2310</v>
-      </c>
-    </row>
-    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A121" s="2" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="122" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B122" s="23" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="123" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B123" s="23" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="124" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F119" s="14" t="n">
+        <f aca="false">D119*E119</f>
+        <v>420</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E120" s="15" t="s">
+        <v>199</v>
+      </c>
+      <c r="F120" s="16" t="n">
+        <f aca="false">SUM(F114:F119)</f>
+        <v>3927</v>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B124" s="23" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B125" s="23" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="126" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B126" s="23" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B128" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B127" s="23" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B128" s="23" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B130" s="2" t="s">
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -3270,12 +3324,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="24" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="25" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3283,16 +3337,16 @@
         <v>14</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="D4" s="26" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E4" s="26" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3300,16 +3354,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="D5" s="27" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E5" s="27" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3317,16 +3371,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="27" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="D6" s="27" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E6" s="27" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3334,16 +3388,16 @@
         <v>3</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="D7" s="27" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="E7" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3351,16 +3405,16 @@
         <v>4</v>
       </c>
       <c r="B8" s="27" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="D8" s="27" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E8" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3368,16 +3422,16 @@
         <v>5</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="D9" s="27" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3385,16 +3439,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="27" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="D10" s="27" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E10" s="27" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3402,16 +3456,16 @@
         <v>7</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E11" s="27" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3419,16 +3473,16 @@
         <v>8</v>
       </c>
       <c r="B12" s="27" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="D12" s="27" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="E12" s="27" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3436,16 +3490,16 @@
         <v>9</v>
       </c>
       <c r="B13" s="27" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E13" s="27" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3453,16 +3507,16 @@
         <v>10</v>
       </c>
       <c r="B14" s="27" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="D14" s="27" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E14" s="27" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3470,16 +3524,16 @@
         <v>11</v>
       </c>
       <c r="B15" s="27" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="D15" s="27" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E15" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3487,16 +3541,16 @@
         <v>12</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="C16" s="27" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3504,16 +3558,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="C17" s="27" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3521,16 +3575,16 @@
         <v>14</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="D18" s="27" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3538,16 +3592,16 @@
         <v>15</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="C19" s="27" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3555,16 +3609,16 @@
         <v>16</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="C20" s="27" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="D20" s="27" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3572,16 +3626,16 @@
         <v>17</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C21" s="27" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="D21" s="27" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3589,16 +3643,16 @@
         <v>18</v>
       </c>
       <c r="B22" s="27" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="D22" s="27" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="E22" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3606,16 +3660,16 @@
         <v>19</v>
       </c>
       <c r="B23" s="27" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C23" s="27" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="D23" s="27" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="E23" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3623,16 +3677,16 @@
         <v>20</v>
       </c>
       <c r="B24" s="27" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C24" s="27" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="D24" s="27" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="E24" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3640,16 +3694,16 @@
         <v>21</v>
       </c>
       <c r="B25" s="27" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="D25" s="27" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="E25" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3657,16 +3711,16 @@
         <v>22</v>
       </c>
       <c r="B26" s="27" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C26" s="27" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="D26" s="27" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E26" s="27" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3674,16 +3728,16 @@
         <v>23</v>
       </c>
       <c r="B27" s="27" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="D27" s="27" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="E27" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3691,16 +3745,16 @@
         <v>24</v>
       </c>
       <c r="B28" s="27" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="C28" s="27" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="D28" s="27" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="E28" s="27" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3708,16 +3762,16 @@
         <v>25</v>
       </c>
       <c r="B29" s="27" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="C29" s="27" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="D29" s="27" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="E29" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3725,16 +3779,16 @@
         <v>26</v>
       </c>
       <c r="B30" s="27" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="C30" s="27" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="D30" s="27" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="E30" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3742,16 +3796,16 @@
         <v>27</v>
       </c>
       <c r="B31" s="27" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="D31" s="27" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="E31" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3759,16 +3813,16 @@
         <v>28</v>
       </c>
       <c r="B32" s="27" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="C32" s="27" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="D32" s="27" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="E32" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3776,16 +3830,16 @@
         <v>29</v>
       </c>
       <c r="B33" s="27" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="C33" s="27" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="D33" s="27" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="E33" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3793,16 +3847,16 @@
         <v>30</v>
       </c>
       <c r="B34" s="27" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="C34" s="27" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="D34" s="27" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E34" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3810,16 +3864,16 @@
         <v>31</v>
       </c>
       <c r="B35" s="27" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="C35" s="27" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="D35" s="27" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E35" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3827,16 +3881,16 @@
         <v>32</v>
       </c>
       <c r="B36" s="27" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="C36" s="27" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="D36" s="27" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E36" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3844,16 +3898,16 @@
         <v>33</v>
       </c>
       <c r="B37" s="27" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="C37" s="27" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="D37" s="27" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E37" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3861,16 +3915,16 @@
         <v>34</v>
       </c>
       <c r="B38" s="27" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C38" s="27" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="D38" s="27" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E38" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3878,16 +3932,16 @@
         <v>35</v>
       </c>
       <c r="B39" s="27" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C39" s="27" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="D39" s="27" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E39" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3895,16 +3949,16 @@
         <v>36</v>
       </c>
       <c r="B40" s="27" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C40" s="27" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="D40" s="27" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E40" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3912,16 +3966,16 @@
         <v>37</v>
       </c>
       <c r="B41" s="27" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C41" s="27" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="D41" s="27" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E41" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3929,21 +3983,21 @@
         <v>38</v>
       </c>
       <c r="B42" s="27" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C42" s="27" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="D42" s="27" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E42" s="27" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C44" s="2" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="D44" s="2" t="n">
         <f aca="false">COUNTA(C5:C42)</f>
@@ -3952,7 +4006,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C45" s="5" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="D45" s="28" t="n">
         <f aca="false">MAX(COUNTIF(B5:B42,"ID1*"),COUNTIF(B5:B42,"ID2*"),COUNTIF(B5:B42,"ID3*"),COUNTIF(B5:B42,"ID4*"),COUNTIF(B5:B42,"ID5*"),COUNTIF(B5:B42,"ID6*"))</f>
@@ -3984,100 +4038,100 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="24" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="29" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ajout onglet références Legrand/Netatmo à chiffrer chez le fournisseur
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BjWSBdyxAjsRnCWBVUUVzr
</commit_message>
<xml_diff>
--- a/devis/Devis_electricite_T4_connecte_Legrand.xlsx
+++ b/devis/Devis_electricite_T4_connecte_Legrand.xlsx
@@ -9,8 +9,9 @@
   </bookViews>
   <sheets>
     <sheet name="Devis" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Tableau électrique" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Points à vérifier" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Références fournisseur" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Tableau électrique" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Points à vérifier" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">Devis!$9:$9</definedName>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="362">
   <si>
     <t xml:space="preserve">MAUREL'EC</t>
   </si>
@@ -646,6 +647,249 @@
   </si>
   <si>
     <t xml:space="preserve">Bon pour accord – Date et signature de la cliente :</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Références Legrand / Netatmo à chiffrer chez le fournisseur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saisir ton prix d'achat HT en colonne F (cellules jaunes). « Vérifié » = référence lue sur legrand.fr (oct. 2026) ; « À confirmer » = à valider avec le fournisseur (gamme en cours de renouvellement). Tarif public = indicatif.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Désignation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réf. Legrand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usage dans le devis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarif public HT (info)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ton prix achat HT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total achat HT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PASSERELLE ET TABLEAU CONNECTÉ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pack de démarrage Drivia with Netatmo : module Control + contacteur connecté</t>
+  </si>
+  <si>
+    <t xml:space="preserve">412191B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Passerelle de toute l'installation (au tableau) + pilotage du cumulus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vérifié</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Module de mesure de consommation connecté Drivia with Netatmo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">412015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suivi des consommations au tableau</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À confirmer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(Alternative) Pack de démarrage Céliane with Netatmo : prise Control + commande Départ/Arrivée, blanc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CB0443</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seulement si on ne prend pas la passerelle Drivia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ÉCLAIRAGE ET COMMANDES CONNECTÉES CÉLIANE WITH NETATMO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interrupteur filaire connecté avec neutre, option variation, avec support et enjoliveur blanc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CB0409</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Éclairage pièces (14), balcons (2), variateur bibliothèque (1), brumisateurs + ventilateurs (4), filtre à air (1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commande sans fils Self-e (sans pile) éclairage et prises, avec support et enjoliveur blanc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CB0420</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Va-et-vient : têtes de lit (3), séjour (1), dégagement (1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commande générale sans fils Départ/Arrivée, avec support et enjoliveur blanc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CB0400</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrée (version noire CN0400 vérifiée)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commande Lever/Coucher Self-e sans fils, sans pile, avec support et enjoliveur blanc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CB0423</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chambre parentale (remplacée par 064884L à épuisement)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VOLETS ROULANTS ET STORES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interrupteur connecté pour volets roulants et stores, avec support et enjoliveur blanc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CB0431</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 volets + 2 stores (moteurs filaires obligatoires)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commande sans fils pour volets roulants, avec support et enjoliveur blanc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CB0432</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commande générale des volets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRISES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prise connectée 16 A Céliane with Netatmo avec support et enjoliveur blanc (mesure conso)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CB0460</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Séjour (2), chambres (3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prise 2P+T Céliane bornes automatiques (mécanisme)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CM0111</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prises standard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enjoliveur prise 2P+T Surface Confort Céliane blanc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CB0111</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Support Céliane 1 poste (pour mécanismes CM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">à confirmer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prises standard + RJ45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prise RJ45 Céliane cat. 6A STP grade 3TV (mécanisme)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CM0346</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enjoliveur RJ45 grade 3TV Céliane blanc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CB0346</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prise 2P+T Plexo étanche IP55 gris à composer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">069551L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Balcons</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boîtier saillie Plexo 1 poste (ou support encastré 069681L)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">069651L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plaque de finition Céliane 1 poste (finition au choix de la cliente)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">selon finition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≈ 1 par appareil (69) – à regrouper en multipostes selon implantation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SÉCURITÉ NETATMO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Détecteur de fumée intelligent Netatmo (pile 10 ans)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NSA-PRO-FR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hall, dégagement, séjour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caméra intérieure intelligente Netatmo (centrale de l'alarme)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NSC-PRO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hall d'entrée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sirène intérieure intelligente Netatmo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NIS01-PRO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hall</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Détecteur d'ouverture intelligent Netatmo (porte / fenêtre)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DTG-PRO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Porte d'entrée + 6 baies (vérifier si vendu par lot)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caméra extérieure intelligente Netatmo (NOC-S-PRO = avec sirène)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOC-PRO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tableau électrique (coffret Drivia 4 rangées, GTL 13 modules, 6 interrupteurs différentiels, 38 disjoncteurs DX3, parafoudre, contacteur jour/nuit, tableau de communication grade 3TV) : à chiffrer par le fournisseur sur la liste de l'onglet « Tableau électrique ».</t>
   </si>
   <si>
     <t xml:space="preserve">Répartition prévisionnelle des circuits – coffret Drivia 4 rangées (hall d'entrée)</t>
@@ -879,7 +1123,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.00&quot; €&quot;;\-#,##0.00&quot; €&quot;;\-"/>
     <numFmt numFmtId="166" formatCode="General"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -989,7 +1233,7 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="12"/>
+      <sz val="13"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -1006,13 +1250,37 @@
     <font>
       <b val="true"/>
       <sz val="9"/>
+      <color rgb="FF1E8E3E"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="9"/>
+      <color rgb="FFC00000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="9"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1035,6 +1303,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFC00000"/>
         <bgColor rgb="FF800000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -1087,7 +1361,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="38">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1188,6 +1462,38 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1204,7 +1510,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1268,7 +1574,7 @@
       <rgbColor rgb="FF666699"/>
       <rgbColor rgb="FF999999"/>
       <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF1E8E3E"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF444444"/>
       <rgbColor rgb="FF993300"/>
@@ -3313,707 +3619,690 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="24" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="25" t="s">
         <v>208</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+    </row>
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="26" t="s">
-        <v>14</v>
+        <v>209</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D4" s="26" t="s">
-        <v>211</v>
+        <v>17</v>
       </c>
       <c r="E4" s="26" t="s">
         <v>212</v>
       </c>
+      <c r="F4" s="26" t="s">
+        <v>213</v>
+      </c>
+      <c r="G4" s="26" t="s">
+        <v>214</v>
+      </c>
+      <c r="H4" s="26" t="s">
+        <v>215</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="27" t="n">
+      <c r="A5" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+    </row>
+    <row r="6" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B6" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="D6" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="27" t="s">
-        <v>213</v>
-      </c>
-      <c r="C5" s="27" t="s">
+      <c r="E6" s="28" t="n">
+        <v>297.2</v>
+      </c>
+      <c r="F6" s="29"/>
+      <c r="G6" s="28" t="n">
+        <f aca="false">D6*F6</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="30" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11" t="s">
+        <v>221</v>
+      </c>
+      <c r="B7" s="27" t="s">
+        <v>222</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>223</v>
+      </c>
+      <c r="D7" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="28"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="28" t="n">
+        <f aca="false">D7*F7</f>
+        <v>0</v>
+      </c>
+      <c r="H7" s="31" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
+        <v>225</v>
+      </c>
+      <c r="B8" s="27" t="s">
+        <v>226</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>227</v>
+      </c>
+      <c r="D8" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="28" t="n">
+        <v>144.1</v>
+      </c>
+      <c r="F8" s="29"/>
+      <c r="G8" s="28" t="n">
+        <f aca="false">D8*F8</f>
+        <v>0</v>
+      </c>
+      <c r="H8" s="30" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+    </row>
+    <row r="10" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="B10" s="27" t="s">
+        <v>230</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="D10" s="12" t="n">
+        <v>22</v>
+      </c>
+      <c r="E10" s="28"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="28" t="n">
+        <f aca="false">D10*F10</f>
+        <v>0</v>
+      </c>
+      <c r="H10" s="30" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="B11" s="27" t="s">
+        <v>233</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="D11" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" s="28"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="28" t="n">
+        <f aca="false">D11*F11</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="31" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="B12" s="27" t="s">
+        <v>236</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="D12" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="28"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="28" t="n">
+        <f aca="false">D12*F12</f>
+        <v>0</v>
+      </c>
+      <c r="H12" s="31" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="B13" s="27" t="s">
+        <v>239</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="D13" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="28" t="n">
+        <v>91.24</v>
+      </c>
+      <c r="F13" s="29"/>
+      <c r="G13" s="28" t="n">
+        <f aca="false">D13*F13</f>
+        <v>0</v>
+      </c>
+      <c r="H13" s="30" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+    </row>
+    <row r="15" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="11" t="s">
+        <v>242</v>
+      </c>
+      <c r="B15" s="27" t="s">
+        <v>243</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>244</v>
+      </c>
+      <c r="D15" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="E15" s="28"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="28" t="n">
+        <f aca="false">D15*F15</f>
+        <v>0</v>
+      </c>
+      <c r="H15" s="30" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="11" t="s">
+        <v>245</v>
+      </c>
+      <c r="B16" s="27" t="s">
+        <v>246</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>247</v>
+      </c>
+      <c r="D16" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="28"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="28" t="n">
+        <f aca="false">D16*F16</f>
+        <v>0</v>
+      </c>
+      <c r="H16" s="30" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="9" t="s">
+        <v>248</v>
+      </c>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+    </row>
+    <row r="18" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="B18" s="27" t="s">
+        <v>250</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="D18" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E18" s="28" t="n">
+        <v>76.8</v>
+      </c>
+      <c r="F18" s="29"/>
+      <c r="G18" s="28" t="n">
+        <f aca="false">D18*F18</f>
+        <v>0</v>
+      </c>
+      <c r="H18" s="30" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="11" t="s">
+        <v>252</v>
+      </c>
+      <c r="B19" s="27" t="s">
+        <v>253</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>254</v>
+      </c>
+      <c r="D19" s="12" t="n">
+        <v>21</v>
+      </c>
+      <c r="E19" s="28"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="28" t="n">
+        <f aca="false">D19*F19</f>
+        <v>0</v>
+      </c>
+      <c r="H19" s="31" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="11" t="s">
+        <v>255</v>
+      </c>
+      <c r="B20" s="27" t="s">
+        <v>256</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>254</v>
+      </c>
+      <c r="D20" s="12" t="n">
+        <v>21</v>
+      </c>
+      <c r="E20" s="28"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="28" t="n">
+        <f aca="false">D20*F20</f>
+        <v>0</v>
+      </c>
+      <c r="H20" s="30" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="11" t="s">
+        <v>257</v>
+      </c>
+      <c r="B21" s="27" t="s">
+        <v>258</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>259</v>
+      </c>
+      <c r="D21" s="12" t="n">
+        <v>26</v>
+      </c>
+      <c r="E21" s="28"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="28" t="n">
+        <f aca="false">D21*F21</f>
+        <v>0</v>
+      </c>
+      <c r="H21" s="31" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="11" t="s">
+        <v>260</v>
+      </c>
+      <c r="B22" s="27" t="s">
+        <v>261</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="D22" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E22" s="28" t="n">
+        <v>24.51</v>
+      </c>
+      <c r="F22" s="29"/>
+      <c r="G22" s="28" t="n">
+        <f aca="false">D22*F22</f>
+        <v>0</v>
+      </c>
+      <c r="H22" s="30" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11" t="s">
+        <v>262</v>
+      </c>
+      <c r="B23" s="27" t="s">
+        <v>263</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="D23" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E23" s="28" t="n">
+        <v>4.76</v>
+      </c>
+      <c r="F23" s="29"/>
+      <c r="G23" s="28" t="n">
+        <f aca="false">D23*F23</f>
+        <v>0</v>
+      </c>
+      <c r="H23" s="30" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="B24" s="27" t="s">
+        <v>265</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>266</v>
+      </c>
+      <c r="D24" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" s="28"/>
+      <c r="F24" s="29"/>
+      <c r="G24" s="28" t="n">
+        <f aca="false">D24*F24</f>
+        <v>0</v>
+      </c>
+      <c r="H24" s="31" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="B25" s="27" t="s">
+        <v>268</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>266</v>
+      </c>
+      <c r="D25" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" s="28"/>
+      <c r="F25" s="29"/>
+      <c r="G25" s="28" t="n">
+        <f aca="false">D25*F25</f>
+        <v>0</v>
+      </c>
+      <c r="H25" s="31" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="11" t="s">
+        <v>269</v>
+      </c>
+      <c r="B26" s="27" t="s">
+        <v>270</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>271</v>
+      </c>
+      <c r="D26" s="12" t="n">
+        <v>69</v>
+      </c>
+      <c r="E26" s="28"/>
+      <c r="F26" s="29"/>
+      <c r="G26" s="28" t="n">
+        <f aca="false">D26*F26</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="31" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="9" t="s">
+        <v>272</v>
+      </c>
+      <c r="B27" s="9"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+    </row>
+    <row r="28" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="11" t="s">
+        <v>273</v>
+      </c>
+      <c r="B28" s="27" t="s">
+        <v>274</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="D28" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E28" s="28" t="n">
+        <v>161.5</v>
+      </c>
+      <c r="F28" s="29"/>
+      <c r="G28" s="28" t="n">
+        <f aca="false">D28*F28</f>
+        <v>0</v>
+      </c>
+      <c r="H28" s="30" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="B29" s="27" t="s">
+        <v>277</v>
+      </c>
+      <c r="C29" s="11" t="s">
+        <v>278</v>
+      </c>
+      <c r="D29" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="28"/>
+      <c r="F29" s="29"/>
+      <c r="G29" s="28" t="n">
+        <f aca="false">D29*F29</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="31" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="11" t="s">
+        <v>279</v>
+      </c>
+      <c r="B30" s="27" t="s">
+        <v>280</v>
+      </c>
+      <c r="C30" s="11" t="s">
+        <v>281</v>
+      </c>
+      <c r="D30" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="28"/>
+      <c r="F30" s="29"/>
+      <c r="G30" s="28" t="n">
+        <f aca="false">D30*F30</f>
+        <v>0</v>
+      </c>
+      <c r="H30" s="31" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="11" t="s">
+        <v>282</v>
+      </c>
+      <c r="B31" s="27" t="s">
+        <v>283</v>
+      </c>
+      <c r="C31" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="D31" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="E31" s="28"/>
+      <c r="F31" s="29"/>
+      <c r="G31" s="28" t="n">
+        <f aca="false">D31*F31</f>
+        <v>0</v>
+      </c>
+      <c r="H31" s="31" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="B32" s="27" t="s">
+        <v>286</v>
+      </c>
+      <c r="C32" s="11" t="s">
+        <v>266</v>
+      </c>
+      <c r="D32" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" s="28"/>
+      <c r="F32" s="29"/>
+      <c r="G32" s="28" t="n">
+        <f aca="false">D32*F32</f>
+        <v>0</v>
+      </c>
+      <c r="H32" s="31" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F34" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="D5" s="27" t="s">
-        <v>215</v>
-      </c>
-      <c r="E5" s="27" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="27" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="27" t="s">
-        <v>213</v>
-      </c>
-      <c r="C6" s="27" t="s">
-        <v>217</v>
-      </c>
-      <c r="D6" s="27" t="s">
-        <v>215</v>
-      </c>
-      <c r="E6" s="27" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="27" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="27" t="s">
-        <v>213</v>
-      </c>
-      <c r="C7" s="27" t="s">
-        <v>218</v>
-      </c>
-      <c r="D7" s="27" t="s">
-        <v>219</v>
-      </c>
-      <c r="E7" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="27" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="27" t="s">
-        <v>213</v>
-      </c>
-      <c r="C8" s="27" t="s">
-        <v>221</v>
-      </c>
-      <c r="D8" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="E8" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="27" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="27" t="s">
-        <v>213</v>
-      </c>
-      <c r="C9" s="27" t="s">
-        <v>223</v>
-      </c>
-      <c r="D9" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="E9" s="27" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="27" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="27" t="s">
-        <v>213</v>
-      </c>
-      <c r="C10" s="27" t="s">
-        <v>224</v>
-      </c>
-      <c r="D10" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="E10" s="27" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="27" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="27" t="s">
-        <v>213</v>
-      </c>
-      <c r="C11" s="27" t="s">
-        <v>225</v>
-      </c>
-      <c r="D11" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="E11" s="27" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="27" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="27" t="s">
-        <v>213</v>
-      </c>
-      <c r="C12" s="27" t="s">
-        <v>226</v>
-      </c>
-      <c r="D12" s="27" t="s">
-        <v>227</v>
-      </c>
-      <c r="E12" s="27" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="27" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="27" t="s">
-        <v>228</v>
-      </c>
-      <c r="C13" s="27" t="s">
-        <v>229</v>
-      </c>
-      <c r="D13" s="27" t="s">
-        <v>215</v>
-      </c>
-      <c r="E13" s="27" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="27" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="27" t="s">
-        <v>228</v>
-      </c>
-      <c r="C14" s="27" t="s">
-        <v>230</v>
-      </c>
-      <c r="D14" s="27" t="s">
-        <v>215</v>
-      </c>
-      <c r="E14" s="27" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="27" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="27" t="s">
-        <v>228</v>
-      </c>
-      <c r="C15" s="27" t="s">
-        <v>231</v>
-      </c>
-      <c r="D15" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="E15" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="27" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="27" t="s">
-        <v>228</v>
-      </c>
-      <c r="C16" s="27" t="s">
-        <v>232</v>
-      </c>
-      <c r="D16" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="E16" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="27" t="n">
-        <v>13</v>
-      </c>
-      <c r="B17" s="27" t="s">
-        <v>228</v>
-      </c>
-      <c r="C17" s="27" t="s">
-        <v>233</v>
-      </c>
-      <c r="D17" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="E17" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="27" t="n">
-        <v>14</v>
-      </c>
-      <c r="B18" s="27" t="s">
-        <v>228</v>
-      </c>
-      <c r="C18" s="27" t="s">
-        <v>234</v>
-      </c>
-      <c r="D18" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="E18" s="27" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="27" t="n">
-        <v>15</v>
-      </c>
-      <c r="B19" s="27" t="s">
-        <v>228</v>
-      </c>
-      <c r="C19" s="27" t="s">
-        <v>235</v>
-      </c>
-      <c r="D19" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="E19" s="27" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="27" t="n">
-        <v>16</v>
-      </c>
-      <c r="B20" s="27" t="s">
-        <v>228</v>
-      </c>
-      <c r="C20" s="27" t="s">
-        <v>236</v>
-      </c>
-      <c r="D20" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="E20" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="27" t="n">
-        <v>17</v>
-      </c>
-      <c r="B21" s="27" t="s">
-        <v>237</v>
-      </c>
-      <c r="C21" s="27" t="s">
-        <v>238</v>
-      </c>
-      <c r="D21" s="27" t="s">
-        <v>219</v>
-      </c>
-      <c r="E21" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="27" t="n">
-        <v>18</v>
-      </c>
-      <c r="B22" s="27" t="s">
-        <v>237</v>
-      </c>
-      <c r="C22" s="27" t="s">
-        <v>239</v>
-      </c>
-      <c r="D22" s="27" t="s">
-        <v>219</v>
-      </c>
-      <c r="E22" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="27" t="n">
-        <v>19</v>
-      </c>
-      <c r="B23" s="27" t="s">
-        <v>237</v>
-      </c>
-      <c r="C23" s="27" t="s">
-        <v>240</v>
-      </c>
-      <c r="D23" s="27" t="s">
-        <v>219</v>
-      </c>
-      <c r="E23" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="27" t="n">
-        <v>20</v>
-      </c>
-      <c r="B24" s="27" t="s">
-        <v>237</v>
-      </c>
-      <c r="C24" s="27" t="s">
-        <v>241</v>
-      </c>
-      <c r="D24" s="27" t="s">
-        <v>219</v>
-      </c>
-      <c r="E24" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="27" t="n">
-        <v>21</v>
-      </c>
-      <c r="B25" s="27" t="s">
-        <v>237</v>
-      </c>
-      <c r="C25" s="27" t="s">
-        <v>242</v>
-      </c>
-      <c r="D25" s="27" t="s">
-        <v>219</v>
-      </c>
-      <c r="E25" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="27" t="n">
-        <v>22</v>
-      </c>
-      <c r="B26" s="27" t="s">
-        <v>237</v>
-      </c>
-      <c r="C26" s="27" t="s">
-        <v>243</v>
-      </c>
-      <c r="D26" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="E26" s="27" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="27" t="n">
-        <v>23</v>
-      </c>
-      <c r="B27" s="27" t="s">
-        <v>237</v>
-      </c>
-      <c r="C27" s="27" t="s">
-        <v>244</v>
-      </c>
-      <c r="D27" s="27" t="s">
-        <v>219</v>
-      </c>
-      <c r="E27" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="27" t="n">
-        <v>24</v>
-      </c>
-      <c r="B28" s="27" t="s">
-        <v>245</v>
-      </c>
-      <c r="C28" s="27" t="s">
-        <v>246</v>
-      </c>
-      <c r="D28" s="27" t="s">
-        <v>247</v>
-      </c>
-      <c r="E28" s="27" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="27" t="n">
-        <v>25</v>
-      </c>
-      <c r="B29" s="27" t="s">
-        <v>245</v>
-      </c>
-      <c r="C29" s="27" t="s">
-        <v>249</v>
-      </c>
-      <c r="D29" s="27" t="s">
-        <v>219</v>
-      </c>
-      <c r="E29" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="27" t="n">
-        <v>26</v>
-      </c>
-      <c r="B30" s="27" t="s">
-        <v>245</v>
-      </c>
-      <c r="C30" s="27" t="s">
-        <v>250</v>
-      </c>
-      <c r="D30" s="27" t="s">
-        <v>219</v>
-      </c>
-      <c r="E30" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="27" t="n">
-        <v>27</v>
-      </c>
-      <c r="B31" s="27" t="s">
-        <v>245</v>
-      </c>
-      <c r="C31" s="27" t="s">
-        <v>251</v>
-      </c>
-      <c r="D31" s="27" t="s">
-        <v>219</v>
-      </c>
-      <c r="E31" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="27" t="n">
-        <v>28</v>
-      </c>
-      <c r="B32" s="27" t="s">
-        <v>245</v>
-      </c>
-      <c r="C32" s="27" t="s">
-        <v>252</v>
-      </c>
-      <c r="D32" s="27" t="s">
-        <v>219</v>
-      </c>
-      <c r="E32" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="27" t="n">
-        <v>29</v>
-      </c>
-      <c r="B33" s="27" t="s">
-        <v>245</v>
-      </c>
-      <c r="C33" s="27" t="s">
-        <v>253</v>
-      </c>
-      <c r="D33" s="27" t="s">
-        <v>219</v>
-      </c>
-      <c r="E33" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="27" t="n">
-        <v>30</v>
-      </c>
-      <c r="B34" s="27" t="s">
-        <v>254</v>
-      </c>
-      <c r="C34" s="27" t="s">
-        <v>255</v>
-      </c>
-      <c r="D34" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="E34" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="27" t="n">
-        <v>31</v>
-      </c>
-      <c r="B35" s="27" t="s">
-        <v>254</v>
-      </c>
-      <c r="C35" s="27" t="s">
-        <v>256</v>
-      </c>
-      <c r="D35" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="E35" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="27" t="n">
-        <v>32</v>
-      </c>
-      <c r="B36" s="27" t="s">
-        <v>254</v>
-      </c>
-      <c r="C36" s="27" t="s">
-        <v>257</v>
-      </c>
-      <c r="D36" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="E36" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="27" t="n">
-        <v>33</v>
-      </c>
-      <c r="B37" s="27" t="s">
-        <v>254</v>
-      </c>
-      <c r="C37" s="27" t="s">
-        <v>258</v>
-      </c>
-      <c r="D37" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="E37" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="27" t="n">
-        <v>34</v>
-      </c>
-      <c r="B38" s="27" t="s">
-        <v>259</v>
-      </c>
-      <c r="C38" s="27" t="s">
-        <v>260</v>
-      </c>
-      <c r="D38" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="E38" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="27" t="n">
-        <v>35</v>
-      </c>
-      <c r="B39" s="27" t="s">
-        <v>259</v>
-      </c>
-      <c r="C39" s="27" t="s">
-        <v>261</v>
-      </c>
-      <c r="D39" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="E39" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="27" t="n">
-        <v>36</v>
-      </c>
-      <c r="B40" s="27" t="s">
-        <v>259</v>
-      </c>
-      <c r="C40" s="27" t="s">
-        <v>262</v>
-      </c>
-      <c r="D40" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="E40" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="27" t="n">
-        <v>37</v>
-      </c>
-      <c r="B41" s="27" t="s">
-        <v>259</v>
-      </c>
-      <c r="C41" s="27" t="s">
-        <v>263</v>
-      </c>
-      <c r="D41" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="E41" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="27" t="n">
-        <v>38</v>
-      </c>
-      <c r="B42" s="27" t="s">
-        <v>259</v>
-      </c>
-      <c r="C42" s="27" t="s">
-        <v>264</v>
-      </c>
-      <c r="D42" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="E42" s="27" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C44" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="D44" s="2" t="n">
-        <f aca="false">COUNTA(C5:C42)</f>
-        <v>38</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C45" s="5" t="s">
-        <v>266</v>
-      </c>
-      <c r="D45" s="28" t="n">
-        <f aca="false">MAX(COUNTIF(B5:B42,"ID1*"),COUNTIF(B5:B42,"ID2*"),COUNTIF(B5:B42,"ID3*"),COUNTIF(B5:B42,"ID4*"),COUNTIF(B5:B42,"ID5*"),COUNTIF(B5:B42,"ID6*"))</f>
-        <v>8</v>
-      </c>
+      <c r="G34" s="16" t="n">
+        <f aca="false">SUM(G5:G32)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="25" t="s">
+        <v>287</v>
+      </c>
+      <c r="B36" s="25"/>
+      <c r="C36" s="25"/>
+      <c r="D36" s="25"/>
+      <c r="E36" s="25"/>
+      <c r="F36" s="25"/>
+      <c r="G36" s="25"/>
+      <c r="H36" s="25"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A36:H36"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -4029,6 +4318,722 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:E45"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="32" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="33" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="34" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="34" t="s">
+        <v>290</v>
+      </c>
+      <c r="C4" s="34" t="s">
+        <v>291</v>
+      </c>
+      <c r="D4" s="34" t="s">
+        <v>292</v>
+      </c>
+      <c r="E4" s="34" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="35" t="s">
+        <v>294</v>
+      </c>
+      <c r="C5" s="35" t="s">
+        <v>295</v>
+      </c>
+      <c r="D5" s="35" t="s">
+        <v>296</v>
+      </c>
+      <c r="E5" s="35" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="35" t="s">
+        <v>294</v>
+      </c>
+      <c r="C6" s="35" t="s">
+        <v>298</v>
+      </c>
+      <c r="D6" s="35" t="s">
+        <v>296</v>
+      </c>
+      <c r="E6" s="35" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="35" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="35" t="s">
+        <v>294</v>
+      </c>
+      <c r="C7" s="35" t="s">
+        <v>299</v>
+      </c>
+      <c r="D7" s="35" t="s">
+        <v>300</v>
+      </c>
+      <c r="E7" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="35" t="s">
+        <v>294</v>
+      </c>
+      <c r="C8" s="35" t="s">
+        <v>302</v>
+      </c>
+      <c r="D8" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="E8" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="35" t="s">
+        <v>294</v>
+      </c>
+      <c r="C9" s="35" t="s">
+        <v>304</v>
+      </c>
+      <c r="D9" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="E9" s="35" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="35" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="35" t="s">
+        <v>294</v>
+      </c>
+      <c r="C10" s="35" t="s">
+        <v>305</v>
+      </c>
+      <c r="D10" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="E10" s="35" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="35" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="35" t="s">
+        <v>294</v>
+      </c>
+      <c r="C11" s="35" t="s">
+        <v>306</v>
+      </c>
+      <c r="D11" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="E11" s="35" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="35" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="35" t="s">
+        <v>294</v>
+      </c>
+      <c r="C12" s="35" t="s">
+        <v>307</v>
+      </c>
+      <c r="D12" s="35" t="s">
+        <v>308</v>
+      </c>
+      <c r="E12" s="35" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="35" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="35" t="s">
+        <v>309</v>
+      </c>
+      <c r="C13" s="35" t="s">
+        <v>310</v>
+      </c>
+      <c r="D13" s="35" t="s">
+        <v>296</v>
+      </c>
+      <c r="E13" s="35" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="35" t="s">
+        <v>309</v>
+      </c>
+      <c r="C14" s="35" t="s">
+        <v>311</v>
+      </c>
+      <c r="D14" s="35" t="s">
+        <v>296</v>
+      </c>
+      <c r="E14" s="35" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="35" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="35" t="s">
+        <v>309</v>
+      </c>
+      <c r="C15" s="35" t="s">
+        <v>312</v>
+      </c>
+      <c r="D15" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="E15" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="35" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="35" t="s">
+        <v>309</v>
+      </c>
+      <c r="C16" s="35" t="s">
+        <v>313</v>
+      </c>
+      <c r="D16" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="E16" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="35" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="35" t="s">
+        <v>309</v>
+      </c>
+      <c r="C17" s="35" t="s">
+        <v>314</v>
+      </c>
+      <c r="D17" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="E17" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="35" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="35" t="s">
+        <v>309</v>
+      </c>
+      <c r="C18" s="35" t="s">
+        <v>315</v>
+      </c>
+      <c r="D18" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="E18" s="35" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="35" t="s">
+        <v>309</v>
+      </c>
+      <c r="C19" s="35" t="s">
+        <v>316</v>
+      </c>
+      <c r="D19" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="E19" s="35" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="35" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="35" t="s">
+        <v>309</v>
+      </c>
+      <c r="C20" s="35" t="s">
+        <v>317</v>
+      </c>
+      <c r="D20" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="E20" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="35" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="35" t="s">
+        <v>318</v>
+      </c>
+      <c r="C21" s="35" t="s">
+        <v>319</v>
+      </c>
+      <c r="D21" s="35" t="s">
+        <v>300</v>
+      </c>
+      <c r="E21" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="35" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="35" t="s">
+        <v>318</v>
+      </c>
+      <c r="C22" s="35" t="s">
+        <v>320</v>
+      </c>
+      <c r="D22" s="35" t="s">
+        <v>300</v>
+      </c>
+      <c r="E22" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="35" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="35" t="s">
+        <v>318</v>
+      </c>
+      <c r="C23" s="35" t="s">
+        <v>321</v>
+      </c>
+      <c r="D23" s="35" t="s">
+        <v>300</v>
+      </c>
+      <c r="E23" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="35" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="35" t="s">
+        <v>318</v>
+      </c>
+      <c r="C24" s="35" t="s">
+        <v>322</v>
+      </c>
+      <c r="D24" s="35" t="s">
+        <v>300</v>
+      </c>
+      <c r="E24" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="35" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="35" t="s">
+        <v>318</v>
+      </c>
+      <c r="C25" s="35" t="s">
+        <v>323</v>
+      </c>
+      <c r="D25" s="35" t="s">
+        <v>300</v>
+      </c>
+      <c r="E25" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="35" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="35" t="s">
+        <v>318</v>
+      </c>
+      <c r="C26" s="35" t="s">
+        <v>324</v>
+      </c>
+      <c r="D26" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="E26" s="35" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="35" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="35" t="s">
+        <v>318</v>
+      </c>
+      <c r="C27" s="35" t="s">
+        <v>325</v>
+      </c>
+      <c r="D27" s="35" t="s">
+        <v>300</v>
+      </c>
+      <c r="E27" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="35" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="35" t="s">
+        <v>326</v>
+      </c>
+      <c r="C28" s="35" t="s">
+        <v>327</v>
+      </c>
+      <c r="D28" s="35" t="s">
+        <v>328</v>
+      </c>
+      <c r="E28" s="35" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="35" t="s">
+        <v>326</v>
+      </c>
+      <c r="C29" s="35" t="s">
+        <v>330</v>
+      </c>
+      <c r="D29" s="35" t="s">
+        <v>300</v>
+      </c>
+      <c r="E29" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="35" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="35" t="s">
+        <v>326</v>
+      </c>
+      <c r="C30" s="35" t="s">
+        <v>331</v>
+      </c>
+      <c r="D30" s="35" t="s">
+        <v>300</v>
+      </c>
+      <c r="E30" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="35" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="35" t="s">
+        <v>326</v>
+      </c>
+      <c r="C31" s="35" t="s">
+        <v>332</v>
+      </c>
+      <c r="D31" s="35" t="s">
+        <v>300</v>
+      </c>
+      <c r="E31" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="35" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="35" t="s">
+        <v>326</v>
+      </c>
+      <c r="C32" s="35" t="s">
+        <v>333</v>
+      </c>
+      <c r="D32" s="35" t="s">
+        <v>300</v>
+      </c>
+      <c r="E32" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="35" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="35" t="s">
+        <v>326</v>
+      </c>
+      <c r="C33" s="35" t="s">
+        <v>334</v>
+      </c>
+      <c r="D33" s="35" t="s">
+        <v>300</v>
+      </c>
+      <c r="E33" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="35" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="35" t="s">
+        <v>335</v>
+      </c>
+      <c r="C34" s="35" t="s">
+        <v>336</v>
+      </c>
+      <c r="D34" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="E34" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="35" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="35" t="s">
+        <v>335</v>
+      </c>
+      <c r="C35" s="35" t="s">
+        <v>337</v>
+      </c>
+      <c r="D35" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="E35" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="35" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="35" t="s">
+        <v>335</v>
+      </c>
+      <c r="C36" s="35" t="s">
+        <v>338</v>
+      </c>
+      <c r="D36" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="E36" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="35" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="35" t="s">
+        <v>335</v>
+      </c>
+      <c r="C37" s="35" t="s">
+        <v>339</v>
+      </c>
+      <c r="D37" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="E37" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="35" t="s">
+        <v>340</v>
+      </c>
+      <c r="C38" s="35" t="s">
+        <v>341</v>
+      </c>
+      <c r="D38" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="E38" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="35" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="35" t="s">
+        <v>340</v>
+      </c>
+      <c r="C39" s="35" t="s">
+        <v>342</v>
+      </c>
+      <c r="D39" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="E39" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="35" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="35" t="s">
+        <v>340</v>
+      </c>
+      <c r="C40" s="35" t="s">
+        <v>343</v>
+      </c>
+      <c r="D40" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="E40" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="35" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="35" t="s">
+        <v>340</v>
+      </c>
+      <c r="C41" s="35" t="s">
+        <v>344</v>
+      </c>
+      <c r="D41" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="E41" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="35" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="35" t="s">
+        <v>340</v>
+      </c>
+      <c r="C42" s="35" t="s">
+        <v>345</v>
+      </c>
+      <c r="D42" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="E42" s="35" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C44" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="D44" s="2" t="n">
+        <f aca="false">COUNTA(C5:C42)</f>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C45" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="D45" s="36" t="n">
+        <f aca="false">MAX(COUNTIF(B5:B42,"ID1*"),COUNTIF(B5:B42,"ID2*"),COUNTIF(B5:B42,"ID3*"),COUNTIF(B5:B42,"ID4*"),COUNTIF(B5:B42,"ID5*"),COUNTIF(B5:B42,"ID6*"))</f>
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:B15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -4037,101 +5042,101 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="24" t="s">
-        <v>267</v>
+      <c r="B1" s="32" t="s">
+        <v>348</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>268</v>
+        <v>349</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>269</v>
+        <v>350</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>268</v>
+        <v>349</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>270</v>
+        <v>351</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>268</v>
+        <v>349</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>271</v>
+        <v>352</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>268</v>
+        <v>349</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>272</v>
+        <v>353</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>268</v>
+        <v>349</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>273</v>
+        <v>354</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>268</v>
+        <v>349</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>274</v>
+        <v>355</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>268</v>
+        <v>349</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>275</v>
+        <v>356</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>268</v>
+        <v>349</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>276</v>
+        <v>357</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>268</v>
+        <v>349</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>277</v>
+        <v>358</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>268</v>
+        <v>349</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>278</v>
+        <v>359</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>268</v>
+        <v>349</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>279</v>
+        <v>360</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="29" t="s">
-        <v>280</v>
+      <c r="B15" s="37" t="s">
+        <v>361</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Devis : suppression détecteurs d'ouverture, prises spécialisées à 195 €
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BjWSBdyxAjsRnCWBVUUVzr
</commit_message>
<xml_diff>
--- a/devis/Devis_electricite_T4_connecte_Legrand.xlsx
+++ b/devis/Devis_electricite_T4_connecte_Legrand.xlsx
@@ -247,19 +247,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E116" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Fourniture : prix d'achat × coefficient de marge (onglet Références fournisseur) + pose 35 €</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E137" authorId="0">
+    <comment ref="E136" authorId="0">
       <text>
         <r>
           <rPr>
@@ -298,7 +286,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="627" uniqueCount="400">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="395">
   <si>
     <t xml:space="preserve">MAUREL'EC</t>
   </si>
@@ -912,18 +900,12 @@
     <t xml:space="preserve">12.4</t>
   </si>
   <si>
-    <t xml:space="preserve">Détecteur d'ouverture connecté Netatmo DTG-PRO (porte d'entrée + 6 baies) – fourniture et pose</t>
+    <t xml:space="preserve">Point d'alimentation caméra sur le circuit alarme/caméras (dérivation + boîte)</t>
   </si>
   <si>
     <t xml:space="preserve">12.5</t>
   </si>
   <si>
-    <t xml:space="preserve">Point d'alimentation caméra sur le circuit alarme/caméras (dérivation + boîte)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12.6</t>
-  </si>
-  <si>
     <t xml:space="preserve">Caméra extérieure Netatmo NOC-PRO (balcons) – fourniture et pose</t>
   </si>
   <si>
@@ -1260,15 +1242,6 @@
     <t xml:space="preserve">Hall</t>
   </si>
   <si>
-    <t xml:space="preserve">Détecteur d'ouverture intelligent Netatmo (porte / fenêtre)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DTG-PRO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Porte d'entrée + 6 baies – prix à l'unité ou par lot ?</t>
-  </si>
-  <si>
     <t xml:space="preserve">Caméra extérieure intelligente Netatmo (NOC-S-PRO = avec sirène)</t>
   </si>
   <si>
@@ -1494,7 +1467,7 @@
     <t xml:space="preserve">Saignées : 160 ml murs + 70 ml sol estimés pour un immeuble béton – à recaler à la visite (ce poste pèse lourd dans le total).</t>
   </si>
   <si>
-    <t xml:space="preserve">PRIX : appareillage connecté et Netatmo = prix d'achat Rexel × 1,40 + pose 35 € par appareil ; création des circuits depuis le tableau = 190 € par circuit (38 circuits), dérivations vers les points comptées à part. Caméras NSC-PRO / NOC-PRO : pas de prix Rexel, prix estimés. Détecteurs d'ouverture DTG-PRO à 89,37 € : vérifier si c'est le prix unitaire ou d'un lot.</t>
+    <t xml:space="preserve">PRIX : appareillage connecté et Netatmo = prix d'achat Rexel × 1,40 + pose 35 € par appareil ; création des circuits depuis le tableau = 190 € par circuit (38 circuits), dérivations vers les points comptées à part. Caméras NSC-PRO / NOC-PRO : pas de prix Rexel, prix estimés.</t>
   </si>
   <si>
     <t xml:space="preserve">Légende : chiffres en BLEU = quantités / prix modifiables. Montants sans TVA (micro-entreprise, art. 293 B du CGI).</t>
@@ -2174,7 +2147,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F149"/>
+  <dimension ref="A1:F148"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -3557,11 +3530,11 @@
         <v>1</v>
       </c>
       <c r="E89" s="13" t="n">
-        <v>50</v>
+        <v>195</v>
       </c>
       <c r="F89" s="14" t="n">
         <f aca="false">D89*E89</f>
-        <v>50</v>
+        <v>195</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3578,11 +3551,11 @@
         <v>1</v>
       </c>
       <c r="E90" s="13" t="n">
-        <v>50</v>
+        <v>195</v>
       </c>
       <c r="F90" s="14" t="n">
         <f aca="false">D90*E90</f>
-        <v>50</v>
+        <v>195</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3620,11 +3593,11 @@
         <v>1</v>
       </c>
       <c r="E92" s="13" t="n">
-        <v>50</v>
+        <v>195</v>
       </c>
       <c r="F92" s="14" t="n">
         <f aca="false">D92*E92</f>
-        <v>50</v>
+        <v>195</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3641,11 +3614,11 @@
         <v>1</v>
       </c>
       <c r="E93" s="13" t="n">
-        <v>50</v>
+        <v>195</v>
       </c>
       <c r="F93" s="14" t="n">
         <f aca="false">D93*E93</f>
-        <v>50</v>
+        <v>195</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3662,11 +3635,11 @@
         <v>1</v>
       </c>
       <c r="E94" s="13" t="n">
-        <v>50</v>
+        <v>195</v>
       </c>
       <c r="F94" s="14" t="n">
         <f aca="false">D94*E94</f>
-        <v>50</v>
+        <v>195</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3704,11 +3677,11 @@
         <v>1</v>
       </c>
       <c r="E96" s="13" t="n">
-        <v>50</v>
+        <v>195</v>
       </c>
       <c r="F96" s="14" t="n">
         <f aca="false">D96*E96</f>
-        <v>50</v>
+        <v>195</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3781,7 +3754,7 @@
       </c>
       <c r="F100" s="16" t="n">
         <f aca="false">SUM(F88:F99)</f>
-        <v>654.87</v>
+        <v>1524.87</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4032,7 +4005,7 @@
         <v>146.17</v>
       </c>
     </row>
-    <row r="116" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="10" t="s">
         <v>203</v>
       </c>
@@ -4043,15 +4016,14 @@
         <v>37</v>
       </c>
       <c r="D116" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="E116" s="14" t="n">
-        <f aca="false">ROUND('Références fournisseur'!$I$32*1+35,2)</f>
-        <v>160.12</v>
+        <v>3</v>
+      </c>
+      <c r="E116" s="13" t="n">
+        <v>55</v>
       </c>
       <c r="F116" s="14" t="n">
         <f aca="false">D116*E116</f>
-        <v>1120.84</v>
+        <v>165</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4065,59 +4037,59 @@
         <v>37</v>
       </c>
       <c r="D117" s="12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E117" s="13" t="n">
-        <v>55</v>
+        <v>350</v>
       </c>
       <c r="F117" s="14" t="n">
         <f aca="false">D117*E117</f>
-        <v>165</v>
-      </c>
-    </row>
-    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A118" s="10" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E118" s="15" t="s">
         <v>207</v>
       </c>
-      <c r="B118" s="11" t="s">
+      <c r="F118" s="16" t="n">
+        <f aca="false">SUM(F113:F117)</f>
+        <v>1807.55</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="C118" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D118" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E118" s="13" t="n">
-        <v>350</v>
-      </c>
-      <c r="F118" s="14" t="n">
-        <f aca="false">D118*E118</f>
-        <v>700</v>
-      </c>
-    </row>
-    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E119" s="15" t="s">
+      <c r="B120" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="F119" s="16" t="n">
-        <f aca="false">SUM(F113:F118)</f>
-        <v>2928.39</v>
-      </c>
-    </row>
-    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A121" s="8" t="s">
+      <c r="C120" s="9"/>
+      <c r="D120" s="9"/>
+      <c r="E120" s="9"/>
+      <c r="F120" s="9"/>
+    </row>
+    <row r="121" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A121" s="10" t="s">
         <v>210</v>
       </c>
-      <c r="B121" s="9" t="s">
+      <c r="B121" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="C121" s="9"/>
-      <c r="D121" s="9"/>
-      <c r="E121" s="9"/>
-      <c r="F121" s="9"/>
-    </row>
-    <row r="122" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C121" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D121" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E121" s="13" t="n">
+        <v>480</v>
+      </c>
+      <c r="F121" s="14" t="n">
+        <f aca="false">D121*E121</f>
+        <v>480</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="10" t="s">
         <v>212</v>
       </c>
@@ -4131,14 +4103,14 @@
         <v>1</v>
       </c>
       <c r="E122" s="13" t="n">
-        <v>480</v>
+        <v>280</v>
       </c>
       <c r="F122" s="14" t="n">
         <f aca="false">D122*E122</f>
-        <v>480</v>
-      </c>
-    </row>
-    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="10" t="s">
         <v>214</v>
       </c>
@@ -4152,72 +4124,72 @@
         <v>1</v>
       </c>
       <c r="E123" s="13" t="n">
-        <v>280</v>
+        <v>360</v>
       </c>
       <c r="F123" s="14" t="n">
         <f aca="false">D123*E123</f>
-        <v>280</v>
-      </c>
-    </row>
-    <row r="124" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A124" s="10" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E124" s="15" t="s">
         <v>216</v>
       </c>
-      <c r="B124" s="11" t="s">
+      <c r="F124" s="16" t="n">
+        <f aca="false">SUM(F121:F123)</f>
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E126" s="17" t="s">
         <v>217</v>
       </c>
-      <c r="C124" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D124" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E124" s="13" t="n">
-        <v>360</v>
-      </c>
-      <c r="F124" s="14" t="n">
-        <f aca="false">D124*E124</f>
-        <v>360</v>
-      </c>
-    </row>
-    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E125" s="15" t="s">
+      <c r="F126" s="18" t="n">
+        <f aca="false">F13+F21+F41+F51+F62+F70+F77+F81+F85+F100+F110+F118+F124</f>
+        <v>40268.16</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E127" s="19" t="s">
         <v>218</v>
       </c>
-      <c r="F125" s="16" t="n">
-        <f aca="false">SUM(F122:F124)</f>
-        <v>1120</v>
-      </c>
-    </row>
-    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E127" s="17" t="s">
+    </row>
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E128" s="20" t="s">
         <v>219</v>
       </c>
-      <c r="F127" s="18" t="n">
-        <f aca="false">F13+F21+F41+F51+F62+F70+F77+F81+F85+F100+F110+F119+F125</f>
-        <v>40519</v>
-      </c>
-    </row>
-    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E128" s="19" t="s">
+      <c r="F128" s="21" t="n">
+        <f aca="false">F126*0.3</f>
+        <v>12080.448</v>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="22" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E129" s="20" t="s">
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A132" s="10" t="s">
         <v>221</v>
       </c>
-      <c r="F129" s="21" t="n">
-        <f aca="false">F127*0.3</f>
-        <v>12155.7</v>
-      </c>
-    </row>
-    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A132" s="22" t="s">
+      <c r="B132" s="11" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C132" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D132" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="E132" s="13" t="n">
+        <v>65</v>
+      </c>
+      <c r="F132" s="14" t="n">
+        <f aca="false">D132*E132</f>
+        <v>780</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="10" t="s">
         <v>223</v>
       </c>
@@ -4228,17 +4200,17 @@
         <v>37</v>
       </c>
       <c r="D133" s="12" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E133" s="13" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="F133" s="14" t="n">
         <f aca="false">D133*E133</f>
-        <v>780</v>
-      </c>
-    </row>
-    <row r="134" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="10" t="s">
         <v>225</v>
       </c>
@@ -4246,17 +4218,17 @@
         <v>226</v>
       </c>
       <c r="C134" s="10" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D134" s="12" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E134" s="13" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="F134" s="14" t="n">
         <f aca="false">D134*E134</f>
-        <v>600</v>
+        <v>390</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4267,20 +4239,20 @@
         <v>228</v>
       </c>
       <c r="C135" s="10" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D135" s="12" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E135" s="13" t="n">
-        <v>65</v>
+        <v>120</v>
       </c>
       <c r="F135" s="14" t="n">
         <f aca="false">D135*E135</f>
-        <v>390</v>
-      </c>
-    </row>
-    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="136" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="10" t="s">
         <v>229</v>
       </c>
@@ -4291,17 +4263,18 @@
         <v>37</v>
       </c>
       <c r="D136" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E136" s="13" t="n">
-        <v>120</v>
+        <v>21</v>
+      </c>
+      <c r="E136" s="14" t="n">
+        <f aca="false">ROUND('Références fournisseur'!$I$19*1+'Références fournisseur'!$I$20*-1+'Références fournisseur'!$I$21*-1+'Références fournisseur'!$I$22*-1+0,2)</f>
+        <v>62.4</v>
       </c>
       <c r="F136" s="14" t="n">
         <f aca="false">D136*E136</f>
-        <v>120</v>
-      </c>
-    </row>
-    <row r="137" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>1310.4</v>
+      </c>
+    </row>
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="10" t="s">
         <v>231</v>
       </c>
@@ -4312,80 +4285,58 @@
         <v>37</v>
       </c>
       <c r="D137" s="12" t="n">
-        <v>21</v>
-      </c>
-      <c r="E137" s="14" t="n">
-        <f aca="false">ROUND('Références fournisseur'!$I$19*1+'Références fournisseur'!$I$20*-1+'Références fournisseur'!$I$21*-1+'Références fournisseur'!$I$22*-1+0,2)</f>
-        <v>62.4</v>
+        <v>1</v>
+      </c>
+      <c r="E137" s="13" t="n">
+        <v>420</v>
       </c>
       <c r="F137" s="14" t="n">
         <f aca="false">D137*E137</f>
-        <v>1310.4</v>
-      </c>
-    </row>
-    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A138" s="10" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E138" s="15" t="s">
         <v>233</v>
       </c>
-      <c r="B138" s="11" t="s">
+      <c r="F138" s="16" t="n">
+        <f aca="false">SUM(F132:F137)</f>
+        <v>3620.4</v>
+      </c>
+    </row>
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A141" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="C138" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D138" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E138" s="13" t="n">
-        <v>420</v>
-      </c>
-      <c r="F138" s="14" t="n">
-        <f aca="false">D138*E138</f>
-        <v>420</v>
-      </c>
-    </row>
-    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E139" s="15" t="s">
+    </row>
+    <row r="142" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B142" s="23" t="s">
         <v>235</v>
       </c>
-      <c r="F139" s="16" t="n">
-        <f aca="false">SUM(F133:F138)</f>
-        <v>3620.4</v>
-      </c>
-    </row>
-    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A142" s="2" t="s">
+    </row>
+    <row r="143" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B143" s="23" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="143" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B143" s="23" t="s">
+    <row r="144" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B144" s="23" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="144" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B144" s="23" t="s">
+    <row r="145" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B145" s="23" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="145" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B145" s="23" t="s">
+    <row r="146" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B146" s="23" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="146" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B146" s="23" t="s">
+    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B148" s="2" t="s">
         <v>240</v>
-      </c>
-    </row>
-    <row r="147" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B147" s="23" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B149" s="2" t="s">
-        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -4405,7 +4356,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -4420,12 +4371,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="24" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="25" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B2" s="25"/>
       <c r="C2" s="25"/>
@@ -4438,7 +4389,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E3" s="26" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="F3" s="27" t="n">
         <v>1.4</v>
@@ -4446,62 +4397,62 @@
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="28" t="s">
+        <v>244</v>
+      </c>
+      <c r="B4" s="28" t="s">
+        <v>245</v>
+      </c>
+      <c r="C4" s="28" t="s">
         <v>246</v>
-      </c>
-      <c r="B4" s="28" t="s">
-        <v>247</v>
-      </c>
-      <c r="C4" s="28" t="s">
-        <v>248</v>
       </c>
       <c r="D4" s="28" t="s">
         <v>17</v>
       </c>
       <c r="E4" s="28" t="s">
+        <v>247</v>
+      </c>
+      <c r="F4" s="28" t="s">
+        <v>248</v>
+      </c>
+      <c r="G4" s="28" t="s">
         <v>249</v>
       </c>
-      <c r="F4" s="28" t="s">
+      <c r="H4" s="28" t="s">
         <v>250</v>
-      </c>
-      <c r="G4" s="28" t="s">
-        <v>251</v>
-      </c>
-      <c r="H4" s="28" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="28" t="s">
+        <v>244</v>
+      </c>
+      <c r="B5" s="28" t="s">
+        <v>245</v>
+      </c>
+      <c r="C5" s="28" t="s">
         <v>246</v>
-      </c>
-      <c r="B5" s="28" t="s">
-        <v>247</v>
-      </c>
-      <c r="C5" s="28" t="s">
-        <v>248</v>
       </c>
       <c r="D5" s="28" t="s">
         <v>17</v>
       </c>
       <c r="E5" s="28" t="s">
+        <v>247</v>
+      </c>
+      <c r="F5" s="28" t="s">
+        <v>248</v>
+      </c>
+      <c r="G5" s="28" t="s">
         <v>249</v>
       </c>
-      <c r="F5" s="28" t="s">
+      <c r="H5" s="28" t="s">
         <v>250</v>
       </c>
-      <c r="G5" s="28" t="s">
+      <c r="I5" s="28" t="s">
         <v>251</v>
-      </c>
-      <c r="H5" s="28" t="s">
-        <v>252</v>
-      </c>
-      <c r="I5" s="28" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -4514,13 +4465,13 @@
     </row>
     <row r="7" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="B7" s="29" t="s">
+        <v>254</v>
+      </c>
+      <c r="C7" s="11" t="s">
         <v>255</v>
-      </c>
-      <c r="B7" s="29" t="s">
-        <v>256</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>257</v>
       </c>
       <c r="D7" s="12" t="n">
         <v>1</v>
@@ -4536,7 +4487,7 @@
         <v>196.54</v>
       </c>
       <c r="H7" s="32" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="I7" s="30" t="n">
         <f aca="false">F7*$F$3</f>
@@ -4545,13 +4496,13 @@
     </row>
     <row r="8" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
+        <v>257</v>
+      </c>
+      <c r="B8" s="29" t="s">
+        <v>258</v>
+      </c>
+      <c r="C8" s="11" t="s">
         <v>259</v>
-      </c>
-      <c r="B8" s="29" t="s">
-        <v>260</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>261</v>
       </c>
       <c r="D8" s="12" t="n">
         <v>1</v>
@@ -4565,7 +4516,7 @@
         <v>92.25</v>
       </c>
       <c r="H8" s="33" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="I8" s="30" t="n">
         <f aca="false">F8*$F$3</f>
@@ -4574,13 +4525,13 @@
     </row>
     <row r="9" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
+        <v>261</v>
+      </c>
+      <c r="B9" s="29" t="s">
+        <v>262</v>
+      </c>
+      <c r="C9" s="11" t="s">
         <v>263</v>
-      </c>
-      <c r="B9" s="29" t="s">
-        <v>264</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>265</v>
       </c>
       <c r="D9" s="12" t="n">
         <v>0</v>
@@ -4594,7 +4545,7 @@
         <v>0</v>
       </c>
       <c r="H9" s="32" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="I9" s="30" t="n">
         <f aca="false">F9*$F$3</f>
@@ -4603,7 +4554,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
@@ -4616,13 +4567,13 @@
     </row>
     <row r="11" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="B11" s="29" t="s">
+        <v>266</v>
+      </c>
+      <c r="C11" s="11" t="s">
         <v>267</v>
-      </c>
-      <c r="B11" s="29" t="s">
-        <v>268</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>269</v>
       </c>
       <c r="D11" s="12" t="n">
         <v>22</v>
@@ -4636,7 +4587,7 @@
         <v>1226.94</v>
       </c>
       <c r="H11" s="32" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="I11" s="30" t="n">
         <f aca="false">F11*$F$3</f>
@@ -4645,13 +4596,13 @@
     </row>
     <row r="12" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
+        <v>268</v>
+      </c>
+      <c r="B12" s="29" t="s">
+        <v>269</v>
+      </c>
+      <c r="C12" s="11" t="s">
         <v>270</v>
-      </c>
-      <c r="B12" s="29" t="s">
-        <v>271</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>272</v>
       </c>
       <c r="D12" s="12" t="n">
         <v>5</v>
@@ -4665,7 +4616,7 @@
         <v>305.7</v>
       </c>
       <c r="H12" s="33" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="I12" s="30" t="n">
         <f aca="false">F12*$F$3</f>
@@ -4674,13 +4625,13 @@
     </row>
     <row r="13" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
+        <v>271</v>
+      </c>
+      <c r="B13" s="29" t="s">
+        <v>272</v>
+      </c>
+      <c r="C13" s="11" t="s">
         <v>273</v>
-      </c>
-      <c r="B13" s="29" t="s">
-        <v>274</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>275</v>
       </c>
       <c r="D13" s="12" t="n">
         <v>1</v>
@@ -4694,7 +4645,7 @@
         <v>27.67</v>
       </c>
       <c r="H13" s="33" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="I13" s="30" t="n">
         <f aca="false">F13*$F$3</f>
@@ -4703,13 +4654,13 @@
     </row>
     <row r="14" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
+        <v>274</v>
+      </c>
+      <c r="B14" s="29" t="s">
+        <v>275</v>
+      </c>
+      <c r="C14" s="11" t="s">
         <v>276</v>
-      </c>
-      <c r="B14" s="29" t="s">
-        <v>277</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>278</v>
       </c>
       <c r="D14" s="12" t="n">
         <v>1</v>
@@ -4725,7 +4676,7 @@
         <v>34</v>
       </c>
       <c r="H14" s="32" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="I14" s="30" t="n">
         <f aca="false">F14*$F$3</f>
@@ -4734,7 +4685,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
@@ -4747,13 +4698,13 @@
     </row>
     <row r="16" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
+        <v>278</v>
+      </c>
+      <c r="B16" s="29" t="s">
+        <v>279</v>
+      </c>
+      <c r="C16" s="11" t="s">
         <v>280</v>
-      </c>
-      <c r="B16" s="29" t="s">
-        <v>281</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>282</v>
       </c>
       <c r="D16" s="12" t="n">
         <v>8</v>
@@ -4767,7 +4718,7 @@
         <v>468.8</v>
       </c>
       <c r="H16" s="32" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="I16" s="30" t="n">
         <f aca="false">F16*$F$3</f>
@@ -4776,13 +4727,13 @@
     </row>
     <row r="17" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
+        <v>281</v>
+      </c>
+      <c r="B17" s="29" t="s">
+        <v>282</v>
+      </c>
+      <c r="C17" s="11" t="s">
         <v>283</v>
-      </c>
-      <c r="B17" s="29" t="s">
-        <v>284</v>
-      </c>
-      <c r="C17" s="11" t="s">
-        <v>285</v>
       </c>
       <c r="D17" s="12" t="n">
         <v>1</v>
@@ -4796,7 +4747,7 @@
         <v>58.63</v>
       </c>
       <c r="H17" s="32" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="I17" s="30" t="n">
         <f aca="false">F17*$F$3</f>
@@ -4805,7 +4756,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -4818,13 +4769,13 @@
     </row>
     <row r="19" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="B19" s="29" t="s">
+        <v>286</v>
+      </c>
+      <c r="C19" s="11" t="s">
         <v>287</v>
-      </c>
-      <c r="B19" s="29" t="s">
-        <v>288</v>
-      </c>
-      <c r="C19" s="11" t="s">
-        <v>289</v>
       </c>
       <c r="D19" s="12" t="n">
         <v>5</v>
@@ -4840,7 +4791,7 @@
         <v>249.6</v>
       </c>
       <c r="H19" s="32" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="I19" s="30" t="n">
         <f aca="false">F19*$F$3</f>
@@ -4849,13 +4800,13 @@
     </row>
     <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="B20" s="29" t="s">
+        <v>289</v>
+      </c>
+      <c r="C20" s="11" t="s">
         <v>290</v>
-      </c>
-      <c r="B20" s="29" t="s">
-        <v>291</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>292</v>
       </c>
       <c r="D20" s="12" t="n">
         <v>21</v>
@@ -4869,7 +4820,7 @@
         <v>63</v>
       </c>
       <c r="H20" s="33" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="I20" s="30" t="n">
         <f aca="false">F20*$F$3</f>
@@ -4878,13 +4829,13 @@
     </row>
     <row r="21" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="B21" s="29" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D21" s="12" t="n">
         <v>21</v>
@@ -4898,7 +4849,7 @@
         <v>17.64</v>
       </c>
       <c r="H21" s="32" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="I21" s="30" t="n">
         <f aca="false">F21*$F$3</f>
@@ -4907,13 +4858,13 @@
     </row>
     <row r="22" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
+        <v>293</v>
+      </c>
+      <c r="B22" s="29" t="s">
+        <v>294</v>
+      </c>
+      <c r="C22" s="11" t="s">
         <v>295</v>
-      </c>
-      <c r="B22" s="29" t="s">
-        <v>296</v>
-      </c>
-      <c r="C22" s="11" t="s">
-        <v>297</v>
       </c>
       <c r="D22" s="12" t="n">
         <v>26</v>
@@ -4927,7 +4878,7 @@
         <v>39.26</v>
       </c>
       <c r="H22" s="33" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="I22" s="30" t="n">
         <f aca="false">F22*$F$3</f>
@@ -4936,13 +4887,13 @@
     </row>
     <row r="23" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B23" s="29" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="D23" s="12" t="n">
         <v>5</v>
@@ -4958,7 +4909,7 @@
         <v>77.35</v>
       </c>
       <c r="H23" s="32" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="I23" s="30" t="n">
         <f aca="false">F23*$F$3</f>
@@ -4967,13 +4918,13 @@
     </row>
     <row r="24" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B24" s="29" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="D24" s="12" t="n">
         <v>5</v>
@@ -4989,7 +4940,7 @@
         <v>11.7</v>
       </c>
       <c r="H24" s="32" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="I24" s="30" t="n">
         <f aca="false">F24*$F$3</f>
@@ -4998,13 +4949,13 @@
     </row>
     <row r="25" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="B25" s="29" t="s">
+        <v>301</v>
+      </c>
+      <c r="C25" s="11" t="s">
         <v>302</v>
-      </c>
-      <c r="B25" s="29" t="s">
-        <v>303</v>
-      </c>
-      <c r="C25" s="11" t="s">
-        <v>304</v>
       </c>
       <c r="D25" s="12" t="n">
         <v>2</v>
@@ -5018,7 +4969,7 @@
         <v>12.64</v>
       </c>
       <c r="H25" s="33" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="I25" s="30" t="n">
         <f aca="false">F25*$F$3</f>
@@ -5027,13 +4978,13 @@
     </row>
     <row r="26" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="B26" s="29" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="D26" s="12" t="n">
         <v>2</v>
@@ -5047,7 +4998,7 @@
         <v>4</v>
       </c>
       <c r="H26" s="33" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="I26" s="30" t="n">
         <f aca="false">F26*$F$3</f>
@@ -5056,13 +5007,13 @@
     </row>
     <row r="27" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
+        <v>305</v>
+      </c>
+      <c r="B27" s="29" t="s">
+        <v>306</v>
+      </c>
+      <c r="C27" s="11" t="s">
         <v>307</v>
-      </c>
-      <c r="B27" s="29" t="s">
-        <v>308</v>
-      </c>
-      <c r="C27" s="11" t="s">
-        <v>309</v>
       </c>
       <c r="D27" s="12" t="n">
         <v>67</v>
@@ -5076,7 +5027,7 @@
         <v>85.76</v>
       </c>
       <c r="H27" s="33" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="I27" s="30" t="n">
         <f aca="false">F27*$F$3</f>
@@ -5085,7 +5036,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B28" s="9"/>
       <c r="C28" s="9"/>
@@ -5098,13 +5049,13 @@
     </row>
     <row r="29" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
+        <v>309</v>
+      </c>
+      <c r="B29" s="29" t="s">
+        <v>310</v>
+      </c>
+      <c r="C29" s="11" t="s">
         <v>311</v>
-      </c>
-      <c r="B29" s="29" t="s">
-        <v>312</v>
-      </c>
-      <c r="C29" s="11" t="s">
-        <v>313</v>
       </c>
       <c r="D29" s="12" t="n">
         <v>3</v>
@@ -5120,7 +5071,7 @@
         <v>300.99</v>
       </c>
       <c r="H29" s="32" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="I29" s="30" t="n">
         <f aca="false">F29*$F$3</f>
@@ -5129,13 +5080,13 @@
     </row>
     <row r="30" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="B30" s="29" t="s">
+        <v>313</v>
+      </c>
+      <c r="C30" s="11" t="s">
         <v>314</v>
-      </c>
-      <c r="B30" s="29" t="s">
-        <v>315</v>
-      </c>
-      <c r="C30" s="11" t="s">
-        <v>316</v>
       </c>
       <c r="D30" s="12" t="n">
         <v>1</v>
@@ -5147,7 +5098,7 @@
         <v>0</v>
       </c>
       <c r="H30" s="33" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="I30" s="30" t="n">
         <f aca="false">F30*$F$3</f>
@@ -5156,13 +5107,13 @@
     </row>
     <row r="31" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
+        <v>315</v>
+      </c>
+      <c r="B31" s="29" t="s">
+        <v>316</v>
+      </c>
+      <c r="C31" s="11" t="s">
         <v>317</v>
-      </c>
-      <c r="B31" s="29" t="s">
-        <v>318</v>
-      </c>
-      <c r="C31" s="11" t="s">
-        <v>319</v>
       </c>
       <c r="D31" s="12" t="n">
         <v>1</v>
@@ -5176,7 +5127,7 @@
         <v>79.41</v>
       </c>
       <c r="H31" s="33" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="I31" s="30" t="n">
         <f aca="false">F31*$F$3</f>
@@ -5185,85 +5136,56 @@
     </row>
     <row r="32" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="s">
+        <v>318</v>
+      </c>
+      <c r="B32" s="29" t="s">
+        <v>319</v>
+      </c>
+      <c r="C32" s="11" t="s">
         <v>320</v>
       </c>
-      <c r="B32" s="29" t="s">
-        <v>321</v>
-      </c>
-      <c r="C32" s="11" t="s">
-        <v>322</v>
-      </c>
       <c r="D32" s="12" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E32" s="30"/>
-      <c r="F32" s="31" t="n">
-        <v>89.37</v>
-      </c>
+      <c r="F32" s="31"/>
       <c r="G32" s="30" t="n">
         <f aca="false">D32*F32</f>
-        <v>625.59</v>
+        <v>0</v>
       </c>
       <c r="H32" s="33" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="I32" s="30" t="n">
         <f aca="false">F32*$F$3</f>
-        <v>125.118</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="11" t="s">
-        <v>323</v>
-      </c>
-      <c r="B33" s="29" t="s">
-        <v>324</v>
-      </c>
-      <c r="C33" s="11" t="s">
-        <v>325</v>
-      </c>
-      <c r="D33" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E33" s="30"/>
-      <c r="F33" s="31"/>
-      <c r="G33" s="30" t="n">
-        <f aca="false">D33*F33</f>
         <v>0</v>
       </c>
-      <c r="H33" s="33" t="s">
-        <v>262</v>
-      </c>
-      <c r="I33" s="30" t="n">
-        <f aca="false">F33*$F$3</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F35" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="G35" s="16" t="n">
-        <f aca="false">SUM(G6:G33)</f>
-        <v>3977.47</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="25" t="s">
-        <v>326</v>
-      </c>
-      <c r="B37" s="25"/>
-      <c r="C37" s="25"/>
-      <c r="D37" s="25"/>
-      <c r="E37" s="25"/>
-      <c r="F37" s="25"/>
-      <c r="G37" s="25"/>
-      <c r="H37" s="25"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F34" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="G34" s="16" t="n">
+        <f aca="false">SUM(G6:G32)</f>
+        <v>3351.88</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="25" t="s">
+        <v>321</v>
+      </c>
+      <c r="B36" s="25"/>
+      <c r="C36" s="25"/>
+      <c r="D36" s="25"/>
+      <c r="E36" s="25"/>
+      <c r="F36" s="25"/>
+      <c r="G36" s="25"/>
+      <c r="H36" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A36:H36"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -5292,12 +5214,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="34" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="35" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5305,16 +5227,16 @@
         <v>14</v>
       </c>
       <c r="B4" s="36" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="C4" s="36" t="s">
         <v>84</v>
       </c>
       <c r="D4" s="36" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="E4" s="36" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5322,16 +5244,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="37" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="C5" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="D5" s="37" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="E5" s="37" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5339,16 +5261,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="C6" s="37" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="D6" s="37" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="E6" s="37" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5356,16 +5278,16 @@
         <v>3</v>
       </c>
       <c r="B7" s="37" t="s">
+        <v>327</v>
+      </c>
+      <c r="C7" s="37" t="s">
         <v>332</v>
       </c>
-      <c r="C7" s="37" t="s">
-        <v>337</v>
-      </c>
       <c r="D7" s="37" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="E7" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5373,16 +5295,16 @@
         <v>4</v>
       </c>
       <c r="B8" s="37" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="C8" s="37" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="D8" s="37" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="E8" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5390,16 +5312,16 @@
         <v>5</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="C9" s="37" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="D9" s="37" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5407,16 +5329,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="C10" s="37" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="D10" s="37" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5424,16 +5346,16 @@
         <v>7</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="C11" s="37" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="D11" s="37" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="E11" s="37" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5441,16 +5363,16 @@
         <v>8</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="C12" s="37" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="D12" s="37" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5458,16 +5380,16 @@
         <v>9</v>
       </c>
       <c r="B13" s="37" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="C13" s="37" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="D13" s="37" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="E13" s="37" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5475,16 +5397,16 @@
         <v>10</v>
       </c>
       <c r="B14" s="37" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="C14" s="37" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="D14" s="37" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="E14" s="37" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5492,16 +5414,16 @@
         <v>11</v>
       </c>
       <c r="B15" s="37" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="C15" s="37" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="D15" s="37" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="E15" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5509,16 +5431,16 @@
         <v>12</v>
       </c>
       <c r="B16" s="37" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="C16" s="37" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="D16" s="37" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="E16" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5526,16 +5448,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="37" t="s">
+        <v>342</v>
+      </c>
+      <c r="C17" s="37" t="s">
         <v>347</v>
       </c>
-      <c r="C17" s="37" t="s">
-        <v>352</v>
-      </c>
       <c r="D17" s="37" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="E17" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5543,16 +5465,16 @@
         <v>14</v>
       </c>
       <c r="B18" s="37" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="C18" s="37" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="D18" s="37" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="E18" s="37" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5560,16 +5482,16 @@
         <v>15</v>
       </c>
       <c r="B19" s="37" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="C19" s="37" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="D19" s="37" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="E19" s="37" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5577,16 +5499,16 @@
         <v>16</v>
       </c>
       <c r="B20" s="37" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="C20" s="37" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="D20" s="37" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="E20" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5594,16 +5516,16 @@
         <v>17</v>
       </c>
       <c r="B21" s="37" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="C21" s="37" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="D21" s="37" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="E21" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5611,16 +5533,16 @@
         <v>18</v>
       </c>
       <c r="B22" s="37" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="C22" s="37" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="D22" s="37" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="E22" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5628,16 +5550,16 @@
         <v>19</v>
       </c>
       <c r="B23" s="37" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="C23" s="37" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="D23" s="37" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="E23" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5645,16 +5567,16 @@
         <v>20</v>
       </c>
       <c r="B24" s="37" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="C24" s="37" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="D24" s="37" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="E24" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5662,16 +5584,16 @@
         <v>21</v>
       </c>
       <c r="B25" s="37" t="s">
+        <v>351</v>
+      </c>
+      <c r="C25" s="37" t="s">
         <v>356</v>
       </c>
-      <c r="C25" s="37" t="s">
-        <v>361</v>
-      </c>
       <c r="D25" s="37" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="E25" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5679,16 +5601,16 @@
         <v>22</v>
       </c>
       <c r="B26" s="37" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="C26" s="37" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="D26" s="37" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="E26" s="37" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5696,16 +5618,16 @@
         <v>23</v>
       </c>
       <c r="B27" s="37" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="C27" s="37" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="D27" s="37" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="E27" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5713,16 +5635,16 @@
         <v>24</v>
       </c>
       <c r="B28" s="37" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="C28" s="37" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="D28" s="37" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="E28" s="37" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5730,16 +5652,16 @@
         <v>25</v>
       </c>
       <c r="B29" s="37" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="C29" s="37" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="D29" s="37" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="E29" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5747,16 +5669,16 @@
         <v>26</v>
       </c>
       <c r="B30" s="37" t="s">
+        <v>359</v>
+      </c>
+      <c r="C30" s="37" t="s">
         <v>364</v>
       </c>
-      <c r="C30" s="37" t="s">
-        <v>369</v>
-      </c>
       <c r="D30" s="37" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="E30" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5764,16 +5686,16 @@
         <v>27</v>
       </c>
       <c r="B31" s="37" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="C31" s="37" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="D31" s="37" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="E31" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5781,16 +5703,16 @@
         <v>28</v>
       </c>
       <c r="B32" s="37" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="C32" s="37" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="D32" s="37" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="E32" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5798,16 +5720,16 @@
         <v>29</v>
       </c>
       <c r="B33" s="37" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="C33" s="37" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="D33" s="37" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="E33" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5815,16 +5737,16 @@
         <v>30</v>
       </c>
       <c r="B34" s="37" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="C34" s="37" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="D34" s="37" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="E34" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5832,16 +5754,16 @@
         <v>31</v>
       </c>
       <c r="B35" s="37" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="C35" s="37" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="D35" s="37" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="E35" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5849,16 +5771,16 @@
         <v>32</v>
       </c>
       <c r="B36" s="37" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="C36" s="37" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="D36" s="37" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="E36" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5866,16 +5788,16 @@
         <v>33</v>
       </c>
       <c r="B37" s="37" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="C37" s="37" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="D37" s="37" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="E37" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5883,16 +5805,16 @@
         <v>34</v>
       </c>
       <c r="B38" s="37" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="C38" s="37" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="D38" s="37" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="E38" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5900,16 +5822,16 @@
         <v>35</v>
       </c>
       <c r="B39" s="37" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="C39" s="37" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="D39" s="37" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="E39" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5917,16 +5839,16 @@
         <v>36</v>
       </c>
       <c r="B40" s="37" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="C40" s="37" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="D40" s="37" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="E40" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5934,16 +5856,16 @@
         <v>37</v>
       </c>
       <c r="B41" s="37" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="C41" s="37" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="D41" s="37" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="E41" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5951,21 +5873,21 @@
         <v>38</v>
       </c>
       <c r="B42" s="37" t="s">
+        <v>373</v>
+      </c>
+      <c r="C42" s="37" t="s">
         <v>378</v>
       </c>
-      <c r="C42" s="37" t="s">
-        <v>383</v>
-      </c>
       <c r="D42" s="37" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="E42" s="37" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C44" s="2" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="D44" s="2" t="n">
         <f aca="false">COUNTA(C5:C42)</f>
@@ -5974,7 +5896,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C45" s="5" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="D45" s="38" t="n">
         <f aca="false">MAX(COUNTIF(B5:B42,"ID1*"),COUNTIF(B5:B42,"ID2*"),COUNTIF(B5:B42,"ID3*"),COUNTIF(B5:B42,"ID4*"),COUNTIF(B5:B42,"ID5*"),COUNTIF(B5:B42,"ID6*"))</f>
@@ -6006,100 +5928,100 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="34" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
+        <v>382</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>387</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>392</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>398</v>
+        <v>393</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="39" t="s">
-        <v>399</v>
+        <v>394</v>
       </c>
     </row>
   </sheetData>

</xml_diff>